<commit_message>
Try run 03 again
</commit_message>
<xml_diff>
--- a/assets/3D/sust yield server/setup.xlsx
+++ b/assets/3D/sust yield server/setup.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmarinriver\Projects\ConfinedLab\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmarinriver\Projects\ConfinedLab\assets\3D\sust yield server\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{566D8907-7F27-48FB-83A0-CB2391BF6ED7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E185B573-6830-4F13-B1E0-778BA6A8D7C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14168" yWindow="2107" windowWidth="21599" windowHeight="11423" firstSheet="9" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="grid" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2459" uniqueCount="1191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2466" uniqueCount="1192">
   <si>
     <t>nlay</t>
   </si>
@@ -3570,9 +3570,6 @@
     <t>Run01</t>
   </si>
   <si>
-    <t>Run02</t>
-  </si>
-  <si>
     <t>kv_1E-12_kh_1E-07</t>
   </si>
   <si>
@@ -3619,6 +3616,12 @@
   </si>
   <si>
     <t>Run03</t>
+  </si>
+  <si>
+    <t>Run02.1</t>
+  </si>
+  <si>
+    <t>Run02.2</t>
   </si>
 </sst>
 </file>
@@ -3675,18 +3678,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="3">
@@ -3732,7 +3729,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -3759,9 +3756,6 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="11" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="11" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="11" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
@@ -4408,15 +4402,8 @@
       <c r="H1" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="I1" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>106</v>
-      </c>
+      <c r="I1" s="4"/>
+      <c r="K1" s="4"/>
       <c r="L1" s="4"/>
       <c r="M1" s="4"/>
     </row>
@@ -4445,15 +4432,8 @@
       <c r="H2" s="4">
         <v>0</v>
       </c>
-      <c r="I2" s="4">
-        <v>0</v>
-      </c>
-      <c r="J2" s="4">
-        <v>0</v>
-      </c>
-      <c r="K2" s="4">
-        <v>0</v>
-      </c>
+      <c r="I2" s="4"/>
+      <c r="K2" s="4"/>
       <c r="L2" s="4"/>
       <c r="M2" s="4"/>
     </row>
@@ -4468,29 +4448,22 @@
         <v>0</v>
       </c>
       <c r="D3" s="4">
-        <v>-100</v>
+        <v>-1000</v>
       </c>
       <c r="E3" s="4">
-        <v>-200</v>
+        <v>-10000</v>
       </c>
       <c r="F3" s="4">
-        <v>-1000</v>
+        <v>-100000</v>
       </c>
       <c r="G3" s="4">
-        <v>-2000</v>
+        <v>-200000</v>
       </c>
       <c r="H3" s="4">
-        <v>-20000</v>
-      </c>
-      <c r="I3" s="4">
-        <v>-100000</v>
-      </c>
-      <c r="J3" s="4">
-        <v>-200000</v>
-      </c>
-      <c r="K3" s="4">
         <v>-600000</v>
       </c>
+      <c r="I3" s="4"/>
+      <c r="K3" s="4"/>
       <c r="L3" s="4"/>
       <c r="M3" s="4"/>
     </row>
@@ -4505,29 +4478,22 @@
         <v>0</v>
       </c>
       <c r="D4" s="4">
-        <v>-100</v>
+        <v>-1000</v>
       </c>
       <c r="E4" s="4">
-        <v>-200</v>
+        <v>-10000</v>
       </c>
       <c r="F4" s="4">
-        <v>-1000</v>
+        <v>-100000</v>
       </c>
       <c r="G4" s="4">
-        <v>-2000</v>
+        <v>-200000</v>
       </c>
       <c r="H4" s="4">
-        <v>-20000</v>
-      </c>
-      <c r="I4" s="4">
-        <v>-100000</v>
-      </c>
-      <c r="J4" s="4">
-        <v>-200000</v>
-      </c>
-      <c r="K4" s="4">
         <v>-600000</v>
       </c>
+      <c r="I4" s="4"/>
+      <c r="K4" s="4"/>
       <c r="L4" s="4"/>
       <c r="M4" s="4"/>
     </row>
@@ -4556,15 +4522,8 @@
       <c r="H5" s="4">
         <v>0</v>
       </c>
-      <c r="I5" s="4">
-        <v>0</v>
-      </c>
-      <c r="J5" s="4">
-        <v>0</v>
-      </c>
-      <c r="K5" s="4">
-        <v>0</v>
-      </c>
+      <c r="I5" s="4"/>
+      <c r="K5" s="4"/>
       <c r="L5" s="4"/>
       <c r="M5" s="4"/>
     </row>
@@ -4579,29 +4538,22 @@
         <v>0</v>
       </c>
       <c r="D6" s="4">
-        <v>-100</v>
+        <v>-1000</v>
       </c>
       <c r="E6" s="4">
-        <v>-200</v>
+        <v>-10000</v>
       </c>
       <c r="F6" s="4">
-        <v>-1000</v>
+        <v>-100000</v>
       </c>
       <c r="G6" s="4">
-        <v>-2000</v>
+        <v>-200000</v>
       </c>
       <c r="H6" s="4">
-        <v>-20000</v>
-      </c>
-      <c r="I6" s="4">
-        <v>-100000</v>
-      </c>
-      <c r="J6" s="4">
-        <v>-200000</v>
-      </c>
-      <c r="K6" s="4">
         <v>-600000</v>
       </c>
+      <c r="I6" s="4"/>
+      <c r="K6" s="4"/>
       <c r="L6" s="4"/>
       <c r="M6" s="4"/>
     </row>
@@ -4616,29 +4568,22 @@
         <v>0</v>
       </c>
       <c r="D7" s="4">
-        <v>-100</v>
+        <v>-1000</v>
       </c>
       <c r="E7" s="4">
-        <v>-200</v>
+        <v>-10000</v>
       </c>
       <c r="F7" s="4">
-        <v>-1000</v>
+        <v>-100000</v>
       </c>
       <c r="G7" s="4">
-        <v>-2000</v>
+        <v>-200000</v>
       </c>
       <c r="H7" s="4">
-        <v>-20000</v>
-      </c>
-      <c r="I7" s="4">
-        <v>-100000</v>
-      </c>
-      <c r="J7" s="4">
-        <v>-200000</v>
-      </c>
-      <c r="K7" s="4">
         <v>-600000</v>
       </c>
+      <c r="I7" s="4"/>
+      <c r="K7" s="4"/>
       <c r="L7" s="4"/>
       <c r="M7" s="4"/>
     </row>
@@ -4667,15 +4612,8 @@
       <c r="H8" s="4">
         <v>0</v>
       </c>
-      <c r="I8" s="4">
-        <v>0</v>
-      </c>
-      <c r="J8" s="4">
-        <v>0</v>
-      </c>
-      <c r="K8" s="4">
-        <v>0</v>
-      </c>
+      <c r="I8" s="4"/>
+      <c r="K8" s="4"/>
       <c r="L8" s="4"/>
       <c r="M8" s="4"/>
     </row>
@@ -4690,29 +4628,22 @@
         <v>0</v>
       </c>
       <c r="D9" s="4">
-        <v>-100</v>
+        <v>-1000</v>
       </c>
       <c r="E9" s="4">
-        <v>-200</v>
+        <v>-10000</v>
       </c>
       <c r="F9" s="4">
-        <v>-1000</v>
+        <v>-100000</v>
       </c>
       <c r="G9" s="4">
-        <v>-2000</v>
+        <v>-200000</v>
       </c>
       <c r="H9" s="4">
-        <v>-20000</v>
-      </c>
-      <c r="I9" s="4">
-        <v>-100000</v>
-      </c>
-      <c r="J9" s="4">
-        <v>-200000</v>
-      </c>
-      <c r="K9" s="4">
         <v>-600000</v>
       </c>
+      <c r="I9" s="4"/>
+      <c r="K9" s="4"/>
       <c r="L9" s="4"/>
       <c r="M9" s="4"/>
     </row>
@@ -4727,29 +4658,22 @@
         <v>0</v>
       </c>
       <c r="D10" s="4">
-        <v>-100</v>
+        <v>-1000</v>
       </c>
       <c r="E10" s="4">
-        <v>-200</v>
+        <v>-10000</v>
       </c>
       <c r="F10" s="4">
-        <v>-1000</v>
+        <v>-100000</v>
       </c>
       <c r="G10" s="4">
-        <v>-2000</v>
+        <v>-200000</v>
       </c>
       <c r="H10" s="4">
-        <v>-20000</v>
-      </c>
-      <c r="I10" s="4">
-        <v>-100000</v>
-      </c>
-      <c r="J10" s="4">
-        <v>-200000</v>
-      </c>
-      <c r="K10" s="4">
         <v>-600000</v>
       </c>
+      <c r="I10" s="4"/>
+      <c r="K10" s="4"/>
       <c r="L10" s="4"/>
       <c r="M10" s="4"/>
     </row>
@@ -4778,15 +4702,8 @@
       <c r="H11" s="4">
         <v>0</v>
       </c>
-      <c r="I11" s="4">
-        <v>0</v>
-      </c>
-      <c r="J11" s="4">
-        <v>0</v>
-      </c>
-      <c r="K11" s="4">
-        <v>0</v>
-      </c>
+      <c r="I11" s="4"/>
+      <c r="K11" s="4"/>
       <c r="L11" s="4"/>
       <c r="M11" s="4"/>
     </row>
@@ -4801,29 +4718,22 @@
         <v>0</v>
       </c>
       <c r="D12" s="4">
-        <v>-100</v>
+        <v>-1000</v>
       </c>
       <c r="E12" s="4">
-        <v>-200</v>
+        <v>-10000</v>
       </c>
       <c r="F12" s="4">
-        <v>-1000</v>
+        <v>-100000</v>
       </c>
       <c r="G12" s="4">
-        <v>-2000</v>
+        <v>-200000</v>
       </c>
       <c r="H12" s="4">
-        <v>-20000</v>
-      </c>
-      <c r="I12" s="4">
-        <v>-100000</v>
-      </c>
-      <c r="J12" s="4">
-        <v>-200000</v>
-      </c>
-      <c r="K12" s="4">
         <v>-600000</v>
       </c>
+      <c r="I12" s="4"/>
+      <c r="K12" s="4"/>
       <c r="L12" s="4"/>
       <c r="M12" s="4"/>
     </row>
@@ -4838,29 +4748,22 @@
         <v>0</v>
       </c>
       <c r="D13" s="4">
-        <v>-100</v>
+        <v>-1000</v>
       </c>
       <c r="E13" s="4">
-        <v>-200</v>
+        <v>-10000</v>
       </c>
       <c r="F13" s="4">
-        <v>-1000</v>
+        <v>-100000</v>
       </c>
       <c r="G13" s="4">
-        <v>-2000</v>
+        <v>-200000</v>
       </c>
       <c r="H13" s="4">
-        <v>-20000</v>
-      </c>
-      <c r="I13" s="4">
-        <v>-100000</v>
-      </c>
-      <c r="J13" s="4">
-        <v>-200000</v>
-      </c>
-      <c r="K13" s="4">
         <v>-600000</v>
       </c>
+      <c r="I13" s="4"/>
+      <c r="K13" s="4"/>
       <c r="L13" s="4"/>
       <c r="M13" s="4"/>
     </row>
@@ -4889,15 +4792,8 @@
       <c r="H14" s="4">
         <v>0</v>
       </c>
-      <c r="I14" s="4">
-        <v>0</v>
-      </c>
-      <c r="J14" s="4">
-        <v>0</v>
-      </c>
-      <c r="K14" s="4">
-        <v>0</v>
-      </c>
+      <c r="I14" s="4"/>
+      <c r="K14" s="4"/>
       <c r="L14" s="4"/>
       <c r="M14" s="4"/>
     </row>
@@ -4912,29 +4808,22 @@
         <v>0</v>
       </c>
       <c r="D15" s="4">
-        <v>-100</v>
+        <v>-1000</v>
       </c>
       <c r="E15" s="4">
-        <v>-200</v>
+        <v>-10000</v>
       </c>
       <c r="F15" s="4">
-        <v>-1000</v>
+        <v>-100000</v>
       </c>
       <c r="G15" s="4">
-        <v>-2000</v>
+        <v>-200000</v>
       </c>
       <c r="H15" s="4">
-        <v>-20000</v>
-      </c>
-      <c r="I15" s="4">
-        <v>-100000</v>
-      </c>
-      <c r="J15" s="4">
-        <v>-200000</v>
-      </c>
-      <c r="K15" s="4">
         <v>-600000</v>
       </c>
+      <c r="I15" s="4"/>
+      <c r="K15" s="4"/>
       <c r="L15" s="4"/>
       <c r="M15" s="4"/>
     </row>
@@ -4949,29 +4838,22 @@
         <v>0</v>
       </c>
       <c r="D16" s="4">
-        <v>-100</v>
+        <v>-1000</v>
       </c>
       <c r="E16" s="4">
-        <v>-200</v>
+        <v>-10000</v>
       </c>
       <c r="F16" s="4">
-        <v>-1000</v>
+        <v>-100000</v>
       </c>
       <c r="G16" s="4">
-        <v>-2000</v>
+        <v>-200000</v>
       </c>
       <c r="H16" s="4">
-        <v>-20000</v>
-      </c>
-      <c r="I16" s="4">
-        <v>-100000</v>
-      </c>
-      <c r="J16" s="4">
-        <v>-200000</v>
-      </c>
-      <c r="K16" s="4">
         <v>-600000</v>
       </c>
+      <c r="I16" s="4"/>
+      <c r="K16" s="4"/>
       <c r="L16" s="4"/>
       <c r="M16" s="4"/>
     </row>
@@ -5229,65 +5111,29 @@
         <v>43</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>1180</v>
+        <v>1157</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>1181</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>1182</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>1183</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>1184</v>
-      </c>
-      <c r="G1" s="19" t="s">
-        <v>1163</v>
-      </c>
-      <c r="H1" s="19" t="s">
-        <v>1164</v>
-      </c>
-      <c r="I1" s="19" t="s">
-        <v>1165</v>
-      </c>
-      <c r="J1" s="19" t="s">
-        <v>1166</v>
-      </c>
-      <c r="K1" s="19" t="s">
-        <v>1167</v>
-      </c>
-      <c r="L1" s="4" t="s">
-        <v>1185</v>
-      </c>
-      <c r="M1" s="4" t="s">
-        <v>1186</v>
-      </c>
-      <c r="N1" s="4" t="s">
-        <v>1187</v>
-      </c>
-      <c r="O1" s="4" t="s">
-        <v>1188</v>
-      </c>
-      <c r="P1" s="4" t="s">
-        <v>1189</v>
-      </c>
-      <c r="Q1" s="19" t="s">
-        <v>1168</v>
-      </c>
-      <c r="R1" s="19" t="s">
-        <v>1169</v>
-      </c>
-      <c r="S1" s="19" t="s">
-        <v>1170</v>
-      </c>
-      <c r="T1" s="19" t="s">
-        <v>1171</v>
-      </c>
-      <c r="U1" s="19" t="s">
-        <v>1172</v>
-      </c>
+        <v>1178</v>
+      </c>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="16"/>
+      <c r="H1" s="16"/>
+      <c r="I1" s="16"/>
+      <c r="J1" s="16"/>
+      <c r="K1" s="16"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
+      <c r="N1" s="4"/>
+      <c r="O1" s="4"/>
+      <c r="P1" s="4"/>
+      <c r="Q1" s="16"/>
+      <c r="R1" s="16"/>
+      <c r="S1" s="16"/>
+      <c r="T1" s="16"/>
+      <c r="U1" s="16"/>
       <c r="V1" s="4"/>
       <c r="W1" s="4"/>
       <c r="X1" s="4"/>
@@ -5314,65 +5160,29 @@
         <v>50</v>
       </c>
       <c r="B2" s="1">
-        <v>8.6400000000000001E-3</v>
+        <v>86.4</v>
       </c>
       <c r="C2" s="1">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="D2" s="1">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="E2" s="1">
-        <v>8.64</v>
-      </c>
-      <c r="F2" s="1">
         <v>86.4</v>
       </c>
-      <c r="G2" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="H2" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="I2" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="J2" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="K2" s="20">
-        <v>86.4</v>
-      </c>
-      <c r="L2" s="1">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="M2" s="1">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="N2" s="1">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="O2" s="1">
-        <v>8.64</v>
-      </c>
-      <c r="P2" s="1">
-        <v>86.4</v>
-      </c>
-      <c r="Q2" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="R2" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="S2" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="T2" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="U2" s="20">
-        <v>86.4</v>
-      </c>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="17"/>
+      <c r="I2" s="17"/>
+      <c r="J2" s="17"/>
+      <c r="K2" s="17"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
+      <c r="N2" s="1"/>
+      <c r="O2" s="1"/>
+      <c r="P2" s="1"/>
+      <c r="Q2" s="17"/>
+      <c r="R2" s="17"/>
+      <c r="S2" s="17"/>
+      <c r="T2" s="17"/>
+      <c r="U2" s="17"/>
       <c r="V2" s="1"/>
       <c r="W2" s="1"/>
       <c r="X2" s="1"/>
@@ -5399,65 +5209,29 @@
         <v>54</v>
       </c>
       <c r="B3" s="13">
-        <v>8.6400000000000003E-6</v>
-      </c>
-      <c r="C3" s="13">
-        <v>8.6400000000000003E-6</v>
-      </c>
-      <c r="D3" s="13">
-        <v>8.6400000000000003E-6</v>
-      </c>
-      <c r="E3" s="13">
-        <v>8.6400000000000003E-6</v>
-      </c>
-      <c r="F3" s="13">
-        <v>8.6400000000000003E-6</v>
-      </c>
-      <c r="G3" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="H3" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="I3" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="J3" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="K3" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="L3" s="13">
-        <v>8.6399999999999997E-4</v>
-      </c>
-      <c r="M3" s="13">
-        <v>8.6399999999999997E-4</v>
-      </c>
-      <c r="N3" s="13">
-        <v>8.6399999999999997E-4</v>
-      </c>
-      <c r="O3" s="13">
-        <v>8.6399999999999997E-4</v>
-      </c>
-      <c r="P3" s="13">
-        <v>8.6399999999999997E-4</v>
-      </c>
-      <c r="Q3" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="R3" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="S3" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="T3" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="U3" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="C3" s="15">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="18"/>
+      <c r="H3" s="18"/>
+      <c r="I3" s="18"/>
+      <c r="J3" s="18"/>
+      <c r="K3" s="18"/>
+      <c r="L3" s="13"/>
+      <c r="M3" s="13"/>
+      <c r="N3" s="13"/>
+      <c r="O3" s="13"/>
+      <c r="P3" s="13"/>
+      <c r="Q3" s="18"/>
+      <c r="R3" s="18"/>
+      <c r="S3" s="18"/>
+      <c r="T3" s="18"/>
+      <c r="U3" s="18"/>
       <c r="V3" s="13"/>
       <c r="W3" s="13"/>
       <c r="X3" s="13"/>
@@ -5484,65 +5258,29 @@
         <v>56</v>
       </c>
       <c r="B4" s="1">
-        <v>8.6400000000000001E-3</v>
+        <v>86.4</v>
       </c>
       <c r="C4" s="1">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="D4" s="1">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="E4" s="1">
-        <v>8.64</v>
-      </c>
-      <c r="F4" s="1">
         <v>86.4</v>
       </c>
-      <c r="G4" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="H4" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="I4" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="J4" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="K4" s="20">
-        <v>86.4</v>
-      </c>
-      <c r="L4" s="1">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="M4" s="1">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="N4" s="1">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="O4" s="1">
-        <v>8.64</v>
-      </c>
-      <c r="P4" s="1">
-        <v>86.4</v>
-      </c>
-      <c r="Q4" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="R4" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="S4" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="T4" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="U4" s="20">
-        <v>86.4</v>
-      </c>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="17"/>
+      <c r="H4" s="17"/>
+      <c r="I4" s="17"/>
+      <c r="J4" s="17"/>
+      <c r="K4" s="17"/>
+      <c r="L4" s="1"/>
+      <c r="M4" s="1"/>
+      <c r="N4" s="1"/>
+      <c r="O4" s="1"/>
+      <c r="P4" s="1"/>
+      <c r="Q4" s="17"/>
+      <c r="R4" s="17"/>
+      <c r="S4" s="17"/>
+      <c r="T4" s="17"/>
+      <c r="U4" s="17"/>
       <c r="V4" s="1"/>
       <c r="W4" s="1"/>
       <c r="X4" s="1"/>
@@ -5569,65 +5307,29 @@
         <v>58</v>
       </c>
       <c r="B5" s="13">
-        <v>8.6400000000000003E-6</v>
-      </c>
-      <c r="C5" s="13">
-        <v>8.6400000000000003E-6</v>
-      </c>
-      <c r="D5" s="13">
-        <v>8.6400000000000003E-6</v>
-      </c>
-      <c r="E5" s="13">
-        <v>8.6400000000000003E-6</v>
-      </c>
-      <c r="F5" s="13">
-        <v>8.6400000000000003E-6</v>
-      </c>
-      <c r="G5" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="H5" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="I5" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="J5" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="K5" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="L5" s="13">
-        <v>8.6399999999999997E-4</v>
-      </c>
-      <c r="M5" s="13">
-        <v>8.6399999999999997E-4</v>
-      </c>
-      <c r="N5" s="13">
-        <v>8.6399999999999997E-4</v>
-      </c>
-      <c r="O5" s="13">
-        <v>8.6399999999999997E-4</v>
-      </c>
-      <c r="P5" s="13">
-        <v>8.6399999999999997E-4</v>
-      </c>
-      <c r="Q5" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="R5" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="S5" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="T5" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="U5" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="C5" s="15">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="13"/>
+      <c r="G5" s="18"/>
+      <c r="H5" s="18"/>
+      <c r="I5" s="18"/>
+      <c r="J5" s="18"/>
+      <c r="K5" s="18"/>
+      <c r="L5" s="13"/>
+      <c r="M5" s="13"/>
+      <c r="N5" s="13"/>
+      <c r="O5" s="13"/>
+      <c r="P5" s="13"/>
+      <c r="Q5" s="18"/>
+      <c r="R5" s="18"/>
+      <c r="S5" s="18"/>
+      <c r="T5" s="18"/>
+      <c r="U5" s="18"/>
       <c r="V5" s="13"/>
       <c r="W5" s="13"/>
       <c r="X5" s="13"/>
@@ -5654,65 +5356,29 @@
         <v>60</v>
       </c>
       <c r="B6" s="1">
-        <v>8.6400000000000001E-3</v>
+        <v>86.4</v>
       </c>
       <c r="C6" s="1">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="D6" s="1">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="E6" s="1">
-        <v>8.64</v>
-      </c>
-      <c r="F6" s="1">
         <v>86.4</v>
       </c>
-      <c r="G6" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="H6" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="I6" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="J6" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="K6" s="20">
-        <v>86.4</v>
-      </c>
-      <c r="L6" s="1">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="M6" s="1">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="N6" s="1">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="O6" s="1">
-        <v>8.64</v>
-      </c>
-      <c r="P6" s="1">
-        <v>86.4</v>
-      </c>
-      <c r="Q6" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="R6" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="S6" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="T6" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="U6" s="20">
-        <v>86.4</v>
-      </c>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+      <c r="F6" s="1"/>
+      <c r="G6" s="17"/>
+      <c r="H6" s="17"/>
+      <c r="I6" s="17"/>
+      <c r="J6" s="17"/>
+      <c r="K6" s="17"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
+      <c r="N6" s="1"/>
+      <c r="O6" s="1"/>
+      <c r="P6" s="1"/>
+      <c r="Q6" s="17"/>
+      <c r="R6" s="17"/>
+      <c r="S6" s="17"/>
+      <c r="T6" s="17"/>
+      <c r="U6" s="17"/>
       <c r="V6" s="1"/>
       <c r="W6" s="1"/>
       <c r="X6" s="1"/>
@@ -5739,65 +5405,29 @@
         <v>62</v>
       </c>
       <c r="B7" s="1">
-        <v>8.6400000000000001E-3</v>
+        <v>86.4</v>
       </c>
       <c r="C7" s="1">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="D7" s="1">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="E7" s="1">
-        <v>8.64</v>
-      </c>
-      <c r="F7" s="1">
         <v>86.4</v>
       </c>
-      <c r="G7" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="H7" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="I7" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="J7" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="K7" s="20">
-        <v>86.4</v>
-      </c>
-      <c r="L7" s="1">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="M7" s="1">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="N7" s="1">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="O7" s="1">
-        <v>8.64</v>
-      </c>
-      <c r="P7" s="1">
-        <v>86.4</v>
-      </c>
-      <c r="Q7" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="R7" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="S7" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="T7" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="U7" s="20">
-        <v>86.4</v>
-      </c>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
+      <c r="G7" s="17"/>
+      <c r="H7" s="17"/>
+      <c r="I7" s="17"/>
+      <c r="J7" s="17"/>
+      <c r="K7" s="17"/>
+      <c r="L7" s="1"/>
+      <c r="M7" s="1"/>
+      <c r="N7" s="1"/>
+      <c r="O7" s="1"/>
+      <c r="P7" s="1"/>
+      <c r="Q7" s="17"/>
+      <c r="R7" s="17"/>
+      <c r="S7" s="17"/>
+      <c r="T7" s="17"/>
+      <c r="U7" s="17"/>
       <c r="V7" s="1"/>
       <c r="W7" s="1"/>
       <c r="X7" s="1"/>
@@ -5824,65 +5454,29 @@
         <v>63</v>
       </c>
       <c r="B8" s="13">
-        <v>8.6400000000000003E-6</v>
-      </c>
-      <c r="C8" s="13">
-        <v>8.6400000000000003E-6</v>
-      </c>
-      <c r="D8" s="13">
-        <v>8.6400000000000003E-6</v>
-      </c>
-      <c r="E8" s="13">
-        <v>8.6400000000000003E-6</v>
-      </c>
-      <c r="F8" s="13">
-        <v>8.6400000000000003E-6</v>
-      </c>
-      <c r="G8" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="H8" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="I8" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="J8" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="K8" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="L8" s="13">
-        <v>8.6399999999999997E-4</v>
-      </c>
-      <c r="M8" s="13">
-        <v>8.6399999999999997E-4</v>
-      </c>
-      <c r="N8" s="13">
-        <v>8.6399999999999997E-4</v>
-      </c>
-      <c r="O8" s="13">
-        <v>8.6399999999999997E-4</v>
-      </c>
-      <c r="P8" s="13">
-        <v>8.6399999999999997E-4</v>
-      </c>
-      <c r="Q8" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="R8" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="S8" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="T8" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="U8" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="C8" s="15">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="D8" s="13"/>
+      <c r="E8" s="13"/>
+      <c r="F8" s="13"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="18"/>
+      <c r="I8" s="18"/>
+      <c r="J8" s="18"/>
+      <c r="K8" s="18"/>
+      <c r="L8" s="13"/>
+      <c r="M8" s="13"/>
+      <c r="N8" s="13"/>
+      <c r="O8" s="13"/>
+      <c r="P8" s="13"/>
+      <c r="Q8" s="18"/>
+      <c r="R8" s="18"/>
+      <c r="S8" s="18"/>
+      <c r="T8" s="18"/>
+      <c r="U8" s="18"/>
       <c r="V8" s="13"/>
       <c r="W8" s="13"/>
       <c r="X8" s="13"/>
@@ -5909,65 +5503,29 @@
         <v>64</v>
       </c>
       <c r="B9" s="1">
-        <v>8.6400000000000001E-3</v>
+        <v>86.4</v>
       </c>
       <c r="C9" s="1">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="D9" s="1">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="E9" s="1">
-        <v>8.64</v>
-      </c>
-      <c r="F9" s="1">
         <v>86.4</v>
       </c>
-      <c r="G9" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="H9" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="I9" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="J9" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="K9" s="20">
-        <v>86.4</v>
-      </c>
-      <c r="L9" s="1">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="M9" s="1">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="N9" s="1">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="O9" s="1">
-        <v>8.64</v>
-      </c>
-      <c r="P9" s="1">
-        <v>86.4</v>
-      </c>
-      <c r="Q9" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="R9" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="S9" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="T9" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="U9" s="20">
-        <v>86.4</v>
-      </c>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1"/>
+      <c r="G9" s="17"/>
+      <c r="H9" s="17"/>
+      <c r="I9" s="17"/>
+      <c r="J9" s="17"/>
+      <c r="K9" s="17"/>
+      <c r="L9" s="1"/>
+      <c r="M9" s="1"/>
+      <c r="N9" s="1"/>
+      <c r="O9" s="1"/>
+      <c r="P9" s="1"/>
+      <c r="Q9" s="17"/>
+      <c r="R9" s="17"/>
+      <c r="S9" s="17"/>
+      <c r="T9" s="17"/>
+      <c r="U9" s="17"/>
       <c r="V9" s="1"/>
       <c r="W9" s="1"/>
       <c r="X9" s="1"/>
@@ -5994,65 +5552,29 @@
         <v>65</v>
       </c>
       <c r="B10" s="13">
-        <v>8.6400000000000003E-6</v>
-      </c>
-      <c r="C10" s="13">
-        <v>8.6400000000000003E-6</v>
-      </c>
-      <c r="D10" s="13">
-        <v>8.6400000000000003E-6</v>
-      </c>
-      <c r="E10" s="13">
-        <v>8.6400000000000003E-6</v>
-      </c>
-      <c r="F10" s="13">
-        <v>8.6400000000000003E-6</v>
-      </c>
-      <c r="G10" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="H10" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="I10" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="J10" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="K10" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="L10" s="13">
-        <v>8.6399999999999997E-4</v>
-      </c>
-      <c r="M10" s="13">
-        <v>8.6399999999999997E-4</v>
-      </c>
-      <c r="N10" s="13">
-        <v>8.6399999999999997E-4</v>
-      </c>
-      <c r="O10" s="13">
-        <v>8.6399999999999997E-4</v>
-      </c>
-      <c r="P10" s="13">
-        <v>8.6399999999999997E-4</v>
-      </c>
-      <c r="Q10" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="R10" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="S10" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="T10" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="U10" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="C10" s="15">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="D10" s="13"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="18"/>
+      <c r="H10" s="18"/>
+      <c r="I10" s="18"/>
+      <c r="J10" s="18"/>
+      <c r="K10" s="18"/>
+      <c r="L10" s="13"/>
+      <c r="M10" s="13"/>
+      <c r="N10" s="13"/>
+      <c r="O10" s="13"/>
+      <c r="P10" s="13"/>
+      <c r="Q10" s="18"/>
+      <c r="R10" s="18"/>
+      <c r="S10" s="18"/>
+      <c r="T10" s="18"/>
+      <c r="U10" s="18"/>
       <c r="V10" s="13"/>
       <c r="W10" s="13"/>
       <c r="X10" s="13"/>
@@ -6079,65 +5601,29 @@
         <v>66</v>
       </c>
       <c r="B11" s="1">
-        <v>8.6400000000000001E-3</v>
+        <v>86.4</v>
       </c>
       <c r="C11" s="1">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="D11" s="1">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="E11" s="1">
-        <v>8.64</v>
-      </c>
-      <c r="F11" s="1">
         <v>86.4</v>
       </c>
-      <c r="G11" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="H11" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="I11" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="J11" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="K11" s="20">
-        <v>86.4</v>
-      </c>
-      <c r="L11" s="1">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="M11" s="1">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="N11" s="1">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="O11" s="1">
-        <v>8.64</v>
-      </c>
-      <c r="P11" s="1">
-        <v>86.4</v>
-      </c>
-      <c r="Q11" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="R11" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="S11" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="T11" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="U11" s="20">
-        <v>86.4</v>
-      </c>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+      <c r="G11" s="17"/>
+      <c r="H11" s="17"/>
+      <c r="I11" s="17"/>
+      <c r="J11" s="17"/>
+      <c r="K11" s="17"/>
+      <c r="L11" s="1"/>
+      <c r="M11" s="1"/>
+      <c r="N11" s="1"/>
+      <c r="O11" s="1"/>
+      <c r="P11" s="1"/>
+      <c r="Q11" s="17"/>
+      <c r="R11" s="17"/>
+      <c r="S11" s="17"/>
+      <c r="T11" s="17"/>
+      <c r="U11" s="17"/>
       <c r="V11" s="1"/>
       <c r="W11" s="1"/>
       <c r="X11" s="1"/>
@@ -6648,6 +6134,7 @@
   <cols>
     <col min="1" max="1" width="15.46484375" style="4" bestFit="1" customWidth="1"/>
     <col min="32" max="32" width="18.59765625" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="27.19921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:37" x14ac:dyDescent="0.45">
@@ -13454,63 +12941,33 @@
         <v>43</v>
       </c>
       <c r="AF91" s="16" t="s">
-        <v>1153</v>
+        <v>1163</v>
       </c>
       <c r="AG91" s="16" t="s">
-        <v>1154</v>
+        <v>1164</v>
       </c>
       <c r="AH91" s="16" t="s">
-        <v>1155</v>
+        <v>1165</v>
       </c>
       <c r="AI91" s="16" t="s">
-        <v>1156</v>
+        <v>1166</v>
       </c>
       <c r="AJ91" s="16" t="s">
-        <v>1157</v>
+        <v>1167</v>
       </c>
       <c r="AK91" s="16" t="s">
-        <v>1158</v>
+        <v>1168</v>
       </c>
       <c r="AL91" s="16" t="s">
-        <v>1159</v>
+        <v>1169</v>
       </c>
       <c r="AM91" s="16" t="s">
-        <v>1160</v>
+        <v>1170</v>
       </c>
       <c r="AN91" s="16" t="s">
-        <v>1161</v>
+        <v>1171</v>
       </c>
       <c r="AO91" s="16" t="s">
-        <v>1162</v>
-      </c>
-      <c r="AP91" s="19" t="s">
-        <v>1163</v>
-      </c>
-      <c r="AQ91" s="19" t="s">
-        <v>1164</v>
-      </c>
-      <c r="AR91" s="19" t="s">
-        <v>1165</v>
-      </c>
-      <c r="AS91" s="19" t="s">
-        <v>1166</v>
-      </c>
-      <c r="AT91" s="19" t="s">
-        <v>1167</v>
-      </c>
-      <c r="AU91" s="19" t="s">
-        <v>1168</v>
-      </c>
-      <c r="AV91" s="19" t="s">
-        <v>1169</v>
-      </c>
-      <c r="AW91" s="19" t="s">
-        <v>1170</v>
-      </c>
-      <c r="AX91" s="19" t="s">
-        <v>1171</v>
-      </c>
-      <c r="AY91" s="19" t="s">
         <v>1172</v>
       </c>
       <c r="BN91" s="4" t="s">
@@ -13639,36 +13096,6 @@
       <c r="AO92" s="17">
         <v>86.4</v>
       </c>
-      <c r="AP92" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AQ92" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="AR92" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="AS92" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="AT92" s="20">
-        <v>86.4</v>
-      </c>
-      <c r="AU92" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AV92" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="AW92" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="AX92" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="AY92" s="20">
-        <v>86.4</v>
-      </c>
       <c r="BN92" s="4" t="s">
         <v>93</v>
       </c>
@@ -13766,63 +13193,33 @@
         <v>54</v>
       </c>
       <c r="AF93" s="18">
-        <v>8.6399999999999999E-9</v>
+        <v>8.6399999999999999E-5</v>
       </c>
       <c r="AG93" s="18">
-        <v>8.6399999999999999E-9</v>
+        <v>8.6399999999999999E-5</v>
       </c>
       <c r="AH93" s="18">
-        <v>8.6399999999999999E-9</v>
+        <v>8.6399999999999999E-5</v>
       </c>
       <c r="AI93" s="18">
-        <v>8.6399999999999999E-9</v>
+        <v>8.6399999999999999E-5</v>
       </c>
       <c r="AJ93" s="18">
-        <v>8.6399999999999999E-9</v>
+        <v>8.6399999999999999E-5</v>
       </c>
       <c r="AK93" s="18">
-        <v>8.6400000000000001E-7</v>
+        <v>8.6400000000000001E-3</v>
       </c>
       <c r="AL93" s="18">
-        <v>8.6400000000000001E-7</v>
+        <v>8.6400000000000001E-3</v>
       </c>
       <c r="AM93" s="18">
-        <v>8.6400000000000001E-7</v>
+        <v>8.6400000000000001E-3</v>
       </c>
       <c r="AN93" s="18">
-        <v>8.6400000000000001E-7</v>
+        <v>8.6400000000000001E-3</v>
       </c>
       <c r="AO93" s="18">
-        <v>8.6400000000000001E-7</v>
-      </c>
-      <c r="AP93" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="AQ93" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="AR93" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="AS93" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="AT93" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="AU93" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AV93" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AW93" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AX93" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AY93" s="21">
         <v>8.6400000000000001E-3</v>
       </c>
       <c r="BN93" s="4" t="s">
@@ -13951,36 +13348,6 @@
       <c r="AO94" s="17">
         <v>86.4</v>
       </c>
-      <c r="AP94" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AQ94" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="AR94" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="AS94" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="AT94" s="20">
-        <v>86.4</v>
-      </c>
-      <c r="AU94" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AV94" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="AW94" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="AX94" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="AY94" s="20">
-        <v>86.4</v>
-      </c>
       <c r="BN94" s="4" t="s">
         <v>94</v>
       </c>
@@ -14078,63 +13445,33 @@
         <v>58</v>
       </c>
       <c r="AF95" s="18">
-        <v>8.6399999999999999E-9</v>
+        <v>8.6399999999999999E-5</v>
       </c>
       <c r="AG95" s="18">
-        <v>8.6399999999999999E-9</v>
+        <v>8.6399999999999999E-5</v>
       </c>
       <c r="AH95" s="18">
-        <v>8.6399999999999999E-9</v>
+        <v>8.6399999999999999E-5</v>
       </c>
       <c r="AI95" s="18">
-        <v>8.6399999999999999E-9</v>
+        <v>8.6399999999999999E-5</v>
       </c>
       <c r="AJ95" s="18">
-        <v>8.6399999999999999E-9</v>
+        <v>8.6399999999999999E-5</v>
       </c>
       <c r="AK95" s="18">
-        <v>8.6400000000000001E-7</v>
+        <v>8.6400000000000001E-3</v>
       </c>
       <c r="AL95" s="18">
-        <v>8.6400000000000001E-7</v>
+        <v>8.6400000000000001E-3</v>
       </c>
       <c r="AM95" s="18">
-        <v>8.6400000000000001E-7</v>
+        <v>8.6400000000000001E-3</v>
       </c>
       <c r="AN95" s="18">
-        <v>8.6400000000000001E-7</v>
+        <v>8.6400000000000001E-3</v>
       </c>
       <c r="AO95" s="18">
-        <v>8.6400000000000001E-7</v>
-      </c>
-      <c r="AP95" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="AQ95" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="AR95" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="AS95" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="AT95" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="AU95" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AV95" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AW95" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AX95" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AY95" s="21">
         <v>8.6400000000000001E-3</v>
       </c>
       <c r="BN95" s="4" t="s">
@@ -14263,36 +13600,6 @@
       <c r="AO96" s="17">
         <v>86.4</v>
       </c>
-      <c r="AP96" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AQ96" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="AR96" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="AS96" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="AT96" s="20">
-        <v>86.4</v>
-      </c>
-      <c r="AU96" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AV96" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="AW96" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="AX96" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="AY96" s="20">
-        <v>86.4</v>
-      </c>
       <c r="BN96" s="4" t="s">
         <v>94</v>
       </c>
@@ -14419,36 +13726,6 @@
       <c r="AO97" s="17">
         <v>86.4</v>
       </c>
-      <c r="AP97" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AQ97" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="AR97" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="AS97" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="AT97" s="20">
-        <v>86.4</v>
-      </c>
-      <c r="AU97" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AV97" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="AW97" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="AX97" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="AY97" s="20">
-        <v>86.4</v>
-      </c>
       <c r="BN97" s="4" t="s">
         <v>95</v>
       </c>
@@ -14546,63 +13823,33 @@
         <v>63</v>
       </c>
       <c r="AF98" s="18">
-        <v>8.6399999999999999E-9</v>
+        <v>8.6399999999999999E-5</v>
       </c>
       <c r="AG98" s="18">
-        <v>8.6399999999999999E-9</v>
+        <v>8.6399999999999999E-5</v>
       </c>
       <c r="AH98" s="18">
-        <v>8.6399999999999999E-9</v>
+        <v>8.6399999999999999E-5</v>
       </c>
       <c r="AI98" s="18">
-        <v>8.6399999999999999E-9</v>
+        <v>8.6399999999999999E-5</v>
       </c>
       <c r="AJ98" s="18">
-        <v>8.6399999999999999E-9</v>
+        <v>8.6399999999999999E-5</v>
       </c>
       <c r="AK98" s="18">
-        <v>8.6400000000000001E-7</v>
+        <v>8.6400000000000001E-3</v>
       </c>
       <c r="AL98" s="18">
-        <v>8.6400000000000001E-7</v>
+        <v>8.6400000000000001E-3</v>
       </c>
       <c r="AM98" s="18">
-        <v>8.6400000000000001E-7</v>
+        <v>8.6400000000000001E-3</v>
       </c>
       <c r="AN98" s="18">
-        <v>8.6400000000000001E-7</v>
+        <v>8.6400000000000001E-3</v>
       </c>
       <c r="AO98" s="18">
-        <v>8.6400000000000001E-7</v>
-      </c>
-      <c r="AP98" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="AQ98" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="AR98" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="AS98" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="AT98" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="AU98" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AV98" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AW98" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AX98" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AY98" s="21">
         <v>8.6400000000000001E-3</v>
       </c>
       <c r="BN98" s="4" t="s">
@@ -14731,36 +13978,6 @@
       <c r="AO99" s="17">
         <v>86.4</v>
       </c>
-      <c r="AP99" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AQ99" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="AR99" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="AS99" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="AT99" s="20">
-        <v>86.4</v>
-      </c>
-      <c r="AU99" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AV99" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="AW99" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="AX99" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="AY99" s="20">
-        <v>86.4</v>
-      </c>
       <c r="BN99" s="4" t="s">
         <v>95</v>
       </c>
@@ -14858,63 +14075,33 @@
         <v>65</v>
       </c>
       <c r="AF100" s="18">
-        <v>8.6399999999999999E-9</v>
+        <v>8.6399999999999999E-5</v>
       </c>
       <c r="AG100" s="18">
-        <v>8.6399999999999999E-9</v>
+        <v>8.6399999999999999E-5</v>
       </c>
       <c r="AH100" s="18">
-        <v>8.6399999999999999E-9</v>
+        <v>8.6399999999999999E-5</v>
       </c>
       <c r="AI100" s="18">
-        <v>8.6399999999999999E-9</v>
+        <v>8.6399999999999999E-5</v>
       </c>
       <c r="AJ100" s="18">
-        <v>8.6399999999999999E-9</v>
+        <v>8.6399999999999999E-5</v>
       </c>
       <c r="AK100" s="18">
-        <v>8.6400000000000001E-7</v>
+        <v>8.6400000000000001E-3</v>
       </c>
       <c r="AL100" s="18">
-        <v>8.6400000000000001E-7</v>
+        <v>8.6400000000000001E-3</v>
       </c>
       <c r="AM100" s="18">
-        <v>8.6400000000000001E-7</v>
+        <v>8.6400000000000001E-3</v>
       </c>
       <c r="AN100" s="18">
-        <v>8.6400000000000001E-7</v>
+        <v>8.6400000000000001E-3</v>
       </c>
       <c r="AO100" s="18">
-        <v>8.6400000000000001E-7</v>
-      </c>
-      <c r="AP100" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="AQ100" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="AR100" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="AS100" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="AT100" s="21">
-        <v>8.6399999999999999E-5</v>
-      </c>
-      <c r="AU100" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AV100" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AW100" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AX100" s="21">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AY100" s="21">
         <v>8.6400000000000001E-3</v>
       </c>
       <c r="BN100" s="4" t="s">
@@ -15043,36 +14230,6 @@
       <c r="AO101" s="17">
         <v>86.4</v>
       </c>
-      <c r="AP101" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AQ101" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="AR101" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="AS101" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="AT101" s="20">
-        <v>86.4</v>
-      </c>
-      <c r="AU101" s="20">
-        <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="AV101" s="20">
-        <v>8.6400000000000005E-2</v>
-      </c>
-      <c r="AW101" s="20">
-        <v>0.86399999999999999</v>
-      </c>
-      <c r="AX101" s="20">
-        <v>8.64</v>
-      </c>
-      <c r="AY101" s="20">
-        <v>86.4</v>
-      </c>
       <c r="BN101" s="4" t="s">
         <v>96</v>
       </c>
@@ -15260,7 +14417,7 @@
         <v>6.1373542849109256E-4</v>
       </c>
       <c r="AE103" s="14" t="s">
-        <v>1174</v>
+        <v>1190</v>
       </c>
       <c r="BN103" s="4" t="s">
         <v>97</v>
@@ -15374,19 +14531,19 @@
         <v>1157</v>
       </c>
       <c r="AK104" s="4" t="s">
+        <v>1174</v>
+      </c>
+      <c r="AL104" s="4" t="s">
         <v>1175</v>
       </c>
-      <c r="AL104" s="4" t="s">
+      <c r="AM104" s="4" t="s">
         <v>1176</v>
       </c>
-      <c r="AM104" s="4" t="s">
+      <c r="AN104" s="4" t="s">
         <v>1177</v>
       </c>
-      <c r="AN104" s="4" t="s">
+      <c r="AO104" s="4" t="s">
         <v>1178</v>
-      </c>
-      <c r="AO104" s="4" t="s">
-        <v>1179</v>
       </c>
       <c r="AP104" s="4" t="s">
         <v>1158</v>
@@ -15890,7 +15047,7 @@
         <v>8.6400000000000001E-7</v>
       </c>
       <c r="BN108" t="s">
-        <v>1174</v>
+        <v>1190</v>
       </c>
     </row>
     <row r="109" spans="1:78" x14ac:dyDescent="0.45">
@@ -16886,7 +16043,7 @@
         <v>9.0184342071178349E-4</v>
       </c>
       <c r="AE116" s="14" t="s">
-        <v>1190</v>
+        <v>1191</v>
       </c>
       <c r="AF116" s="4"/>
       <c r="AG116" s="4"/>
@@ -16990,63 +16147,63 @@
         <v>43</v>
       </c>
       <c r="AF117" s="4" t="s">
+        <v>1179</v>
+      </c>
+      <c r="AG117" s="4" t="s">
         <v>1180</v>
       </c>
-      <c r="AG117" s="4" t="s">
+      <c r="AH117" s="4" t="s">
         <v>1181</v>
       </c>
-      <c r="AH117" s="4" t="s">
+      <c r="AI117" s="4" t="s">
         <v>1182</v>
       </c>
-      <c r="AI117" s="4" t="s">
+      <c r="AJ117" s="4" t="s">
         <v>1183</v>
       </c>
-      <c r="AJ117" s="4" t="s">
+      <c r="AK117" s="16" t="s">
+        <v>1163</v>
+      </c>
+      <c r="AL117" s="16" t="s">
+        <v>1164</v>
+      </c>
+      <c r="AM117" s="16" t="s">
+        <v>1165</v>
+      </c>
+      <c r="AN117" s="16" t="s">
+        <v>1166</v>
+      </c>
+      <c r="AO117" s="16" t="s">
+        <v>1167</v>
+      </c>
+      <c r="AP117" s="4" t="s">
         <v>1184</v>
       </c>
-      <c r="AK117" s="19" t="s">
-        <v>1163</v>
-      </c>
-      <c r="AL117" s="19" t="s">
-        <v>1164</v>
-      </c>
-      <c r="AM117" s="19" t="s">
-        <v>1165</v>
-      </c>
-      <c r="AN117" s="19" t="s">
-        <v>1166</v>
-      </c>
-      <c r="AO117" s="19" t="s">
-        <v>1167</v>
-      </c>
-      <c r="AP117" s="4" t="s">
+      <c r="AQ117" s="4" t="s">
         <v>1185</v>
       </c>
-      <c r="AQ117" s="4" t="s">
+      <c r="AR117" s="4" t="s">
         <v>1186</v>
       </c>
-      <c r="AR117" s="4" t="s">
+      <c r="AS117" s="4" t="s">
         <v>1187</v>
       </c>
-      <c r="AS117" s="4" t="s">
+      <c r="AT117" s="4" t="s">
         <v>1188</v>
       </c>
-      <c r="AT117" s="4" t="s">
-        <v>1189</v>
-      </c>
-      <c r="AU117" s="19" t="s">
+      <c r="AU117" s="16" t="s">
         <v>1168</v>
       </c>
-      <c r="AV117" s="19" t="s">
+      <c r="AV117" s="16" t="s">
         <v>1169</v>
       </c>
-      <c r="AW117" s="19" t="s">
+      <c r="AW117" s="16" t="s">
         <v>1170</v>
       </c>
-      <c r="AX117" s="19" t="s">
+      <c r="AX117" s="16" t="s">
         <v>1171</v>
       </c>
-      <c r="AY117" s="19" t="s">
+      <c r="AY117" s="16" t="s">
         <v>1172</v>
       </c>
       <c r="AZ117" s="4"/>
@@ -17165,19 +16322,19 @@
       <c r="AJ118" s="1">
         <v>86.4</v>
       </c>
-      <c r="AK118" s="20">
+      <c r="AK118" s="17">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AL118" s="20">
+      <c r="AL118" s="17">
         <v>8.6400000000000005E-2</v>
       </c>
-      <c r="AM118" s="20">
+      <c r="AM118" s="17">
         <v>0.86399999999999999</v>
       </c>
-      <c r="AN118" s="20">
+      <c r="AN118" s="17">
         <v>8.64</v>
       </c>
-      <c r="AO118" s="20">
+      <c r="AO118" s="17">
         <v>86.4</v>
       </c>
       <c r="AP118" s="1">
@@ -17195,19 +16352,19 @@
       <c r="AT118" s="1">
         <v>86.4</v>
       </c>
-      <c r="AU118" s="20">
+      <c r="AU118" s="17">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AV118" s="20">
+      <c r="AV118" s="17">
         <v>8.6400000000000005E-2</v>
       </c>
-      <c r="AW118" s="20">
+      <c r="AW118" s="17">
         <v>0.86399999999999999</v>
       </c>
-      <c r="AX118" s="20">
+      <c r="AX118" s="17">
         <v>8.64</v>
       </c>
-      <c r="AY118" s="20">
+      <c r="AY118" s="17">
         <v>86.4</v>
       </c>
       <c r="AZ118" s="1"/>
@@ -17326,19 +16483,19 @@
       <c r="AJ119" s="13">
         <v>8.6400000000000003E-6</v>
       </c>
-      <c r="AK119" s="21">
+      <c r="AK119" s="18">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="AL119" s="21">
+      <c r="AL119" s="18">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="AM119" s="21">
+      <c r="AM119" s="18">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="AN119" s="21">
+      <c r="AN119" s="18">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="AO119" s="21">
+      <c r="AO119" s="18">
         <v>8.6399999999999999E-5</v>
       </c>
       <c r="AP119" s="13">
@@ -17356,19 +16513,19 @@
       <c r="AT119" s="13">
         <v>8.6399999999999997E-4</v>
       </c>
-      <c r="AU119" s="21">
+      <c r="AU119" s="18">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AV119" s="21">
+      <c r="AV119" s="18">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AW119" s="21">
+      <c r="AW119" s="18">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AX119" s="21">
+      <c r="AX119" s="18">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AY119" s="21">
+      <c r="AY119" s="18">
         <v>8.6400000000000001E-3</v>
       </c>
       <c r="AZ119" s="13"/>
@@ -17487,19 +16644,19 @@
       <c r="AJ120" s="1">
         <v>86.4</v>
       </c>
-      <c r="AK120" s="20">
+      <c r="AK120" s="17">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AL120" s="20">
+      <c r="AL120" s="17">
         <v>8.6400000000000005E-2</v>
       </c>
-      <c r="AM120" s="20">
+      <c r="AM120" s="17">
         <v>0.86399999999999999</v>
       </c>
-      <c r="AN120" s="20">
+      <c r="AN120" s="17">
         <v>8.64</v>
       </c>
-      <c r="AO120" s="20">
+      <c r="AO120" s="17">
         <v>86.4</v>
       </c>
       <c r="AP120" s="1">
@@ -17517,19 +16674,19 @@
       <c r="AT120" s="1">
         <v>86.4</v>
       </c>
-      <c r="AU120" s="20">
+      <c r="AU120" s="17">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AV120" s="20">
+      <c r="AV120" s="17">
         <v>8.6400000000000005E-2</v>
       </c>
-      <c r="AW120" s="20">
+      <c r="AW120" s="17">
         <v>0.86399999999999999</v>
       </c>
-      <c r="AX120" s="20">
+      <c r="AX120" s="17">
         <v>8.64</v>
       </c>
-      <c r="AY120" s="20">
+      <c r="AY120" s="17">
         <v>86.4</v>
       </c>
       <c r="AZ120" s="1"/>
@@ -17648,19 +16805,19 @@
       <c r="AJ121" s="13">
         <v>8.6400000000000003E-6</v>
       </c>
-      <c r="AK121" s="21">
+      <c r="AK121" s="18">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="AL121" s="21">
+      <c r="AL121" s="18">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="AM121" s="21">
+      <c r="AM121" s="18">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="AN121" s="21">
+      <c r="AN121" s="18">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="AO121" s="21">
+      <c r="AO121" s="18">
         <v>8.6399999999999999E-5</v>
       </c>
       <c r="AP121" s="13">
@@ -17678,19 +16835,19 @@
       <c r="AT121" s="13">
         <v>8.6399999999999997E-4</v>
       </c>
-      <c r="AU121" s="21">
+      <c r="AU121" s="18">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AV121" s="21">
+      <c r="AV121" s="18">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AW121" s="21">
+      <c r="AW121" s="18">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AX121" s="21">
+      <c r="AX121" s="18">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AY121" s="21">
+      <c r="AY121" s="18">
         <v>8.6400000000000001E-3</v>
       </c>
       <c r="AZ121" s="13"/>
@@ -17809,19 +16966,19 @@
       <c r="AJ122" s="1">
         <v>86.4</v>
       </c>
-      <c r="AK122" s="20">
+      <c r="AK122" s="17">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AL122" s="20">
+      <c r="AL122" s="17">
         <v>8.6400000000000005E-2</v>
       </c>
-      <c r="AM122" s="20">
+      <c r="AM122" s="17">
         <v>0.86399999999999999</v>
       </c>
-      <c r="AN122" s="20">
+      <c r="AN122" s="17">
         <v>8.64</v>
       </c>
-      <c r="AO122" s="20">
+      <c r="AO122" s="17">
         <v>86.4</v>
       </c>
       <c r="AP122" s="1">
@@ -17839,19 +16996,19 @@
       <c r="AT122" s="1">
         <v>86.4</v>
       </c>
-      <c r="AU122" s="20">
+      <c r="AU122" s="17">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AV122" s="20">
+      <c r="AV122" s="17">
         <v>8.6400000000000005E-2</v>
       </c>
-      <c r="AW122" s="20">
+      <c r="AW122" s="17">
         <v>0.86399999999999999</v>
       </c>
-      <c r="AX122" s="20">
+      <c r="AX122" s="17">
         <v>8.64</v>
       </c>
-      <c r="AY122" s="20">
+      <c r="AY122" s="17">
         <v>86.4</v>
       </c>
       <c r="AZ122" s="1"/>
@@ -17970,19 +17127,19 @@
       <c r="AJ123" s="1">
         <v>86.4</v>
       </c>
-      <c r="AK123" s="20">
+      <c r="AK123" s="17">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AL123" s="20">
+      <c r="AL123" s="17">
         <v>8.6400000000000005E-2</v>
       </c>
-      <c r="AM123" s="20">
+      <c r="AM123" s="17">
         <v>0.86399999999999999</v>
       </c>
-      <c r="AN123" s="20">
+      <c r="AN123" s="17">
         <v>8.64</v>
       </c>
-      <c r="AO123" s="20">
+      <c r="AO123" s="17">
         <v>86.4</v>
       </c>
       <c r="AP123" s="1">
@@ -18000,19 +17157,19 @@
       <c r="AT123" s="1">
         <v>86.4</v>
       </c>
-      <c r="AU123" s="20">
+      <c r="AU123" s="17">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AV123" s="20">
+      <c r="AV123" s="17">
         <v>8.6400000000000005E-2</v>
       </c>
-      <c r="AW123" s="20">
+      <c r="AW123" s="17">
         <v>0.86399999999999999</v>
       </c>
-      <c r="AX123" s="20">
+      <c r="AX123" s="17">
         <v>8.64</v>
       </c>
-      <c r="AY123" s="20">
+      <c r="AY123" s="17">
         <v>86.4</v>
       </c>
       <c r="AZ123" s="1"/>
@@ -18131,19 +17288,19 @@
       <c r="AJ124" s="13">
         <v>8.6400000000000003E-6</v>
       </c>
-      <c r="AK124" s="21">
+      <c r="AK124" s="18">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="AL124" s="21">
+      <c r="AL124" s="18">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="AM124" s="21">
+      <c r="AM124" s="18">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="AN124" s="21">
+      <c r="AN124" s="18">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="AO124" s="21">
+      <c r="AO124" s="18">
         <v>8.6399999999999999E-5</v>
       </c>
       <c r="AP124" s="13">
@@ -18161,19 +17318,19 @@
       <c r="AT124" s="13">
         <v>8.6399999999999997E-4</v>
       </c>
-      <c r="AU124" s="21">
+      <c r="AU124" s="18">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AV124" s="21">
+      <c r="AV124" s="18">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AW124" s="21">
+      <c r="AW124" s="18">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AX124" s="21">
+      <c r="AX124" s="18">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AY124" s="21">
+      <c r="AY124" s="18">
         <v>8.6400000000000001E-3</v>
       </c>
       <c r="AZ124" s="13"/>
@@ -18292,19 +17449,19 @@
       <c r="AJ125" s="1">
         <v>86.4</v>
       </c>
-      <c r="AK125" s="20">
+      <c r="AK125" s="17">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AL125" s="20">
+      <c r="AL125" s="17">
         <v>8.6400000000000005E-2</v>
       </c>
-      <c r="AM125" s="20">
+      <c r="AM125" s="17">
         <v>0.86399999999999999</v>
       </c>
-      <c r="AN125" s="20">
+      <c r="AN125" s="17">
         <v>8.64</v>
       </c>
-      <c r="AO125" s="20">
+      <c r="AO125" s="17">
         <v>86.4</v>
       </c>
       <c r="AP125" s="1">
@@ -18322,19 +17479,19 @@
       <c r="AT125" s="1">
         <v>86.4</v>
       </c>
-      <c r="AU125" s="20">
+      <c r="AU125" s="17">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AV125" s="20">
+      <c r="AV125" s="17">
         <v>8.6400000000000005E-2</v>
       </c>
-      <c r="AW125" s="20">
+      <c r="AW125" s="17">
         <v>0.86399999999999999</v>
       </c>
-      <c r="AX125" s="20">
+      <c r="AX125" s="17">
         <v>8.64</v>
       </c>
-      <c r="AY125" s="20">
+      <c r="AY125" s="17">
         <v>86.4</v>
       </c>
       <c r="AZ125" s="1"/>
@@ -18414,19 +17571,19 @@
       <c r="AJ126" s="13">
         <v>8.6400000000000003E-6</v>
       </c>
-      <c r="AK126" s="21">
+      <c r="AK126" s="18">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="AL126" s="21">
+      <c r="AL126" s="18">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="AM126" s="21">
+      <c r="AM126" s="18">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="AN126" s="21">
+      <c r="AN126" s="18">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="AO126" s="21">
+      <c r="AO126" s="18">
         <v>8.6399999999999999E-5</v>
       </c>
       <c r="AP126" s="13">
@@ -18444,19 +17601,19 @@
       <c r="AT126" s="13">
         <v>8.6399999999999997E-4</v>
       </c>
-      <c r="AU126" s="21">
+      <c r="AU126" s="18">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AV126" s="21">
+      <c r="AV126" s="18">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AW126" s="21">
+      <c r="AW126" s="18">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AX126" s="21">
+      <c r="AX126" s="18">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AY126" s="21">
+      <c r="AY126" s="18">
         <v>8.6400000000000001E-3</v>
       </c>
       <c r="AZ126" s="13"/>
@@ -18536,19 +17693,19 @@
       <c r="AJ127" s="1">
         <v>86.4</v>
       </c>
-      <c r="AK127" s="20">
+      <c r="AK127" s="17">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AL127" s="20">
+      <c r="AL127" s="17">
         <v>8.6400000000000005E-2</v>
       </c>
-      <c r="AM127" s="20">
+      <c r="AM127" s="17">
         <v>0.86399999999999999</v>
       </c>
-      <c r="AN127" s="20">
+      <c r="AN127" s="17">
         <v>8.64</v>
       </c>
-      <c r="AO127" s="20">
+      <c r="AO127" s="17">
         <v>86.4</v>
       </c>
       <c r="AP127" s="1">
@@ -18566,19 +17723,19 @@
       <c r="AT127" s="1">
         <v>86.4</v>
       </c>
-      <c r="AU127" s="20">
+      <c r="AU127" s="17">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="AV127" s="20">
+      <c r="AV127" s="17">
         <v>8.6400000000000005E-2</v>
       </c>
-      <c r="AW127" s="20">
+      <c r="AW127" s="17">
         <v>0.86399999999999999</v>
       </c>
-      <c r="AX127" s="20">
+      <c r="AX127" s="17">
         <v>8.64</v>
       </c>
-      <c r="AY127" s="20">
+      <c r="AY127" s="17">
         <v>86.4</v>
       </c>
       <c r="AZ127" s="1"/>
@@ -18587,7 +17744,7 @@
       <c r="BC127" s="1"/>
       <c r="BD127" s="1"/>
       <c r="BN127" t="s">
-        <v>1190</v>
+        <v>1191</v>
       </c>
     </row>
     <row r="128" spans="1:78" x14ac:dyDescent="0.45">
@@ -18731,6 +17888,9 @@
       <c r="AA129" s="1">
         <f t="shared" si="15"/>
         <v>6.7192904177343729E-4</v>
+      </c>
+      <c r="AE129" s="14" t="s">
+        <v>1189</v>
       </c>
       <c r="AF129" s="1"/>
       <c r="AG129" s="1"/>
@@ -18834,8 +17994,15 @@
         <f t="shared" ref="AA130:AA154" si="19">+W130</f>
         <v>6.8402164621609858E-4</v>
       </c>
-      <c r="AF130" s="1"/>
-      <c r="AG130" s="1"/>
+      <c r="AE130" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="AF130" s="4" t="s">
+        <v>1157</v>
+      </c>
+      <c r="AG130" s="4" t="s">
+        <v>1178</v>
+      </c>
       <c r="AH130" s="1"/>
       <c r="AI130" s="1"/>
       <c r="AJ130" s="1"/>
@@ -18936,8 +18103,15 @@
         <f t="shared" si="19"/>
         <v>7.3510433221211555E-4</v>
       </c>
-      <c r="AF131" s="1"/>
-      <c r="AG131" s="1"/>
+      <c r="AE131" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="AF131" s="1">
+        <v>86.4</v>
+      </c>
+      <c r="AG131" s="1">
+        <v>86.4</v>
+      </c>
       <c r="AH131" s="1"/>
       <c r="AI131" s="1"/>
       <c r="AJ131" s="1"/>
@@ -19038,6 +18212,15 @@
         <f t="shared" si="19"/>
         <v>6.8958168854050443E-4</v>
       </c>
+      <c r="AE132" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="AF132" s="13">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="AG132" s="15">
+        <v>8.6400000000000006E-8</v>
+      </c>
       <c r="BN132" s="4" t="s">
         <v>94</v>
       </c>
@@ -19125,6 +18308,15 @@
         <f t="shared" si="19"/>
         <v>7.0175093423377206E-4</v>
       </c>
+      <c r="AE133" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="AF133" s="1">
+        <v>86.4</v>
+      </c>
+      <c r="AG133" s="1">
+        <v>86.4</v>
+      </c>
       <c r="BN133" s="4" t="s">
         <v>94</v>
       </c>
@@ -19212,6 +18404,15 @@
         <f t="shared" si="19"/>
         <v>9.24392529713391E-4</v>
       </c>
+      <c r="AE134" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="AF134" s="13">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="AG134" s="15">
+        <v>8.6400000000000006E-8</v>
+      </c>
       <c r="BN134" s="4" t="s">
         <v>94</v>
       </c>
@@ -19299,6 +18500,15 @@
         <f t="shared" si="19"/>
         <v>4.2679489394130968E-4</v>
       </c>
+      <c r="AE135" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="AF135" s="1">
+        <v>86.4</v>
+      </c>
+      <c r="AG135" s="1">
+        <v>86.4</v>
+      </c>
       <c r="BN135" s="4" t="s">
         <v>95</v>
       </c>
@@ -19386,6 +18596,15 @@
         <f t="shared" si="19"/>
         <v>7.0492044974188462E-4</v>
       </c>
+      <c r="AE136" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="AF136" s="1">
+        <v>86.4</v>
+      </c>
+      <c r="AG136" s="1">
+        <v>86.4</v>
+      </c>
       <c r="BN136" s="4" t="s">
         <v>95</v>
       </c>
@@ -19473,6 +18692,15 @@
         <f t="shared" si="19"/>
         <v>6.0317831663807579E-4</v>
       </c>
+      <c r="AE137" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="AF137" s="13">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="AG137" s="15">
+        <v>8.6400000000000006E-8</v>
+      </c>
       <c r="BN137" s="4" t="s">
         <v>95</v>
       </c>
@@ -19560,6 +18788,15 @@
         <f t="shared" si="19"/>
         <v>5.3431529879549361E-4</v>
       </c>
+      <c r="AE138" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="AF138" s="1">
+        <v>86.4</v>
+      </c>
+      <c r="AG138" s="1">
+        <v>86.4</v>
+      </c>
       <c r="BN138" s="4" t="s">
         <v>96</v>
       </c>
@@ -19647,6 +18884,15 @@
         <f t="shared" si="19"/>
         <v>9.2650687165257131E-4</v>
       </c>
+      <c r="AE139" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="AF139" s="13">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="AG139" s="15">
+        <v>8.6400000000000006E-8</v>
+      </c>
       <c r="BN139" s="4" t="s">
         <v>96</v>
       </c>
@@ -19734,6 +18980,15 @@
         <f t="shared" si="19"/>
         <v>4.9093461376614072E-4</v>
       </c>
+      <c r="AE140" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="AF140" s="1">
+        <v>86.4</v>
+      </c>
+      <c r="AG140" s="1">
+        <v>86.4</v>
+      </c>
       <c r="BN140" s="4" t="s">
         <v>96</v>
       </c>
@@ -20083,7 +19338,7 @@
         <v>6.785411243790979E-4</v>
       </c>
     </row>
-    <row r="145" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="145" spans="1:76" x14ac:dyDescent="0.45">
       <c r="A145" t="s">
         <v>264</v>
       </c>
@@ -20137,7 +19392,7 @@
         <v>7.2348983877483703E-4</v>
       </c>
     </row>
-    <row r="146" spans="1:27" x14ac:dyDescent="0.45">
+    <row r="146" spans="1:76" x14ac:dyDescent="0.45">
       <c r="A146" t="s">
         <v>265</v>
       </c>
@@ -20190,8 +19445,11 @@
         <f t="shared" si="19"/>
         <v>6.5532909863160892E-4</v>
       </c>
-    </row>
-    <row r="147" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="BN146" t="s">
+        <v>1189</v>
+      </c>
+    </row>
+    <row r="147" spans="1:76" x14ac:dyDescent="0.45">
       <c r="A147" t="s">
         <v>266</v>
       </c>
@@ -20244,8 +19502,35 @@
         <f t="shared" si="19"/>
         <v>7.5474341979737567E-4</v>
       </c>
-    </row>
-    <row r="148" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="BN147" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="BO147" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="BP147" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="BQ147" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="BR147" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="BS147" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="BT147" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="BU147" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="BV147" s="4"/>
+      <c r="BW147" s="4"/>
+      <c r="BX147" s="4"/>
+    </row>
+    <row r="148" spans="1:76" x14ac:dyDescent="0.45">
       <c r="A148" t="s">
         <v>267</v>
       </c>
@@ -20298,8 +19583,32 @@
         <f t="shared" si="19"/>
         <v>5.7669688744116539E-4</v>
       </c>
-    </row>
-    <row r="149" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="BN148" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="BO148" s="4">
+        <v>0</v>
+      </c>
+      <c r="BP148" s="4">
+        <v>0</v>
+      </c>
+      <c r="BQ148" s="4">
+        <v>0</v>
+      </c>
+      <c r="BR148" s="4">
+        <v>0</v>
+      </c>
+      <c r="BS148" s="4">
+        <v>0</v>
+      </c>
+      <c r="BT148" s="4">
+        <v>0</v>
+      </c>
+      <c r="BU148" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="149" spans="1:76" x14ac:dyDescent="0.45">
       <c r="A149" t="s">
         <v>268</v>
       </c>
@@ -20352,8 +19661,32 @@
         <f t="shared" si="19"/>
         <v>8.0697176066542612E-4</v>
       </c>
-    </row>
-    <row r="150" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="BN149" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="BO149" s="3">
+        <v>3600000</v>
+      </c>
+      <c r="BP149" s="4">
+        <v>0</v>
+      </c>
+      <c r="BQ149" s="4">
+        <v>-1000</v>
+      </c>
+      <c r="BR149" s="4">
+        <v>-10000</v>
+      </c>
+      <c r="BS149" s="4">
+        <v>-100000</v>
+      </c>
+      <c r="BT149" s="4">
+        <v>-200000</v>
+      </c>
+      <c r="BU149" s="4">
+        <v>-600000</v>
+      </c>
+    </row>
+    <row r="150" spans="1:76" x14ac:dyDescent="0.45">
       <c r="A150" t="s">
         <v>269</v>
       </c>
@@ -20406,8 +19739,32 @@
         <f t="shared" si="19"/>
         <v>6.0999509381094925E-4</v>
       </c>
-    </row>
-    <row r="151" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="BN150" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="BO150" s="3">
+        <v>800000000</v>
+      </c>
+      <c r="BP150" s="4">
+        <v>0</v>
+      </c>
+      <c r="BQ150" s="4">
+        <v>-1000</v>
+      </c>
+      <c r="BR150" s="4">
+        <v>-10000</v>
+      </c>
+      <c r="BS150" s="4">
+        <v>-100000</v>
+      </c>
+      <c r="BT150" s="4">
+        <v>-200000</v>
+      </c>
+      <c r="BU150" s="4">
+        <v>-600000</v>
+      </c>
+    </row>
+    <row r="151" spans="1:76" x14ac:dyDescent="0.45">
       <c r="A151" t="s">
         <v>270</v>
       </c>
@@ -20460,8 +19817,32 @@
         <f t="shared" si="19"/>
         <v>5.3117803129513444E-4</v>
       </c>
-    </row>
-    <row r="152" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="BN151" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="BO151" s="4">
+        <v>0</v>
+      </c>
+      <c r="BP151" s="4">
+        <v>0</v>
+      </c>
+      <c r="BQ151" s="4">
+        <v>0</v>
+      </c>
+      <c r="BR151" s="4">
+        <v>0</v>
+      </c>
+      <c r="BS151" s="4">
+        <v>0</v>
+      </c>
+      <c r="BT151" s="4">
+        <v>0</v>
+      </c>
+      <c r="BU151" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="152" spans="1:76" x14ac:dyDescent="0.45">
       <c r="A152" t="s">
         <v>271</v>
       </c>
@@ -20514,8 +19895,32 @@
         <f t="shared" si="19"/>
         <v>6.8402085428227407E-4</v>
       </c>
-    </row>
-    <row r="153" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="BN152" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="BO152" s="3">
+        <v>3600000</v>
+      </c>
+      <c r="BP152" s="4">
+        <v>0</v>
+      </c>
+      <c r="BQ152" s="4">
+        <v>-1000</v>
+      </c>
+      <c r="BR152" s="4">
+        <v>-10000</v>
+      </c>
+      <c r="BS152" s="4">
+        <v>-100000</v>
+      </c>
+      <c r="BT152" s="4">
+        <v>-200000</v>
+      </c>
+      <c r="BU152" s="4">
+        <v>-600000</v>
+      </c>
+    </row>
+    <row r="153" spans="1:76" x14ac:dyDescent="0.45">
       <c r="A153" t="s">
         <v>272</v>
       </c>
@@ -20568,8 +19973,32 @@
         <f t="shared" si="19"/>
         <v>5.6115552392589597E-4</v>
       </c>
-    </row>
-    <row r="154" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="BN153" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="BO153" s="3">
+        <v>800000000</v>
+      </c>
+      <c r="BP153" s="4">
+        <v>0</v>
+      </c>
+      <c r="BQ153" s="4">
+        <v>-1000</v>
+      </c>
+      <c r="BR153" s="4">
+        <v>-10000</v>
+      </c>
+      <c r="BS153" s="4">
+        <v>-100000</v>
+      </c>
+      <c r="BT153" s="4">
+        <v>-200000</v>
+      </c>
+      <c r="BU153" s="4">
+        <v>-600000</v>
+      </c>
+    </row>
+    <row r="154" spans="1:76" x14ac:dyDescent="0.45">
       <c r="A154" t="s">
         <v>273</v>
       </c>
@@ -20622,8 +20051,32 @@
         <f t="shared" si="19"/>
         <v>5.6175108458420442E-4</v>
       </c>
-    </row>
-    <row r="155" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="BN154" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="BO154" s="4">
+        <v>0</v>
+      </c>
+      <c r="BP154" s="4">
+        <v>0</v>
+      </c>
+      <c r="BQ154" s="4">
+        <v>0</v>
+      </c>
+      <c r="BR154" s="4">
+        <v>0</v>
+      </c>
+      <c r="BS154" s="4">
+        <v>0</v>
+      </c>
+      <c r="BT154" s="4">
+        <v>0</v>
+      </c>
+      <c r="BU154" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="155" spans="1:76" x14ac:dyDescent="0.45">
       <c r="A155" t="s">
         <v>274</v>
       </c>
@@ -20651,8 +20104,32 @@
       <c r="I155">
         <v>36000</v>
       </c>
-    </row>
-    <row r="156" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="BN155" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="BO155" s="3">
+        <v>3600000</v>
+      </c>
+      <c r="BP155" s="4">
+        <v>0</v>
+      </c>
+      <c r="BQ155" s="4">
+        <v>-1000</v>
+      </c>
+      <c r="BR155" s="4">
+        <v>-10000</v>
+      </c>
+      <c r="BS155" s="4">
+        <v>-100000</v>
+      </c>
+      <c r="BT155" s="4">
+        <v>-200000</v>
+      </c>
+      <c r="BU155" s="4">
+        <v>-600000</v>
+      </c>
+    </row>
+    <row r="156" spans="1:76" x14ac:dyDescent="0.45">
       <c r="A156" t="s">
         <v>275</v>
       </c>
@@ -20680,8 +20157,32 @@
       <c r="I156">
         <v>36000</v>
       </c>
-    </row>
-    <row r="157" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="BN156" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="BO156" s="3">
+        <v>800000000</v>
+      </c>
+      <c r="BP156" s="4">
+        <v>0</v>
+      </c>
+      <c r="BQ156" s="4">
+        <v>-1000</v>
+      </c>
+      <c r="BR156" s="4">
+        <v>-10000</v>
+      </c>
+      <c r="BS156" s="4">
+        <v>-100000</v>
+      </c>
+      <c r="BT156" s="4">
+        <v>-200000</v>
+      </c>
+      <c r="BU156" s="4">
+        <v>-600000</v>
+      </c>
+    </row>
+    <row r="157" spans="1:76" x14ac:dyDescent="0.45">
       <c r="A157" t="s">
         <v>276</v>
       </c>
@@ -20709,8 +20210,32 @@
       <c r="I157">
         <v>36000</v>
       </c>
-    </row>
-    <row r="158" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="BN157" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="BO157" s="4">
+        <v>0</v>
+      </c>
+      <c r="BP157" s="4">
+        <v>0</v>
+      </c>
+      <c r="BQ157" s="4">
+        <v>0</v>
+      </c>
+      <c r="BR157" s="4">
+        <v>0</v>
+      </c>
+      <c r="BS157" s="4">
+        <v>0</v>
+      </c>
+      <c r="BT157" s="4">
+        <v>0</v>
+      </c>
+      <c r="BU157" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="158" spans="1:76" x14ac:dyDescent="0.45">
       <c r="A158" t="s">
         <v>277</v>
       </c>
@@ -20738,8 +20263,32 @@
       <c r="I158">
         <v>36000</v>
       </c>
-    </row>
-    <row r="159" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="BN158" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="BO158" s="3">
+        <v>3600000</v>
+      </c>
+      <c r="BP158" s="4">
+        <v>0</v>
+      </c>
+      <c r="BQ158" s="4">
+        <v>-1000</v>
+      </c>
+      <c r="BR158" s="4">
+        <v>-10000</v>
+      </c>
+      <c r="BS158" s="4">
+        <v>-100000</v>
+      </c>
+      <c r="BT158" s="4">
+        <v>-200000</v>
+      </c>
+      <c r="BU158" s="4">
+        <v>-600000</v>
+      </c>
+    </row>
+    <row r="159" spans="1:76" x14ac:dyDescent="0.45">
       <c r="A159" t="s">
         <v>278</v>
       </c>
@@ -20767,8 +20316,32 @@
       <c r="I159">
         <v>36000</v>
       </c>
-    </row>
-    <row r="160" spans="1:27" x14ac:dyDescent="0.45">
+      <c r="BN159" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="BO159" s="3">
+        <v>800000000</v>
+      </c>
+      <c r="BP159" s="4">
+        <v>0</v>
+      </c>
+      <c r="BQ159" s="4">
+        <v>-1000</v>
+      </c>
+      <c r="BR159" s="4">
+        <v>-10000</v>
+      </c>
+      <c r="BS159" s="4">
+        <v>-100000</v>
+      </c>
+      <c r="BT159" s="4">
+        <v>-200000</v>
+      </c>
+      <c r="BU159" s="4">
+        <v>-600000</v>
+      </c>
+    </row>
+    <row r="160" spans="1:76" x14ac:dyDescent="0.45">
       <c r="A160" t="s">
         <v>279</v>
       </c>
@@ -20796,8 +20369,32 @@
       <c r="I160">
         <v>36000</v>
       </c>
-    </row>
-    <row r="161" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="BN160" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="BO160" s="4">
+        <v>0</v>
+      </c>
+      <c r="BP160" s="4">
+        <v>0</v>
+      </c>
+      <c r="BQ160" s="4">
+        <v>0</v>
+      </c>
+      <c r="BR160" s="4">
+        <v>0</v>
+      </c>
+      <c r="BS160" s="4">
+        <v>0</v>
+      </c>
+      <c r="BT160" s="4">
+        <v>0</v>
+      </c>
+      <c r="BU160" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="161" spans="1:73" x14ac:dyDescent="0.45">
       <c r="A161" t="s">
         <v>280</v>
       </c>
@@ -20825,8 +20422,32 @@
       <c r="I161">
         <v>36000</v>
       </c>
-    </row>
-    <row r="162" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="BN161" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="BO161" s="3">
+        <v>3600000</v>
+      </c>
+      <c r="BP161" s="4">
+        <v>0</v>
+      </c>
+      <c r="BQ161" s="4">
+        <v>-1000</v>
+      </c>
+      <c r="BR161" s="4">
+        <v>-10000</v>
+      </c>
+      <c r="BS161" s="4">
+        <v>-100000</v>
+      </c>
+      <c r="BT161" s="4">
+        <v>-200000</v>
+      </c>
+      <c r="BU161" s="4">
+        <v>-600000</v>
+      </c>
+    </row>
+    <row r="162" spans="1:73" x14ac:dyDescent="0.45">
       <c r="A162" t="s">
         <v>281</v>
       </c>
@@ -20854,8 +20475,32 @@
       <c r="I162">
         <v>36000</v>
       </c>
-    </row>
-    <row r="163" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="BN162" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="BO162" s="3">
+        <v>800000000</v>
+      </c>
+      <c r="BP162" s="4">
+        <v>0</v>
+      </c>
+      <c r="BQ162" s="4">
+        <v>-1000</v>
+      </c>
+      <c r="BR162" s="4">
+        <v>-10000</v>
+      </c>
+      <c r="BS162" s="4">
+        <v>-100000</v>
+      </c>
+      <c r="BT162" s="4">
+        <v>-200000</v>
+      </c>
+      <c r="BU162" s="4">
+        <v>-600000</v>
+      </c>
+    </row>
+    <row r="163" spans="1:73" x14ac:dyDescent="0.45">
       <c r="A163" t="s">
         <v>282</v>
       </c>
@@ -20884,7 +20529,7 @@
         <v>36000</v>
       </c>
     </row>
-    <row r="164" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="164" spans="1:73" x14ac:dyDescent="0.45">
       <c r="A164" t="s">
         <v>283</v>
       </c>
@@ -20913,7 +20558,7 @@
         <v>36000</v>
       </c>
     </row>
-    <row r="165" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="165" spans="1:73" x14ac:dyDescent="0.45">
       <c r="A165" t="s">
         <v>284</v>
       </c>
@@ -20942,7 +20587,7 @@
         <v>36000</v>
       </c>
     </row>
-    <row r="166" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="166" spans="1:73" x14ac:dyDescent="0.45">
       <c r="A166" t="s">
         <v>285</v>
       </c>
@@ -20971,7 +20616,7 @@
         <v>36000</v>
       </c>
     </row>
-    <row r="167" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="167" spans="1:73" x14ac:dyDescent="0.45">
       <c r="A167" t="s">
         <v>286</v>
       </c>
@@ -21000,7 +20645,7 @@
         <v>36000</v>
       </c>
     </row>
-    <row r="168" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="168" spans="1:73" x14ac:dyDescent="0.45">
       <c r="A168" t="s">
         <v>287</v>
       </c>
@@ -21029,7 +20674,7 @@
         <v>36000</v>
       </c>
     </row>
-    <row r="169" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="169" spans="1:73" x14ac:dyDescent="0.45">
       <c r="A169" t="s">
         <v>288</v>
       </c>
@@ -21058,7 +20703,7 @@
         <v>36000</v>
       </c>
     </row>
-    <row r="170" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="170" spans="1:73" x14ac:dyDescent="0.45">
       <c r="A170" t="s">
         <v>289</v>
       </c>
@@ -21087,7 +20732,7 @@
         <v>36000</v>
       </c>
     </row>
-    <row r="171" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="171" spans="1:73" x14ac:dyDescent="0.45">
       <c r="A171" t="s">
         <v>290</v>
       </c>
@@ -21116,7 +20761,7 @@
         <v>36000</v>
       </c>
     </row>
-    <row r="172" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="172" spans="1:73" x14ac:dyDescent="0.45">
       <c r="A172" t="s">
         <v>291</v>
       </c>
@@ -21145,7 +20790,7 @@
         <v>36000</v>
       </c>
     </row>
-    <row r="173" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="173" spans="1:73" x14ac:dyDescent="0.45">
       <c r="A173" t="s">
         <v>292</v>
       </c>
@@ -21174,7 +20819,7 @@
         <v>36000</v>
       </c>
     </row>
-    <row r="174" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="174" spans="1:73" x14ac:dyDescent="0.45">
       <c r="A174" t="s">
         <v>293</v>
       </c>
@@ -21203,7 +20848,7 @@
         <v>36000</v>
       </c>
     </row>
-    <row r="175" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="175" spans="1:73" x14ac:dyDescent="0.45">
       <c r="A175" t="s">
         <v>294</v>
       </c>
@@ -21232,7 +20877,7 @@
         <v>36000</v>
       </c>
     </row>
-    <row r="176" spans="1:9" x14ac:dyDescent="0.45">
+    <row r="176" spans="1:73" x14ac:dyDescent="0.45">
       <c r="A176" t="s">
         <v>295</v>
       </c>
@@ -28654,8 +28299,8 @@
       <c r="A22" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="B22">
-        <v>5.5555555555555599E-4</v>
+      <c r="B22" s="1">
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="C22">
         <v>3.1154231364886891E-4</v>
@@ -28680,8 +28325,8 @@
       <c r="A23" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="B23">
-        <v>5.5555555555555599E-4</v>
+      <c r="B23" s="1">
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="C23">
         <v>3.1154231364886891E-5</v>
@@ -28706,8 +28351,8 @@
       <c r="A24" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="B24">
-        <v>5.5555555555555599E-4</v>
+      <c r="B24" s="1">
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="C24">
         <v>3.1154231364886891E-4</v>
@@ -28732,8 +28377,8 @@
       <c r="A25" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="B25">
-        <v>5.5555555555555599E-4</v>
+      <c r="B25" s="1">
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="C25">
         <v>3.1154231364886891E-5</v>
@@ -28758,8 +28403,8 @@
       <c r="A26" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="B26">
-        <v>5.5555555555555599E-4</v>
+      <c r="B26" s="1">
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="C26">
         <v>3.1154231364886891E-4</v>
@@ -28945,19 +28590,19 @@
         <v>0</v>
       </c>
       <c r="B2" s="1">
-        <v>5.5555555555555599E-4</v>
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="C2" s="1">
-        <v>5.5555555555555599E-4</v>
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="D2" s="1">
-        <v>5.5555555555555599E-4</v>
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="E2" s="1">
-        <v>5.5555555555555599E-4</v>
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="F2" s="1">
-        <v>5.5555555555555599E-4</v>
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="G2" s="1"/>
       <c r="I2" s="1"/>
@@ -28970,19 +28615,19 @@
         <v>3600000</v>
       </c>
       <c r="B3" s="1">
-        <v>5.5555555555555599E-4</v>
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="C3" s="1">
-        <v>5.5555555555555599E-4</v>
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="D3" s="1">
-        <v>5.5555555555555599E-4</v>
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="E3" s="1">
-        <v>5.5555555555555599E-4</v>
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="F3" s="1">
-        <v>5.5555555555555599E-4</v>
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="G3" s="1"/>
       <c r="I3" s="1"/>
@@ -28995,19 +28640,19 @@
         <v>800000000</v>
       </c>
       <c r="B4" s="1">
-        <v>5.5555555555555599E-4</v>
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="C4" s="1">
-        <v>5.5555555555555599E-4</v>
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="D4" s="1">
-        <v>5.5555555555555599E-4</v>
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="E4" s="1">
-        <v>5.5555555555555599E-4</v>
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="F4" s="1">
-        <v>5.5555555555555599E-4</v>
+        <v>5.5555555555555556E-4</v>
       </c>
       <c r="G4" s="1"/>
     </row>
@@ -45418,13 +45063,13 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="12.265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A1" s="5" t="s">
         <v>91</v>
       </c>
@@ -45444,7 +45089,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>93</v>
       </c>
@@ -45463,8 +45108,9 @@
       <c r="F2" s="4">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="G2" s="4"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>93</v>
       </c>
@@ -45483,8 +45129,9 @@
       <c r="F3" s="4">
         <v>-50</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="G3" s="4"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>93</v>
       </c>
@@ -45503,8 +45150,9 @@
       <c r="F4" s="4">
         <v>-50</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="G4" s="4"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>94</v>
       </c>
@@ -45523,8 +45171,9 @@
       <c r="F5" s="4">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="G5" s="4"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>94</v>
       </c>
@@ -45543,8 +45192,9 @@
       <c r="F6" s="4">
         <v>-50</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="G6" s="4"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>94</v>
       </c>
@@ -45563,8 +45213,9 @@
       <c r="F7" s="4">
         <v>-50</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="G7" s="4"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>95</v>
       </c>
@@ -45583,8 +45234,9 @@
       <c r="F8" s="4">
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="G8" s="4"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>95</v>
       </c>
@@ -45603,8 +45255,9 @@
       <c r="F9" s="4">
         <v>-50</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="G9" s="4"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>95</v>
       </c>
@@ -45623,8 +45276,9 @@
       <c r="F10" s="4">
         <v>-50</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="G10" s="4"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>96</v>
       </c>
@@ -45643,8 +45297,9 @@
       <c r="F11" s="4">
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="G11" s="4"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>96</v>
       </c>
@@ -45663,8 +45318,9 @@
       <c r="F12" s="4">
         <v>-50</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="G12" s="4"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>96</v>
       </c>
@@ -45683,8 +45339,9 @@
       <c r="F13" s="4">
         <v>-50</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="G13" s="4"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>97</v>
       </c>
@@ -45703,8 +45360,9 @@
       <c r="F14" s="4">
         <v>0</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="G14" s="4"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>97</v>
       </c>
@@ -45723,8 +45381,9 @@
       <c r="F15" s="4">
         <v>-50</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="G15" s="4"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>97</v>
       </c>
@@ -45743,6 +45402,19 @@
       <c r="F16" s="4">
         <v>-50</v>
       </c>
+      <c r="G16" s="4"/>
+    </row>
+    <row r="17" spans="7:7" x14ac:dyDescent="0.45">
+      <c r="G17" s="4"/>
+    </row>
+    <row r="18" spans="7:7" x14ac:dyDescent="0.45">
+      <c r="G18" s="4"/>
+    </row>
+    <row r="19" spans="7:7" x14ac:dyDescent="0.45">
+      <c r="G19" s="4"/>
+    </row>
+    <row r="20" spans="7:7" x14ac:dyDescent="0.45">
+      <c r="G20" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fixed storage formulation of unconfined areas. Increased number of iterations for run 03
</commit_message>
<xml_diff>
--- a/assets/3D/sust yield server/setup.xlsx
+++ b/assets/3D/sust yield server/setup.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmarinriver\Projects\ConfinedLab\assets\3D\sust yield server\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E185B573-6830-4F13-B1E0-778BA6A8D7C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{193EF687-4CBE-4DEC-B582-9A5B7AE67EE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" firstSheet="1" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="grid" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Little fixes for Sustainable Yield 3D model runs
</commit_message>
<xml_diff>
--- a/assets/3D/sust yield server/setup.xlsx
+++ b/assets/3D/sust yield server/setup.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmarinriver\Projects\ConfinedLab\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmarinriver\Projects\ConfinedLab\assets\3D\sust yield server\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{981DAE2D-6E47-4B5B-BB95-F8F040630306}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3179C0F9-D5FF-4DC2-8E52-431C9321CA93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="grid" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2465" uniqueCount="1192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2504" uniqueCount="1192">
   <si>
     <t>nlay</t>
   </si>
@@ -3740,7 +3740,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -3767,6 +3767,9 @@
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="11" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -4386,420 +4389,660 @@
     <col min="10" max="10" width="10.9296875" style="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A1" t="s">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A1" s="12" t="s">
         <v>884</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="12" t="s">
         <v>919</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="12" t="s">
         <v>909</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="12" t="s">
         <v>910</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="12" t="s">
         <v>911</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="12" t="s">
         <v>912</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="12" t="s">
         <v>913</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
+      <c r="I1" s="12" t="s">
+        <v>914</v>
+      </c>
+      <c r="J1" s="12" t="s">
+        <v>915</v>
+      </c>
+      <c r="K1" s="12" t="s">
+        <v>916</v>
+      </c>
+      <c r="L1" s="12" t="s">
+        <v>917</v>
+      </c>
+      <c r="M1" s="12" t="s">
+        <v>918</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A2" s="12" t="s">
         <v>886</v>
       </c>
-      <c r="B2">
-        <v>0</v>
-      </c>
-      <c r="C2">
-        <v>0</v>
-      </c>
-      <c r="D2">
-        <v>0</v>
-      </c>
-      <c r="E2">
-        <v>0</v>
-      </c>
-      <c r="F2">
-        <v>0</v>
-      </c>
-      <c r="G2">
-        <v>0</v>
-      </c>
-      <c r="H2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
+      <c r="B2" s="12">
+        <v>0</v>
+      </c>
+      <c r="C2" s="12">
+        <v>0</v>
+      </c>
+      <c r="D2" s="12">
+        <v>0</v>
+      </c>
+      <c r="E2" s="12">
+        <v>0</v>
+      </c>
+      <c r="F2" s="12">
+        <v>0</v>
+      </c>
+      <c r="G2" s="12">
+        <v>0</v>
+      </c>
+      <c r="H2" s="12">
+        <v>0</v>
+      </c>
+      <c r="I2" s="12">
+        <v>0</v>
+      </c>
+      <c r="J2" s="12">
+        <v>0</v>
+      </c>
+      <c r="K2" s="12">
+        <v>0</v>
+      </c>
+      <c r="L2" s="12">
+        <v>0</v>
+      </c>
+      <c r="M2" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A3" s="12" t="s">
         <v>886</v>
       </c>
       <c r="B3" s="2">
         <v>3600000</v>
       </c>
-      <c r="C3">
-        <v>0</v>
-      </c>
-      <c r="D3">
+      <c r="C3" s="12">
+        <v>0</v>
+      </c>
+      <c r="D3" s="12">
+        <v>-100</v>
+      </c>
+      <c r="E3" s="12">
+        <v>-200</v>
+      </c>
+      <c r="F3" s="12">
         <v>-1000</v>
       </c>
-      <c r="E3">
-        <v>-10000</v>
-      </c>
-      <c r="F3">
+      <c r="G3" s="12">
+        <v>-2000</v>
+      </c>
+      <c r="H3" s="12">
+        <v>-20000</v>
+      </c>
+      <c r="I3" s="12">
         <v>-100000</v>
       </c>
-      <c r="G3">
+      <c r="J3" s="12">
         <v>-200000</v>
       </c>
-      <c r="H3">
+      <c r="K3" s="12">
         <v>-600000</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
+      <c r="L3" s="12">
+        <v>-1200000</v>
+      </c>
+      <c r="M3" s="12">
+        <v>-2400000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A4" s="12" t="s">
         <v>886</v>
       </c>
       <c r="B4" s="2">
         <v>800000000</v>
       </c>
-      <c r="C4">
-        <v>0</v>
-      </c>
-      <c r="D4">
+      <c r="C4" s="12">
+        <v>0</v>
+      </c>
+      <c r="D4" s="12">
+        <v>-100</v>
+      </c>
+      <c r="E4" s="12">
+        <v>-200</v>
+      </c>
+      <c r="F4" s="12">
         <v>-1000</v>
       </c>
-      <c r="E4">
-        <v>-10000</v>
-      </c>
-      <c r="F4">
+      <c r="G4" s="12">
+        <v>-2000</v>
+      </c>
+      <c r="H4" s="12">
+        <v>-20000</v>
+      </c>
+      <c r="I4" s="12">
         <v>-100000</v>
       </c>
-      <c r="G4">
+      <c r="J4" s="12">
         <v>-200000</v>
       </c>
-      <c r="H4">
+      <c r="K4" s="12">
         <v>-600000</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A5" t="s">
+      <c r="L4" s="12">
+        <v>-1200000</v>
+      </c>
+      <c r="M4" s="12">
+        <v>-2400000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A5" s="12" t="s">
         <v>887</v>
       </c>
-      <c r="B5">
-        <v>0</v>
-      </c>
-      <c r="C5">
-        <v>0</v>
-      </c>
-      <c r="D5">
-        <v>0</v>
-      </c>
-      <c r="E5">
-        <v>0</v>
-      </c>
-      <c r="F5">
-        <v>0</v>
-      </c>
-      <c r="G5">
-        <v>0</v>
-      </c>
-      <c r="H5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A6" t="s">
+      <c r="B5" s="12">
+        <v>0</v>
+      </c>
+      <c r="C5" s="12">
+        <v>0</v>
+      </c>
+      <c r="D5" s="12">
+        <v>0</v>
+      </c>
+      <c r="E5" s="12">
+        <v>0</v>
+      </c>
+      <c r="F5" s="12">
+        <v>0</v>
+      </c>
+      <c r="G5" s="12">
+        <v>0</v>
+      </c>
+      <c r="H5" s="12">
+        <v>0</v>
+      </c>
+      <c r="I5" s="12">
+        <v>0</v>
+      </c>
+      <c r="J5" s="12">
+        <v>0</v>
+      </c>
+      <c r="K5" s="12">
+        <v>0</v>
+      </c>
+      <c r="L5" s="12">
+        <v>0</v>
+      </c>
+      <c r="M5" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A6" s="12" t="s">
         <v>887</v>
       </c>
       <c r="B6" s="2">
         <v>3600000</v>
       </c>
-      <c r="C6">
-        <v>0</v>
-      </c>
-      <c r="D6">
+      <c r="C6" s="12">
+        <v>0</v>
+      </c>
+      <c r="D6" s="12">
+        <v>-100</v>
+      </c>
+      <c r="E6" s="12">
+        <v>-200</v>
+      </c>
+      <c r="F6" s="12">
         <v>-1000</v>
       </c>
-      <c r="E6">
-        <v>-10000</v>
-      </c>
-      <c r="F6">
+      <c r="G6" s="12">
+        <v>-2000</v>
+      </c>
+      <c r="H6" s="12">
+        <v>-20000</v>
+      </c>
+      <c r="I6" s="12">
         <v>-100000</v>
       </c>
-      <c r="G6">
+      <c r="J6" s="12">
         <v>-200000</v>
       </c>
-      <c r="H6">
+      <c r="K6" s="12">
         <v>-600000</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A7" t="s">
+      <c r="L6" s="12">
+        <v>-1200000</v>
+      </c>
+      <c r="M6" s="12">
+        <v>-2400000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A7" s="12" t="s">
         <v>887</v>
       </c>
       <c r="B7" s="2">
         <v>800000000</v>
       </c>
-      <c r="C7">
-        <v>0</v>
-      </c>
-      <c r="D7">
+      <c r="C7" s="12">
+        <v>0</v>
+      </c>
+      <c r="D7" s="12">
+        <v>-100</v>
+      </c>
+      <c r="E7" s="12">
+        <v>-200</v>
+      </c>
+      <c r="F7" s="12">
         <v>-1000</v>
       </c>
-      <c r="E7">
-        <v>-10000</v>
-      </c>
-      <c r="F7">
+      <c r="G7" s="12">
+        <v>-2000</v>
+      </c>
+      <c r="H7" s="12">
+        <v>-20000</v>
+      </c>
+      <c r="I7" s="12">
         <v>-100000</v>
       </c>
-      <c r="G7">
+      <c r="J7" s="12">
         <v>-200000</v>
       </c>
-      <c r="H7">
+      <c r="K7" s="12">
         <v>-600000</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A8" t="s">
+      <c r="L7" s="12">
+        <v>-1200000</v>
+      </c>
+      <c r="M7" s="12">
+        <v>-2400000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A8" s="12" t="s">
         <v>888</v>
       </c>
-      <c r="B8">
-        <v>0</v>
-      </c>
-      <c r="C8">
-        <v>0</v>
-      </c>
-      <c r="D8">
-        <v>0</v>
-      </c>
-      <c r="E8">
-        <v>0</v>
-      </c>
-      <c r="F8">
-        <v>0</v>
-      </c>
-      <c r="G8">
-        <v>0</v>
-      </c>
-      <c r="H8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A9" t="s">
+      <c r="B8" s="12">
+        <v>0</v>
+      </c>
+      <c r="C8" s="12">
+        <v>0</v>
+      </c>
+      <c r="D8" s="12">
+        <v>0</v>
+      </c>
+      <c r="E8" s="12">
+        <v>0</v>
+      </c>
+      <c r="F8" s="12">
+        <v>0</v>
+      </c>
+      <c r="G8" s="12">
+        <v>0</v>
+      </c>
+      <c r="H8" s="12">
+        <v>0</v>
+      </c>
+      <c r="I8" s="12">
+        <v>0</v>
+      </c>
+      <c r="J8" s="12">
+        <v>0</v>
+      </c>
+      <c r="K8" s="12">
+        <v>0</v>
+      </c>
+      <c r="L8" s="12">
+        <v>0</v>
+      </c>
+      <c r="M8" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A9" s="12" t="s">
         <v>888</v>
       </c>
       <c r="B9" s="2">
         <v>3600000</v>
       </c>
-      <c r="C9">
-        <v>0</v>
-      </c>
-      <c r="D9">
+      <c r="C9" s="12">
+        <v>0</v>
+      </c>
+      <c r="D9" s="12">
+        <v>-100</v>
+      </c>
+      <c r="E9" s="12">
+        <v>-200</v>
+      </c>
+      <c r="F9" s="12">
         <v>-1000</v>
       </c>
-      <c r="E9">
-        <v>-10000</v>
-      </c>
-      <c r="F9">
+      <c r="G9" s="12">
+        <v>-2000</v>
+      </c>
+      <c r="H9" s="12">
+        <v>-20000</v>
+      </c>
+      <c r="I9" s="12">
         <v>-100000</v>
       </c>
-      <c r="G9">
+      <c r="J9" s="12">
         <v>-200000</v>
       </c>
-      <c r="H9">
+      <c r="K9" s="12">
         <v>-600000</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A10" t="s">
+      <c r="L9" s="12">
+        <v>-1200000</v>
+      </c>
+      <c r="M9" s="12">
+        <v>-2400000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A10" s="12" t="s">
         <v>888</v>
       </c>
       <c r="B10" s="2">
         <v>800000000</v>
       </c>
-      <c r="C10">
-        <v>0</v>
-      </c>
-      <c r="D10">
+      <c r="C10" s="12">
+        <v>0</v>
+      </c>
+      <c r="D10" s="12">
+        <v>-100</v>
+      </c>
+      <c r="E10" s="12">
+        <v>-200</v>
+      </c>
+      <c r="F10" s="12">
         <v>-1000</v>
       </c>
-      <c r="E10">
-        <v>-10000</v>
-      </c>
-      <c r="F10">
+      <c r="G10" s="12">
+        <v>-2000</v>
+      </c>
+      <c r="H10" s="12">
+        <v>-20000</v>
+      </c>
+      <c r="I10" s="12">
         <v>-100000</v>
       </c>
-      <c r="G10">
+      <c r="J10" s="12">
         <v>-200000</v>
       </c>
-      <c r="H10">
+      <c r="K10" s="12">
         <v>-600000</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A11" t="s">
+      <c r="L10" s="12">
+        <v>-1200000</v>
+      </c>
+      <c r="M10" s="12">
+        <v>-2400000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A11" s="12" t="s">
         <v>889</v>
       </c>
-      <c r="B11">
-        <v>0</v>
-      </c>
-      <c r="C11">
-        <v>0</v>
-      </c>
-      <c r="D11">
-        <v>0</v>
-      </c>
-      <c r="E11">
-        <v>0</v>
-      </c>
-      <c r="F11">
-        <v>0</v>
-      </c>
-      <c r="G11">
-        <v>0</v>
-      </c>
-      <c r="H11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A12" t="s">
+      <c r="B11" s="12">
+        <v>0</v>
+      </c>
+      <c r="C11" s="12">
+        <v>0</v>
+      </c>
+      <c r="D11" s="12">
+        <v>0</v>
+      </c>
+      <c r="E11" s="12">
+        <v>0</v>
+      </c>
+      <c r="F11" s="12">
+        <v>0</v>
+      </c>
+      <c r="G11" s="12">
+        <v>0</v>
+      </c>
+      <c r="H11" s="12">
+        <v>0</v>
+      </c>
+      <c r="I11" s="12">
+        <v>0</v>
+      </c>
+      <c r="J11" s="12">
+        <v>0</v>
+      </c>
+      <c r="K11" s="12">
+        <v>0</v>
+      </c>
+      <c r="L11" s="12">
+        <v>0</v>
+      </c>
+      <c r="M11" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A12" s="12" t="s">
         <v>889</v>
       </c>
       <c r="B12" s="2">
         <v>3600000</v>
       </c>
-      <c r="C12">
-        <v>0</v>
-      </c>
-      <c r="D12">
+      <c r="C12" s="12">
+        <v>0</v>
+      </c>
+      <c r="D12" s="12">
+        <v>-100</v>
+      </c>
+      <c r="E12" s="12">
+        <v>-200</v>
+      </c>
+      <c r="F12" s="12">
         <v>-1000</v>
       </c>
-      <c r="E12">
-        <v>-10000</v>
-      </c>
-      <c r="F12">
+      <c r="G12" s="12">
+        <v>-2000</v>
+      </c>
+      <c r="H12" s="12">
+        <v>-20000</v>
+      </c>
+      <c r="I12" s="12">
         <v>-100000</v>
       </c>
-      <c r="G12">
+      <c r="J12" s="12">
         <v>-200000</v>
       </c>
-      <c r="H12">
+      <c r="K12" s="12">
         <v>-600000</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A13" t="s">
+      <c r="L12" s="12">
+        <v>-1200000</v>
+      </c>
+      <c r="M12" s="12">
+        <v>-2400000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A13" s="12" t="s">
         <v>889</v>
       </c>
       <c r="B13" s="2">
         <v>800000000</v>
       </c>
-      <c r="C13">
-        <v>0</v>
-      </c>
-      <c r="D13">
+      <c r="C13" s="12">
+        <v>0</v>
+      </c>
+      <c r="D13" s="12">
+        <v>-100</v>
+      </c>
+      <c r="E13" s="12">
+        <v>-200</v>
+      </c>
+      <c r="F13" s="12">
         <v>-1000</v>
       </c>
-      <c r="E13">
-        <v>-10000</v>
-      </c>
-      <c r="F13">
+      <c r="G13" s="12">
+        <v>-2000</v>
+      </c>
+      <c r="H13" s="12">
+        <v>-20000</v>
+      </c>
+      <c r="I13" s="12">
         <v>-100000</v>
       </c>
-      <c r="G13">
+      <c r="J13" s="12">
         <v>-200000</v>
       </c>
-      <c r="H13">
+      <c r="K13" s="12">
         <v>-600000</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A14" t="s">
+      <c r="L13" s="12">
+        <v>-1200000</v>
+      </c>
+      <c r="M13" s="12">
+        <v>-2400000</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A14" s="12" t="s">
         <v>890</v>
       </c>
-      <c r="B14">
-        <v>0</v>
-      </c>
-      <c r="C14">
-        <v>0</v>
-      </c>
-      <c r="D14">
-        <v>0</v>
-      </c>
-      <c r="E14">
-        <v>0</v>
-      </c>
-      <c r="F14">
-        <v>0</v>
-      </c>
-      <c r="G14">
-        <v>0</v>
-      </c>
-      <c r="H14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A15" t="s">
+      <c r="B14" s="12">
+        <v>0</v>
+      </c>
+      <c r="C14" s="12">
+        <v>0</v>
+      </c>
+      <c r="D14" s="12">
+        <v>0</v>
+      </c>
+      <c r="E14" s="12">
+        <v>0</v>
+      </c>
+      <c r="F14" s="12">
+        <v>0</v>
+      </c>
+      <c r="G14" s="12">
+        <v>0</v>
+      </c>
+      <c r="H14" s="12">
+        <v>0</v>
+      </c>
+      <c r="I14" s="12">
+        <v>0</v>
+      </c>
+      <c r="J14" s="12">
+        <v>0</v>
+      </c>
+      <c r="K14" s="12">
+        <v>0</v>
+      </c>
+      <c r="L14" s="12">
+        <v>0</v>
+      </c>
+      <c r="M14" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A15" s="12" t="s">
         <v>890</v>
       </c>
       <c r="B15" s="2">
         <v>3600000</v>
       </c>
-      <c r="C15">
-        <v>0</v>
-      </c>
-      <c r="D15">
+      <c r="C15" s="12">
+        <v>0</v>
+      </c>
+      <c r="D15" s="12">
+        <v>-100</v>
+      </c>
+      <c r="E15" s="12">
+        <v>-200</v>
+      </c>
+      <c r="F15" s="12">
         <v>-1000</v>
       </c>
-      <c r="E15">
-        <v>-10000</v>
-      </c>
-      <c r="F15">
+      <c r="G15" s="12">
+        <v>-2000</v>
+      </c>
+      <c r="H15" s="12">
+        <v>-20000</v>
+      </c>
+      <c r="I15" s="12">
         <v>-100000</v>
       </c>
-      <c r="G15">
+      <c r="J15" s="12">
         <v>-200000</v>
       </c>
-      <c r="H15">
+      <c r="K15" s="12">
         <v>-600000</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A16" t="s">
+      <c r="L15" s="12">
+        <v>-1200000</v>
+      </c>
+      <c r="M15" s="12">
+        <v>-2400000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A16" s="12" t="s">
         <v>890</v>
       </c>
       <c r="B16" s="2">
         <v>800000000</v>
       </c>
-      <c r="C16">
-        <v>0</v>
-      </c>
-      <c r="D16">
+      <c r="C16" s="12">
+        <v>0</v>
+      </c>
+      <c r="D16" s="12">
+        <v>-100</v>
+      </c>
+      <c r="E16" s="12">
+        <v>-200</v>
+      </c>
+      <c r="F16" s="12">
         <v>-1000</v>
       </c>
-      <c r="E16">
-        <v>-10000</v>
-      </c>
-      <c r="F16">
+      <c r="G16" s="12">
+        <v>-2000</v>
+      </c>
+      <c r="H16" s="12">
+        <v>-20000</v>
+      </c>
+      <c r="I16" s="12">
         <v>-100000</v>
       </c>
-      <c r="G16">
+      <c r="J16" s="12">
         <v>-200000</v>
       </c>
-      <c r="H16">
+      <c r="K16" s="12">
         <v>-600000</v>
+      </c>
+      <c r="L16" s="12">
+        <v>-1200000</v>
+      </c>
+      <c r="M16" s="12">
+        <v>-2400000</v>
       </c>
     </row>
     <row r="18" spans="2:18" x14ac:dyDescent="0.45">
@@ -5047,55 +5290,224 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:41" x14ac:dyDescent="0.45">
-      <c r="A1" t="s">
+      <c r="A1" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="12" t="s">
+        <v>1086</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>1087</v>
+      </c>
+      <c r="D1" s="12" t="s">
+        <v>1088</v>
+      </c>
+      <c r="E1" s="12" t="s">
+        <v>1089</v>
+      </c>
+      <c r="F1" s="12" t="s">
+        <v>1090</v>
+      </c>
+      <c r="G1" s="12" t="s">
+        <v>1035</v>
+      </c>
+      <c r="H1" s="12" t="s">
+        <v>1036</v>
+      </c>
+      <c r="I1" s="12" t="s">
+        <v>1037</v>
+      </c>
+      <c r="J1" s="12" t="s">
+        <v>1038</v>
+      </c>
+      <c r="K1" s="12" t="s">
+        <v>1039</v>
+      </c>
+      <c r="L1" s="12" t="s">
+        <v>1091</v>
+      </c>
+      <c r="M1" s="12" t="s">
+        <v>1092</v>
+      </c>
+      <c r="N1" s="12" t="s">
+        <v>1093</v>
+      </c>
+      <c r="O1" s="12" t="s">
+        <v>1094</v>
+      </c>
+      <c r="P1" s="12" t="s">
+        <v>1095</v>
+      </c>
+      <c r="Q1" s="12" t="s">
+        <v>1040</v>
+      </c>
+      <c r="R1" s="12" t="s">
+        <v>1041</v>
+      </c>
+      <c r="S1" s="12" t="s">
+        <v>1042</v>
+      </c>
+      <c r="T1" s="12" t="s">
+        <v>1043</v>
+      </c>
+      <c r="U1" s="12" t="s">
+        <v>1044</v>
+      </c>
+      <c r="V1" s="12" t="s">
+        <v>1059</v>
+      </c>
+      <c r="W1" s="12" t="s">
+        <v>1060</v>
+      </c>
+      <c r="X1" s="12" t="s">
+        <v>1061</v>
+      </c>
+      <c r="Y1" s="12" t="s">
+        <v>1062</v>
+      </c>
+      <c r="Z1" s="12" t="s">
         <v>920</v>
       </c>
-      <c r="C1"/>
+      <c r="AA1" s="12" t="s">
+        <v>1063</v>
+      </c>
+      <c r="AB1" s="12" t="s">
+        <v>1064</v>
+      </c>
+      <c r="AC1" s="12" t="s">
+        <v>1065</v>
+      </c>
+      <c r="AD1" s="12" t="s">
+        <v>1066</v>
+      </c>
+      <c r="AE1" s="12" t="s">
+        <v>921</v>
+      </c>
+      <c r="AF1" s="12" t="s">
+        <v>1067</v>
+      </c>
+      <c r="AG1" s="12" t="s">
+        <v>1068</v>
+      </c>
+      <c r="AH1" s="12" t="s">
+        <v>1069</v>
+      </c>
+      <c r="AI1" s="12" t="s">
+        <v>1070</v>
+      </c>
+      <c r="AJ1" s="12" t="s">
+        <v>1071</v>
+      </c>
     </row>
     <row r="2" spans="1:41" x14ac:dyDescent="0.45">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="16" t="s">
         <v>42</v>
       </c>
       <c r="B2" s="13">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="C2" s="13">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="D2" s="13">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="E2" s="13">
+        <v>8.64</v>
+      </c>
+      <c r="F2" s="13">
         <v>86.4</v>
       </c>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13"/>
-      <c r="H2" s="13"/>
-      <c r="I2" s="13"/>
-      <c r="J2" s="13"/>
-      <c r="K2" s="13"/>
-      <c r="L2" s="13"/>
-      <c r="M2" s="13"/>
-      <c r="N2" s="13"/>
-      <c r="O2" s="13"/>
-      <c r="P2" s="13"/>
-      <c r="Q2" s="13"/>
-      <c r="R2" s="13"/>
-      <c r="S2" s="13"/>
-      <c r="T2" s="13"/>
-      <c r="U2" s="13"/>
-      <c r="V2" s="13"/>
-      <c r="W2" s="13"/>
-      <c r="X2" s="13"/>
-      <c r="Y2" s="13"/>
-      <c r="Z2" s="13"/>
-      <c r="AA2" s="13"/>
-      <c r="AB2" s="13"/>
-      <c r="AC2" s="13"/>
-      <c r="AD2" s="13"/>
-      <c r="AE2" s="13"/>
-      <c r="AF2" s="13"/>
-      <c r="AG2" s="13"/>
-      <c r="AH2" s="13"/>
-      <c r="AI2" s="13"/>
-      <c r="AJ2" s="13"/>
+      <c r="G2" s="13">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="H2" s="13">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="I2" s="13">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="J2" s="13">
+        <v>8.64</v>
+      </c>
+      <c r="K2" s="13">
+        <v>86.4</v>
+      </c>
+      <c r="L2" s="13">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="M2" s="13">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="N2" s="13">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="O2" s="13">
+        <v>8.64</v>
+      </c>
+      <c r="P2" s="13">
+        <v>86.4</v>
+      </c>
+      <c r="Q2" s="13">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="R2" s="13">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="S2" s="13">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="T2" s="13">
+        <v>8.64</v>
+      </c>
+      <c r="U2" s="13">
+        <v>86.4</v>
+      </c>
+      <c r="V2" s="13">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="W2" s="13">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="X2" s="13">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="Y2" s="13">
+        <v>8.64</v>
+      </c>
+      <c r="Z2" s="13">
+        <v>86.4</v>
+      </c>
+      <c r="AA2" s="13">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="AB2" s="13">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="AC2" s="13">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="AD2" s="13">
+        <v>8.64</v>
+      </c>
+      <c r="AE2" s="13">
+        <v>86.4</v>
+      </c>
+      <c r="AF2" s="13">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="AG2" s="13">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="AH2" s="13">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="AI2" s="13">
+        <v>8.64</v>
+      </c>
+      <c r="AJ2" s="13">
+        <v>86.4</v>
+      </c>
       <c r="AK2" s="13"/>
       <c r="AL2" s="13"/>
       <c r="AM2" s="13"/>
@@ -5103,46 +5515,114 @@
       <c r="AO2" s="13"/>
     </row>
     <row r="3" spans="1:41" x14ac:dyDescent="0.45">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="16" t="s">
         <v>46</v>
       </c>
       <c r="B3" s="14">
+        <v>8.6400000000000003E-6</v>
+      </c>
+      <c r="C3" s="14">
+        <v>8.6400000000000003E-6</v>
+      </c>
+      <c r="D3" s="14">
+        <v>8.6400000000000003E-6</v>
+      </c>
+      <c r="E3" s="14">
+        <v>8.6400000000000003E-6</v>
+      </c>
+      <c r="F3" s="14">
+        <v>8.6400000000000003E-6</v>
+      </c>
+      <c r="G3" s="14">
+        <v>8.6399999999999999E-5</v>
+      </c>
+      <c r="H3" s="14">
+        <v>8.6399999999999999E-5</v>
+      </c>
+      <c r="I3" s="14">
+        <v>8.6399999999999999E-5</v>
+      </c>
+      <c r="J3" s="14">
+        <v>8.6399999999999999E-5</v>
+      </c>
+      <c r="K3" s="14">
+        <v>8.6399999999999999E-5</v>
+      </c>
+      <c r="L3" s="14">
+        <v>8.6399999999999997E-4</v>
+      </c>
+      <c r="M3" s="14">
+        <v>8.6399999999999997E-4</v>
+      </c>
+      <c r="N3" s="14">
+        <v>8.6399999999999997E-4</v>
+      </c>
+      <c r="O3" s="14">
+        <v>8.6399999999999997E-4</v>
+      </c>
+      <c r="P3" s="14">
+        <v>8.6399999999999997E-4</v>
+      </c>
+      <c r="Q3" s="14">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="R3" s="14">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="S3" s="14">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="T3" s="14">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="U3" s="14">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="V3" s="14">
         <v>8.6399999999999999E-9</v>
       </c>
-      <c r="C3" s="11"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="14"/>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="14"/>
-      <c r="L3" s="14"/>
-      <c r="M3" s="14"/>
-      <c r="N3" s="14"/>
-      <c r="O3" s="14"/>
-      <c r="P3" s="14"/>
-      <c r="Q3" s="14"/>
-      <c r="R3" s="14"/>
-      <c r="S3" s="14"/>
-      <c r="T3" s="14"/>
-      <c r="U3" s="14"/>
-      <c r="V3" s="14"/>
-      <c r="W3" s="14"/>
-      <c r="X3" s="14"/>
-      <c r="Y3" s="14"/>
-      <c r="Z3" s="14"/>
-      <c r="AA3" s="13"/>
-      <c r="AB3" s="13"/>
-      <c r="AC3" s="13"/>
-      <c r="AD3" s="13"/>
-      <c r="AE3" s="13"/>
-      <c r="AF3" s="13"/>
-      <c r="AG3" s="13"/>
-      <c r="AH3" s="13"/>
-      <c r="AI3" s="13"/>
-      <c r="AJ3" s="13"/>
+      <c r="W3" s="14">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="X3" s="14">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="Y3" s="14">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="Z3" s="14">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="AA3" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="AB3" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="AC3" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="AD3" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="AE3" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="AF3" s="14">
+        <v>8.6400000000000001E-7</v>
+      </c>
+      <c r="AG3" s="14">
+        <v>8.6400000000000001E-7</v>
+      </c>
+      <c r="AH3" s="14">
+        <v>8.6400000000000001E-7</v>
+      </c>
+      <c r="AI3" s="14">
+        <v>8.6400000000000001E-7</v>
+      </c>
+      <c r="AJ3" s="14">
+        <v>8.6400000000000001E-7</v>
+      </c>
       <c r="AK3" s="13"/>
       <c r="AL3" s="13"/>
       <c r="AM3" s="13"/>
@@ -5150,46 +5630,114 @@
       <c r="AO3" s="13"/>
     </row>
     <row r="4" spans="1:41" x14ac:dyDescent="0.45">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="16" t="s">
         <v>48</v>
       </c>
       <c r="B4" s="13">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="C4" s="13">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="D4" s="13">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="E4" s="13">
+        <v>8.64</v>
+      </c>
+      <c r="F4" s="13">
         <v>86.4</v>
       </c>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="13"/>
-      <c r="F4" s="13"/>
-      <c r="G4" s="13"/>
-      <c r="H4" s="13"/>
-      <c r="I4" s="13"/>
-      <c r="J4" s="13"/>
-      <c r="K4" s="13"/>
-      <c r="L4" s="13"/>
-      <c r="M4" s="13"/>
-      <c r="N4" s="13"/>
-      <c r="O4" s="13"/>
-      <c r="P4" s="13"/>
-      <c r="Q4" s="13"/>
-      <c r="R4" s="13"/>
-      <c r="S4" s="13"/>
-      <c r="T4" s="13"/>
-      <c r="U4" s="13"/>
-      <c r="V4" s="13"/>
-      <c r="W4" s="13"/>
-      <c r="X4" s="13"/>
-      <c r="Y4" s="13"/>
-      <c r="Z4" s="13"/>
-      <c r="AA4" s="13"/>
-      <c r="AB4" s="13"/>
-      <c r="AC4" s="13"/>
-      <c r="AD4" s="13"/>
-      <c r="AE4" s="13"/>
-      <c r="AF4" s="13"/>
-      <c r="AG4" s="13"/>
-      <c r="AH4" s="13"/>
-      <c r="AI4" s="13"/>
-      <c r="AJ4" s="13"/>
+      <c r="G4" s="13">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="H4" s="13">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="I4" s="13">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="J4" s="13">
+        <v>8.64</v>
+      </c>
+      <c r="K4" s="13">
+        <v>86.4</v>
+      </c>
+      <c r="L4" s="13">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="M4" s="13">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="N4" s="13">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="O4" s="13">
+        <v>8.64</v>
+      </c>
+      <c r="P4" s="13">
+        <v>86.4</v>
+      </c>
+      <c r="Q4" s="13">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="R4" s="13">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="S4" s="13">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="T4" s="13">
+        <v>8.64</v>
+      </c>
+      <c r="U4" s="13">
+        <v>86.4</v>
+      </c>
+      <c r="V4" s="13">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="W4" s="13">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="X4" s="13">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="Y4" s="13">
+        <v>8.64</v>
+      </c>
+      <c r="Z4" s="13">
+        <v>86.4</v>
+      </c>
+      <c r="AA4" s="13">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="AB4" s="13">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="AC4" s="13">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="AD4" s="13">
+        <v>8.64</v>
+      </c>
+      <c r="AE4" s="13">
+        <v>86.4</v>
+      </c>
+      <c r="AF4" s="13">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="AG4" s="13">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="AH4" s="13">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="AI4" s="13">
+        <v>8.64</v>
+      </c>
+      <c r="AJ4" s="13">
+        <v>86.4</v>
+      </c>
       <c r="AK4" s="13"/>
       <c r="AL4" s="13"/>
       <c r="AM4" s="13"/>
@@ -5197,46 +5745,114 @@
       <c r="AO4" s="13"/>
     </row>
     <row r="5" spans="1:41" x14ac:dyDescent="0.45">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="16" t="s">
         <v>50</v>
       </c>
       <c r="B5" s="14">
+        <v>8.6400000000000003E-6</v>
+      </c>
+      <c r="C5" s="14">
+        <v>8.6400000000000003E-6</v>
+      </c>
+      <c r="D5" s="14">
+        <v>8.6400000000000003E-6</v>
+      </c>
+      <c r="E5" s="14">
+        <v>8.6400000000000003E-6</v>
+      </c>
+      <c r="F5" s="14">
+        <v>8.6400000000000003E-6</v>
+      </c>
+      <c r="G5" s="14">
+        <v>8.6399999999999999E-5</v>
+      </c>
+      <c r="H5" s="14">
+        <v>8.6399999999999999E-5</v>
+      </c>
+      <c r="I5" s="14">
+        <v>8.6399999999999999E-5</v>
+      </c>
+      <c r="J5" s="14">
+        <v>8.6399999999999999E-5</v>
+      </c>
+      <c r="K5" s="14">
+        <v>8.6399999999999999E-5</v>
+      </c>
+      <c r="L5" s="14">
+        <v>8.6399999999999997E-4</v>
+      </c>
+      <c r="M5" s="14">
+        <v>8.6399999999999997E-4</v>
+      </c>
+      <c r="N5" s="14">
+        <v>8.6399999999999997E-4</v>
+      </c>
+      <c r="O5" s="14">
+        <v>8.6399999999999997E-4</v>
+      </c>
+      <c r="P5" s="14">
+        <v>8.6399999999999997E-4</v>
+      </c>
+      <c r="Q5" s="14">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="R5" s="14">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="S5" s="14">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="T5" s="14">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="U5" s="14">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="V5" s="14">
         <v>8.6399999999999999E-9</v>
       </c>
-      <c r="C5" s="11"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="14"/>
-      <c r="F5" s="14"/>
-      <c r="G5" s="14"/>
-      <c r="H5" s="14"/>
-      <c r="I5" s="14"/>
-      <c r="J5" s="14"/>
-      <c r="K5" s="14"/>
-      <c r="L5" s="14"/>
-      <c r="M5" s="14"/>
-      <c r="N5" s="14"/>
-      <c r="O5" s="14"/>
-      <c r="P5" s="14"/>
-      <c r="Q5" s="14"/>
-      <c r="R5" s="14"/>
-      <c r="S5" s="14"/>
-      <c r="T5" s="14"/>
-      <c r="U5" s="14"/>
-      <c r="V5" s="14"/>
-      <c r="W5" s="14"/>
-      <c r="X5" s="14"/>
-      <c r="Y5" s="14"/>
-      <c r="Z5" s="14"/>
-      <c r="AA5" s="13"/>
-      <c r="AB5" s="13"/>
-      <c r="AC5" s="13"/>
-      <c r="AD5" s="13"/>
-      <c r="AE5" s="13"/>
-      <c r="AF5" s="13"/>
-      <c r="AG5" s="13"/>
-      <c r="AH5" s="13"/>
-      <c r="AI5" s="13"/>
-      <c r="AJ5" s="13"/>
+      <c r="W5" s="14">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="X5" s="14">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="Y5" s="14">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="Z5" s="14">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="AA5" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="AB5" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="AC5" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="AD5" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="AE5" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="AF5" s="14">
+        <v>8.6400000000000001E-7</v>
+      </c>
+      <c r="AG5" s="14">
+        <v>8.6400000000000001E-7</v>
+      </c>
+      <c r="AH5" s="14">
+        <v>8.6400000000000001E-7</v>
+      </c>
+      <c r="AI5" s="14">
+        <v>8.6400000000000001E-7</v>
+      </c>
+      <c r="AJ5" s="14">
+        <v>8.6400000000000001E-7</v>
+      </c>
       <c r="AK5" s="13"/>
       <c r="AL5" s="13"/>
       <c r="AM5" s="13"/>
@@ -5244,46 +5860,114 @@
       <c r="AO5" s="13"/>
     </row>
     <row r="6" spans="1:41" x14ac:dyDescent="0.45">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="16" t="s">
         <v>52</v>
       </c>
       <c r="B6" s="13">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="C6" s="13">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="D6" s="13">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="E6" s="13">
+        <v>8.64</v>
+      </c>
+      <c r="F6" s="13">
         <v>86.4</v>
       </c>
-      <c r="C6" s="13"/>
-      <c r="D6" s="13"/>
-      <c r="E6" s="13"/>
-      <c r="F6" s="13"/>
-      <c r="G6" s="13"/>
-      <c r="H6" s="13"/>
-      <c r="I6" s="13"/>
-      <c r="J6" s="13"/>
-      <c r="K6" s="13"/>
-      <c r="L6" s="13"/>
-      <c r="M6" s="13"/>
-      <c r="N6" s="13"/>
-      <c r="O6" s="13"/>
-      <c r="P6" s="13"/>
-      <c r="Q6" s="13"/>
-      <c r="R6" s="13"/>
-      <c r="S6" s="13"/>
-      <c r="T6" s="13"/>
-      <c r="U6" s="13"/>
-      <c r="V6" s="13"/>
-      <c r="W6" s="13"/>
-      <c r="X6" s="13"/>
-      <c r="Y6" s="13"/>
-      <c r="Z6" s="13"/>
-      <c r="AA6" s="13"/>
-      <c r="AB6" s="13"/>
-      <c r="AC6" s="13"/>
-      <c r="AD6" s="13"/>
-      <c r="AE6" s="13"/>
-      <c r="AF6" s="13"/>
-      <c r="AG6" s="13"/>
-      <c r="AH6" s="13"/>
-      <c r="AI6" s="13"/>
-      <c r="AJ6" s="13"/>
+      <c r="G6" s="13">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="H6" s="13">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="I6" s="13">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="J6" s="13">
+        <v>8.64</v>
+      </c>
+      <c r="K6" s="13">
+        <v>86.4</v>
+      </c>
+      <c r="L6" s="13">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="M6" s="13">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="N6" s="13">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="O6" s="13">
+        <v>8.64</v>
+      </c>
+      <c r="P6" s="13">
+        <v>86.4</v>
+      </c>
+      <c r="Q6" s="13">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="R6" s="13">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="S6" s="13">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="T6" s="13">
+        <v>8.64</v>
+      </c>
+      <c r="U6" s="13">
+        <v>86.4</v>
+      </c>
+      <c r="V6" s="13">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="W6" s="13">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="X6" s="13">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="Y6" s="13">
+        <v>8.64</v>
+      </c>
+      <c r="Z6" s="13">
+        <v>86.4</v>
+      </c>
+      <c r="AA6" s="13">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="AB6" s="13">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="AC6" s="13">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="AD6" s="13">
+        <v>8.64</v>
+      </c>
+      <c r="AE6" s="13">
+        <v>86.4</v>
+      </c>
+      <c r="AF6" s="13">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="AG6" s="13">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="AH6" s="13">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="AI6" s="13">
+        <v>8.64</v>
+      </c>
+      <c r="AJ6" s="13">
+        <v>86.4</v>
+      </c>
       <c r="AK6" s="13"/>
       <c r="AL6" s="13"/>
       <c r="AM6" s="13"/>
@@ -5291,46 +5975,114 @@
       <c r="AO6" s="13"/>
     </row>
     <row r="7" spans="1:41" x14ac:dyDescent="0.45">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="16" t="s">
         <v>54</v>
       </c>
       <c r="B7" s="13">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="C7" s="13">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="D7" s="13">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="E7" s="13">
+        <v>8.64</v>
+      </c>
+      <c r="F7" s="13">
         <v>86.4</v>
       </c>
-      <c r="C7" s="13"/>
-      <c r="D7" s="13"/>
-      <c r="E7" s="13"/>
-      <c r="F7" s="13"/>
-      <c r="G7" s="13"/>
-      <c r="H7" s="13"/>
-      <c r="I7" s="13"/>
-      <c r="J7" s="13"/>
-      <c r="K7" s="13"/>
-      <c r="L7" s="13"/>
-      <c r="M7" s="13"/>
-      <c r="N7" s="13"/>
-      <c r="O7" s="13"/>
-      <c r="P7" s="13"/>
-      <c r="Q7" s="13"/>
-      <c r="R7" s="13"/>
-      <c r="S7" s="13"/>
-      <c r="T7" s="13"/>
-      <c r="U7" s="13"/>
-      <c r="V7" s="13"/>
-      <c r="W7" s="13"/>
-      <c r="X7" s="13"/>
-      <c r="Y7" s="13"/>
-      <c r="Z7" s="13"/>
-      <c r="AA7" s="13"/>
-      <c r="AB7" s="13"/>
-      <c r="AC7" s="13"/>
-      <c r="AD7" s="13"/>
-      <c r="AE7" s="13"/>
-      <c r="AF7" s="13"/>
-      <c r="AG7" s="13"/>
-      <c r="AH7" s="13"/>
-      <c r="AI7" s="13"/>
-      <c r="AJ7" s="13"/>
+      <c r="G7" s="13">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="H7" s="13">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="I7" s="13">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="J7" s="13">
+        <v>8.64</v>
+      </c>
+      <c r="K7" s="13">
+        <v>86.4</v>
+      </c>
+      <c r="L7" s="13">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="M7" s="13">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="N7" s="13">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="O7" s="13">
+        <v>8.64</v>
+      </c>
+      <c r="P7" s="13">
+        <v>86.4</v>
+      </c>
+      <c r="Q7" s="13">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="R7" s="13">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="S7" s="13">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="T7" s="13">
+        <v>8.64</v>
+      </c>
+      <c r="U7" s="13">
+        <v>86.4</v>
+      </c>
+      <c r="V7" s="13">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="W7" s="13">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="X7" s="13">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="Y7" s="13">
+        <v>8.64</v>
+      </c>
+      <c r="Z7" s="13">
+        <v>86.4</v>
+      </c>
+      <c r="AA7" s="13">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="AB7" s="13">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="AC7" s="13">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="AD7" s="13">
+        <v>8.64</v>
+      </c>
+      <c r="AE7" s="13">
+        <v>86.4</v>
+      </c>
+      <c r="AF7" s="13">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="AG7" s="13">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="AH7" s="13">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="AI7" s="13">
+        <v>8.64</v>
+      </c>
+      <c r="AJ7" s="13">
+        <v>86.4</v>
+      </c>
       <c r="AK7" s="13"/>
       <c r="AL7" s="13"/>
       <c r="AM7" s="13"/>
@@ -5338,46 +6090,114 @@
       <c r="AO7" s="13"/>
     </row>
     <row r="8" spans="1:41" x14ac:dyDescent="0.45">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="16" t="s">
         <v>55</v>
       </c>
       <c r="B8" s="14">
+        <v>8.6400000000000003E-6</v>
+      </c>
+      <c r="C8" s="14">
+        <v>8.6400000000000003E-6</v>
+      </c>
+      <c r="D8" s="14">
+        <v>8.6400000000000003E-6</v>
+      </c>
+      <c r="E8" s="14">
+        <v>8.6400000000000003E-6</v>
+      </c>
+      <c r="F8" s="14">
+        <v>8.6400000000000003E-6</v>
+      </c>
+      <c r="G8" s="14">
+        <v>8.6399999999999999E-5</v>
+      </c>
+      <c r="H8" s="14">
+        <v>8.6399999999999999E-5</v>
+      </c>
+      <c r="I8" s="14">
+        <v>8.6399999999999999E-5</v>
+      </c>
+      <c r="J8" s="14">
+        <v>8.6399999999999999E-5</v>
+      </c>
+      <c r="K8" s="14">
+        <v>8.6399999999999999E-5</v>
+      </c>
+      <c r="L8" s="14">
+        <v>8.6399999999999997E-4</v>
+      </c>
+      <c r="M8" s="14">
+        <v>8.6399999999999997E-4</v>
+      </c>
+      <c r="N8" s="14">
+        <v>8.6399999999999997E-4</v>
+      </c>
+      <c r="O8" s="14">
+        <v>8.6399999999999997E-4</v>
+      </c>
+      <c r="P8" s="14">
+        <v>8.6399999999999997E-4</v>
+      </c>
+      <c r="Q8" s="14">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="R8" s="14">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="S8" s="14">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="T8" s="14">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="U8" s="14">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="V8" s="14">
         <v>8.6399999999999999E-9</v>
       </c>
-      <c r="C8" s="11"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
-      <c r="I8" s="14"/>
-      <c r="J8" s="14"/>
-      <c r="K8" s="14"/>
-      <c r="L8" s="14"/>
-      <c r="M8" s="14"/>
-      <c r="N8" s="14"/>
-      <c r="O8" s="14"/>
-      <c r="P8" s="14"/>
-      <c r="Q8" s="14"/>
-      <c r="R8" s="14"/>
-      <c r="S8" s="14"/>
-      <c r="T8" s="14"/>
-      <c r="U8" s="14"/>
-      <c r="V8" s="14"/>
-      <c r="W8" s="14"/>
-      <c r="X8" s="14"/>
-      <c r="Y8" s="14"/>
-      <c r="Z8" s="14"/>
-      <c r="AA8" s="13"/>
-      <c r="AB8" s="13"/>
-      <c r="AC8" s="13"/>
-      <c r="AD8" s="13"/>
-      <c r="AE8" s="13"/>
-      <c r="AF8" s="13"/>
-      <c r="AG8" s="13"/>
-      <c r="AH8" s="13"/>
-      <c r="AI8" s="13"/>
-      <c r="AJ8" s="13"/>
+      <c r="W8" s="14">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="X8" s="14">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="Y8" s="14">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="Z8" s="14">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="AA8" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="AB8" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="AC8" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="AD8" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="AE8" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="AF8" s="14">
+        <v>8.6400000000000001E-7</v>
+      </c>
+      <c r="AG8" s="14">
+        <v>8.6400000000000001E-7</v>
+      </c>
+      <c r="AH8" s="14">
+        <v>8.6400000000000001E-7</v>
+      </c>
+      <c r="AI8" s="14">
+        <v>8.6400000000000001E-7</v>
+      </c>
+      <c r="AJ8" s="14">
+        <v>8.6400000000000001E-7</v>
+      </c>
       <c r="AK8" s="13"/>
       <c r="AL8" s="13"/>
       <c r="AM8" s="13"/>
@@ -5385,46 +6205,114 @@
       <c r="AO8" s="13"/>
     </row>
     <row r="9" spans="1:41" x14ac:dyDescent="0.45">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="16" t="s">
         <v>56</v>
       </c>
       <c r="B9" s="13">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="C9" s="13">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="D9" s="13">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="E9" s="13">
+        <v>8.64</v>
+      </c>
+      <c r="F9" s="13">
         <v>86.4</v>
       </c>
-      <c r="C9" s="13"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="13"/>
-      <c r="F9" s="13"/>
-      <c r="G9" s="13"/>
-      <c r="H9" s="13"/>
-      <c r="I9" s="13"/>
-      <c r="J9" s="13"/>
-      <c r="K9" s="13"/>
-      <c r="L9" s="13"/>
-      <c r="M9" s="13"/>
-      <c r="N9" s="13"/>
-      <c r="O9" s="13"/>
-      <c r="P9" s="13"/>
-      <c r="Q9" s="13"/>
-      <c r="R9" s="13"/>
-      <c r="S9" s="13"/>
-      <c r="T9" s="13"/>
-      <c r="U9" s="13"/>
-      <c r="V9" s="13"/>
-      <c r="W9" s="13"/>
-      <c r="X9" s="13"/>
-      <c r="Y9" s="13"/>
-      <c r="Z9" s="13"/>
-      <c r="AA9" s="13"/>
-      <c r="AB9" s="13"/>
-      <c r="AC9" s="13"/>
-      <c r="AD9" s="13"/>
-      <c r="AE9" s="13"/>
-      <c r="AF9" s="13"/>
-      <c r="AG9" s="13"/>
-      <c r="AH9" s="13"/>
-      <c r="AI9" s="13"/>
-      <c r="AJ9" s="13"/>
+      <c r="G9" s="13">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="H9" s="13">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="I9" s="13">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="J9" s="13">
+        <v>8.64</v>
+      </c>
+      <c r="K9" s="13">
+        <v>86.4</v>
+      </c>
+      <c r="L9" s="13">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="M9" s="13">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="N9" s="13">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="O9" s="13">
+        <v>8.64</v>
+      </c>
+      <c r="P9" s="13">
+        <v>86.4</v>
+      </c>
+      <c r="Q9" s="13">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="R9" s="13">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="S9" s="13">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="T9" s="13">
+        <v>8.64</v>
+      </c>
+      <c r="U9" s="13">
+        <v>86.4</v>
+      </c>
+      <c r="V9" s="13">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="W9" s="13">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="X9" s="13">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="Y9" s="13">
+        <v>8.64</v>
+      </c>
+      <c r="Z9" s="13">
+        <v>86.4</v>
+      </c>
+      <c r="AA9" s="13">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="AB9" s="13">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="AC9" s="13">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="AD9" s="13">
+        <v>8.64</v>
+      </c>
+      <c r="AE9" s="13">
+        <v>86.4</v>
+      </c>
+      <c r="AF9" s="13">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="AG9" s="13">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="AH9" s="13">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="AI9" s="13">
+        <v>8.64</v>
+      </c>
+      <c r="AJ9" s="13">
+        <v>86.4</v>
+      </c>
       <c r="AK9" s="13"/>
       <c r="AL9" s="13"/>
       <c r="AM9" s="13"/>
@@ -5432,46 +6320,114 @@
       <c r="AO9" s="13"/>
     </row>
     <row r="10" spans="1:41" x14ac:dyDescent="0.45">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="16" t="s">
         <v>57</v>
       </c>
       <c r="B10" s="14">
+        <v>8.6400000000000003E-6</v>
+      </c>
+      <c r="C10" s="14">
+        <v>8.6400000000000003E-6</v>
+      </c>
+      <c r="D10" s="14">
+        <v>8.6400000000000003E-6</v>
+      </c>
+      <c r="E10" s="14">
+        <v>8.6400000000000003E-6</v>
+      </c>
+      <c r="F10" s="14">
+        <v>8.6400000000000003E-6</v>
+      </c>
+      <c r="G10" s="14">
+        <v>8.6399999999999999E-5</v>
+      </c>
+      <c r="H10" s="14">
+        <v>8.6399999999999999E-5</v>
+      </c>
+      <c r="I10" s="14">
+        <v>8.6399999999999999E-5</v>
+      </c>
+      <c r="J10" s="14">
+        <v>8.6399999999999999E-5</v>
+      </c>
+      <c r="K10" s="14">
+        <v>8.6399999999999999E-5</v>
+      </c>
+      <c r="L10" s="14">
+        <v>8.6399999999999997E-4</v>
+      </c>
+      <c r="M10" s="14">
+        <v>8.6399999999999997E-4</v>
+      </c>
+      <c r="N10" s="14">
+        <v>8.6399999999999997E-4</v>
+      </c>
+      <c r="O10" s="14">
+        <v>8.6399999999999997E-4</v>
+      </c>
+      <c r="P10" s="14">
+        <v>8.6399999999999997E-4</v>
+      </c>
+      <c r="Q10" s="14">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="R10" s="14">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="S10" s="14">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="T10" s="14">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="U10" s="14">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="V10" s="14">
         <v>8.6399999999999999E-9</v>
       </c>
-      <c r="C10" s="11"/>
-      <c r="D10" s="14"/>
-      <c r="E10" s="14"/>
-      <c r="F10" s="14"/>
-      <c r="G10" s="14"/>
-      <c r="H10" s="14"/>
-      <c r="I10" s="14"/>
-      <c r="J10" s="14"/>
-      <c r="K10" s="14"/>
-      <c r="L10" s="14"/>
-      <c r="M10" s="14"/>
-      <c r="N10" s="14"/>
-      <c r="O10" s="14"/>
-      <c r="P10" s="14"/>
-      <c r="Q10" s="14"/>
-      <c r="R10" s="14"/>
-      <c r="S10" s="14"/>
-      <c r="T10" s="14"/>
-      <c r="U10" s="14"/>
-      <c r="V10" s="14"/>
-      <c r="W10" s="14"/>
-      <c r="X10" s="14"/>
-      <c r="Y10" s="14"/>
-      <c r="Z10" s="14"/>
-      <c r="AA10" s="13"/>
-      <c r="AB10" s="13"/>
-      <c r="AC10" s="13"/>
-      <c r="AD10" s="13"/>
-      <c r="AE10" s="13"/>
-      <c r="AF10" s="13"/>
-      <c r="AG10" s="13"/>
-      <c r="AH10" s="13"/>
-      <c r="AI10" s="13"/>
-      <c r="AJ10" s="13"/>
+      <c r="W10" s="14">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="X10" s="14">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="Y10" s="14">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="Z10" s="14">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="AA10" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="AB10" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="AC10" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="AD10" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="AE10" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="AF10" s="14">
+        <v>8.6400000000000001E-7</v>
+      </c>
+      <c r="AG10" s="14">
+        <v>8.6400000000000001E-7</v>
+      </c>
+      <c r="AH10" s="14">
+        <v>8.6400000000000001E-7</v>
+      </c>
+      <c r="AI10" s="14">
+        <v>8.6400000000000001E-7</v>
+      </c>
+      <c r="AJ10" s="14">
+        <v>8.6400000000000001E-7</v>
+      </c>
       <c r="AK10" s="13"/>
       <c r="AL10" s="13"/>
       <c r="AM10" s="13"/>
@@ -5479,46 +6435,114 @@
       <c r="AO10" s="13"/>
     </row>
     <row r="11" spans="1:41" x14ac:dyDescent="0.45">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="16" t="s">
         <v>58</v>
       </c>
       <c r="B11" s="13">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="C11" s="13">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="D11" s="13">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="E11" s="13">
+        <v>8.64</v>
+      </c>
+      <c r="F11" s="13">
         <v>86.4</v>
       </c>
-      <c r="C11" s="13"/>
-      <c r="D11" s="13"/>
-      <c r="E11" s="13"/>
-      <c r="F11" s="13"/>
-      <c r="G11" s="13"/>
-      <c r="H11" s="13"/>
-      <c r="I11" s="13"/>
-      <c r="J11" s="13"/>
-      <c r="K11" s="13"/>
-      <c r="L11" s="13"/>
-      <c r="M11" s="13"/>
-      <c r="N11" s="13"/>
-      <c r="O11" s="13"/>
-      <c r="P11" s="13"/>
-      <c r="Q11" s="13"/>
-      <c r="R11" s="13"/>
-      <c r="S11" s="13"/>
-      <c r="T11" s="13"/>
-      <c r="U11" s="13"/>
-      <c r="V11" s="13"/>
-      <c r="W11" s="13"/>
-      <c r="X11" s="13"/>
-      <c r="Y11" s="13"/>
-      <c r="Z11" s="13"/>
-      <c r="AA11" s="13"/>
-      <c r="AB11" s="13"/>
-      <c r="AC11" s="13"/>
-      <c r="AD11" s="13"/>
-      <c r="AE11" s="13"/>
-      <c r="AF11" s="13"/>
-      <c r="AG11" s="13"/>
-      <c r="AH11" s="13"/>
-      <c r="AI11" s="13"/>
-      <c r="AJ11" s="13"/>
+      <c r="G11" s="13">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="H11" s="13">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="I11" s="13">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="J11" s="13">
+        <v>8.64</v>
+      </c>
+      <c r="K11" s="13">
+        <v>86.4</v>
+      </c>
+      <c r="L11" s="13">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="M11" s="13">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="N11" s="13">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="O11" s="13">
+        <v>8.64</v>
+      </c>
+      <c r="P11" s="13">
+        <v>86.4</v>
+      </c>
+      <c r="Q11" s="13">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="R11" s="13">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="S11" s="13">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="T11" s="13">
+        <v>8.64</v>
+      </c>
+      <c r="U11" s="13">
+        <v>86.4</v>
+      </c>
+      <c r="V11" s="13">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="W11" s="13">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="X11" s="13">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="Y11" s="13">
+        <v>8.64</v>
+      </c>
+      <c r="Z11" s="13">
+        <v>86.4</v>
+      </c>
+      <c r="AA11" s="13">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="AB11" s="13">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="AC11" s="13">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="AD11" s="13">
+        <v>8.64</v>
+      </c>
+      <c r="AE11" s="13">
+        <v>86.4</v>
+      </c>
+      <c r="AF11" s="13">
+        <v>8.6400000000000001E-3</v>
+      </c>
+      <c r="AG11" s="13">
+        <v>8.6400000000000005E-2</v>
+      </c>
+      <c r="AH11" s="13">
+        <v>0.86399999999999999</v>
+      </c>
+      <c r="AI11" s="13">
+        <v>8.64</v>
+      </c>
+      <c r="AJ11" s="13">
+        <v>86.4</v>
+      </c>
       <c r="AK11" s="13"/>
       <c r="AL11" s="13"/>
       <c r="AM11" s="13"/>

</xml_diff>

<commit_message>
Updated files for the sustainable yield estimation using 3D model
</commit_message>
<xml_diff>
--- a/assets/3D/sust yield server/setup.xlsx
+++ b/assets/3D/sust yield server/setup.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmarinriver\Projects\ConfinedLab\assets\3D\sust yield server\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3179C0F9-D5FF-4DC2-8E52-431C9321CA93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7403F4B1-8A79-44A4-829C-6CC146A0529B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" firstSheet="3" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="grid" sheetId="1" r:id="rId1"/>
@@ -24,8 +24,9 @@
     <sheet name="response_times" sheetId="9" r:id="rId9"/>
     <sheet name="q_values_st" sheetId="10" r:id="rId10"/>
     <sheet name="q_values_tr" sheetId="11" r:id="rId11"/>
-    <sheet name="parameter_analysis" sheetId="12" r:id="rId12"/>
-    <sheet name="workplace" sheetId="13" r:id="rId13"/>
+    <sheet name="q_values_init" sheetId="14" r:id="rId12"/>
+    <sheet name="parameter_analysis" sheetId="12" r:id="rId13"/>
+    <sheet name="workplace" sheetId="13" r:id="rId14"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -46,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2504" uniqueCount="1192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2541" uniqueCount="1193">
   <si>
     <t>nlay</t>
   </si>
@@ -3622,13 +3623,16 @@
   </si>
   <si>
     <t>No data projection</t>
+  </si>
+  <si>
+    <t>q_init</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3672,6 +3676,12 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -3740,7 +3750,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -3772,6 +3782,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="11" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4482,34 +4495,34 @@
         <v>0</v>
       </c>
       <c r="D3" s="12">
-        <v>-100</v>
+        <v>-200</v>
       </c>
       <c r="E3" s="12">
-        <v>-200</v>
+        <v>-1000</v>
       </c>
       <c r="F3" s="12">
-        <v>-1000</v>
+        <v>-2000</v>
       </c>
       <c r="G3" s="12">
-        <v>-2000</v>
+        <v>-20000</v>
       </c>
       <c r="H3" s="12">
-        <v>-20000</v>
+        <v>-100000</v>
       </c>
       <c r="I3" s="12">
-        <v>-100000</v>
+        <v>-200000</v>
       </c>
       <c r="J3" s="12">
-        <v>-200000</v>
+        <v>-600000</v>
       </c>
       <c r="K3" s="12">
-        <v>-600000</v>
+        <v>-1200000</v>
       </c>
       <c r="L3" s="12">
-        <v>-1200000</v>
+        <v>-2400000</v>
       </c>
       <c r="M3" s="12">
-        <v>-2400000</v>
+        <v>-4800000</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.45">
@@ -4523,34 +4536,34 @@
         <v>0</v>
       </c>
       <c r="D4" s="12">
-        <v>-100</v>
+        <v>-200</v>
       </c>
       <c r="E4" s="12">
-        <v>-200</v>
+        <v>-1000</v>
       </c>
       <c r="F4" s="12">
-        <v>-1000</v>
+        <v>-2000</v>
       </c>
       <c r="G4" s="12">
-        <v>-2000</v>
+        <v>-20000</v>
       </c>
       <c r="H4" s="12">
-        <v>-20000</v>
+        <v>-100000</v>
       </c>
       <c r="I4" s="12">
-        <v>-100000</v>
+        <v>-200000</v>
       </c>
       <c r="J4" s="12">
-        <v>-200000</v>
+        <v>-600000</v>
       </c>
       <c r="K4" s="12">
-        <v>-600000</v>
+        <v>-1200000</v>
       </c>
       <c r="L4" s="12">
-        <v>-1200000</v>
+        <v>-2400000</v>
       </c>
       <c r="M4" s="12">
-        <v>-2400000</v>
+        <v>-4800000</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.45">
@@ -4605,34 +4618,34 @@
         <v>0</v>
       </c>
       <c r="D6" s="12">
-        <v>-100</v>
+        <v>-200</v>
       </c>
       <c r="E6" s="12">
-        <v>-200</v>
+        <v>-1000</v>
       </c>
       <c r="F6" s="12">
-        <v>-1000</v>
+        <v>-2000</v>
       </c>
       <c r="G6" s="12">
-        <v>-2000</v>
+        <v>-20000</v>
       </c>
       <c r="H6" s="12">
-        <v>-20000</v>
+        <v>-100000</v>
       </c>
       <c r="I6" s="12">
-        <v>-100000</v>
+        <v>-200000</v>
       </c>
       <c r="J6" s="12">
-        <v>-200000</v>
+        <v>-600000</v>
       </c>
       <c r="K6" s="12">
-        <v>-600000</v>
+        <v>-1200000</v>
       </c>
       <c r="L6" s="12">
-        <v>-1200000</v>
+        <v>-2400000</v>
       </c>
       <c r="M6" s="12">
-        <v>-2400000</v>
+        <v>-4800000</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.45">
@@ -4646,34 +4659,34 @@
         <v>0</v>
       </c>
       <c r="D7" s="12">
-        <v>-100</v>
+        <v>-200</v>
       </c>
       <c r="E7" s="12">
-        <v>-200</v>
+        <v>-1000</v>
       </c>
       <c r="F7" s="12">
-        <v>-1000</v>
+        <v>-2000</v>
       </c>
       <c r="G7" s="12">
-        <v>-2000</v>
+        <v>-20000</v>
       </c>
       <c r="H7" s="12">
-        <v>-20000</v>
+        <v>-100000</v>
       </c>
       <c r="I7" s="12">
-        <v>-100000</v>
+        <v>-200000</v>
       </c>
       <c r="J7" s="12">
-        <v>-200000</v>
+        <v>-600000</v>
       </c>
       <c r="K7" s="12">
-        <v>-600000</v>
+        <v>-1200000</v>
       </c>
       <c r="L7" s="12">
-        <v>-1200000</v>
+        <v>-2400000</v>
       </c>
       <c r="M7" s="12">
-        <v>-2400000</v>
+        <v>-4800000</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.45">
@@ -4728,34 +4741,34 @@
         <v>0</v>
       </c>
       <c r="D9" s="12">
-        <v>-100</v>
+        <v>-200</v>
       </c>
       <c r="E9" s="12">
-        <v>-200</v>
+        <v>-1000</v>
       </c>
       <c r="F9" s="12">
-        <v>-1000</v>
+        <v>-2000</v>
       </c>
       <c r="G9" s="12">
-        <v>-2000</v>
+        <v>-20000</v>
       </c>
       <c r="H9" s="12">
-        <v>-20000</v>
+        <v>-100000</v>
       </c>
       <c r="I9" s="12">
-        <v>-100000</v>
+        <v>-200000</v>
       </c>
       <c r="J9" s="12">
-        <v>-200000</v>
+        <v>-600000</v>
       </c>
       <c r="K9" s="12">
-        <v>-600000</v>
+        <v>-1200000</v>
       </c>
       <c r="L9" s="12">
-        <v>-1200000</v>
+        <v>-2400000</v>
       </c>
       <c r="M9" s="12">
-        <v>-2400000</v>
+        <v>-4800000</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.45">
@@ -4769,34 +4782,34 @@
         <v>0</v>
       </c>
       <c r="D10" s="12">
-        <v>-100</v>
+        <v>-200</v>
       </c>
       <c r="E10" s="12">
-        <v>-200</v>
+        <v>-1000</v>
       </c>
       <c r="F10" s="12">
-        <v>-1000</v>
+        <v>-2000</v>
       </c>
       <c r="G10" s="12">
-        <v>-2000</v>
+        <v>-20000</v>
       </c>
       <c r="H10" s="12">
-        <v>-20000</v>
+        <v>-100000</v>
       </c>
       <c r="I10" s="12">
-        <v>-100000</v>
+        <v>-200000</v>
       </c>
       <c r="J10" s="12">
-        <v>-200000</v>
+        <v>-600000</v>
       </c>
       <c r="K10" s="12">
-        <v>-600000</v>
+        <v>-1200000</v>
       </c>
       <c r="L10" s="12">
-        <v>-1200000</v>
+        <v>-2400000</v>
       </c>
       <c r="M10" s="12">
-        <v>-2400000</v>
+        <v>-4800000</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.45">
@@ -4851,34 +4864,34 @@
         <v>0</v>
       </c>
       <c r="D12" s="12">
-        <v>-100</v>
+        <v>-200</v>
       </c>
       <c r="E12" s="12">
-        <v>-200</v>
+        <v>-1000</v>
       </c>
       <c r="F12" s="12">
-        <v>-1000</v>
+        <v>-2000</v>
       </c>
       <c r="G12" s="12">
-        <v>-2000</v>
+        <v>-20000</v>
       </c>
       <c r="H12" s="12">
-        <v>-20000</v>
+        <v>-100000</v>
       </c>
       <c r="I12" s="12">
-        <v>-100000</v>
+        <v>-200000</v>
       </c>
       <c r="J12" s="12">
-        <v>-200000</v>
+        <v>-600000</v>
       </c>
       <c r="K12" s="12">
-        <v>-600000</v>
+        <v>-1200000</v>
       </c>
       <c r="L12" s="12">
-        <v>-1200000</v>
+        <v>-2400000</v>
       </c>
       <c r="M12" s="12">
-        <v>-2400000</v>
+        <v>-4800000</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.45">
@@ -4892,34 +4905,34 @@
         <v>0</v>
       </c>
       <c r="D13" s="12">
-        <v>-100</v>
+        <v>-200</v>
       </c>
       <c r="E13" s="12">
-        <v>-200</v>
+        <v>-1000</v>
       </c>
       <c r="F13" s="12">
-        <v>-1000</v>
+        <v>-2000</v>
       </c>
       <c r="G13" s="12">
-        <v>-2000</v>
+        <v>-20000</v>
       </c>
       <c r="H13" s="12">
-        <v>-20000</v>
+        <v>-100000</v>
       </c>
       <c r="I13" s="12">
-        <v>-100000</v>
+        <v>-200000</v>
       </c>
       <c r="J13" s="12">
-        <v>-200000</v>
+        <v>-600000</v>
       </c>
       <c r="K13" s="12">
-        <v>-600000</v>
+        <v>-1200000</v>
       </c>
       <c r="L13" s="12">
-        <v>-1200000</v>
+        <v>-2400000</v>
       </c>
       <c r="M13" s="12">
-        <v>-2400000</v>
+        <v>-4800000</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.45">
@@ -4974,34 +4987,34 @@
         <v>0</v>
       </c>
       <c r="D15" s="12">
-        <v>-100</v>
+        <v>-200</v>
       </c>
       <c r="E15" s="12">
-        <v>-200</v>
+        <v>-1000</v>
       </c>
       <c r="F15" s="12">
-        <v>-1000</v>
+        <v>-2000</v>
       </c>
       <c r="G15" s="12">
-        <v>-2000</v>
+        <v>-20000</v>
       </c>
       <c r="H15" s="12">
-        <v>-20000</v>
+        <v>-100000</v>
       </c>
       <c r="I15" s="12">
-        <v>-100000</v>
+        <v>-200000</v>
       </c>
       <c r="J15" s="12">
-        <v>-200000</v>
+        <v>-600000</v>
       </c>
       <c r="K15" s="12">
-        <v>-600000</v>
+        <v>-1200000</v>
       </c>
       <c r="L15" s="12">
-        <v>-1200000</v>
+        <v>-2400000</v>
       </c>
       <c r="M15" s="12">
-        <v>-2400000</v>
+        <v>-4800000</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.45">
@@ -5015,34 +5028,34 @@
         <v>0</v>
       </c>
       <c r="D16" s="12">
-        <v>-100</v>
+        <v>-200</v>
       </c>
       <c r="E16" s="12">
-        <v>-200</v>
+        <v>-1000</v>
       </c>
       <c r="F16" s="12">
-        <v>-1000</v>
+        <v>-2000</v>
       </c>
       <c r="G16" s="12">
-        <v>-2000</v>
+        <v>-20000</v>
       </c>
       <c r="H16" s="12">
-        <v>-20000</v>
+        <v>-100000</v>
       </c>
       <c r="I16" s="12">
-        <v>-100000</v>
+        <v>-200000</v>
       </c>
       <c r="J16" s="12">
-        <v>-200000</v>
+        <v>-600000</v>
       </c>
       <c r="K16" s="12">
-        <v>-600000</v>
+        <v>-1200000</v>
       </c>
       <c r="L16" s="12">
-        <v>-1200000</v>
+        <v>-2400000</v>
       </c>
       <c r="M16" s="12">
-        <v>-2400000</v>
+        <v>-4800000</v>
       </c>
     </row>
     <row r="18" spans="2:18" x14ac:dyDescent="0.45">
@@ -5282,11 +5295,634 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86C01BDA-8DD4-46BA-AD8C-0AB3FD0C776D}">
+  <dimension ref="A1:AJ36"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="16.265625" style="17" bestFit="1" customWidth="1"/>
+    <col min="2" max="16384" width="10.6640625" style="17"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:36" x14ac:dyDescent="0.45">
+      <c r="A1" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B1" s="17" t="s">
+        <v>1192</v>
+      </c>
+    </row>
+    <row r="2" spans="1:36" x14ac:dyDescent="0.45">
+      <c r="A2" s="17" t="s">
+        <v>1059</v>
+      </c>
+      <c r="B2" s="18">
+        <v>-20</v>
+      </c>
+      <c r="C2" s="18"/>
+      <c r="D2" s="18"/>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="18"/>
+      <c r="H2" s="18"/>
+      <c r="I2" s="18"/>
+      <c r="J2" s="18"/>
+      <c r="K2" s="18"/>
+      <c r="L2" s="18"/>
+      <c r="M2" s="18"/>
+      <c r="N2" s="18"/>
+      <c r="O2" s="18"/>
+      <c r="P2" s="18"/>
+      <c r="Q2" s="18"/>
+      <c r="R2" s="18"/>
+      <c r="S2" s="18"/>
+      <c r="T2" s="18"/>
+      <c r="U2" s="18"/>
+      <c r="V2" s="18"/>
+      <c r="W2" s="18"/>
+      <c r="X2" s="18"/>
+      <c r="Y2" s="18"/>
+      <c r="Z2" s="18"/>
+      <c r="AA2" s="18"/>
+      <c r="AB2" s="18"/>
+      <c r="AC2" s="18"/>
+      <c r="AD2" s="18"/>
+      <c r="AE2" s="18"/>
+      <c r="AF2" s="18"/>
+      <c r="AG2" s="18"/>
+      <c r="AH2" s="18"/>
+      <c r="AI2" s="18"/>
+      <c r="AJ2" s="18"/>
+    </row>
+    <row r="3" spans="1:36" x14ac:dyDescent="0.45">
+      <c r="A3" s="17" t="s">
+        <v>1060</v>
+      </c>
+      <c r="B3" s="18">
+        <v>-167</v>
+      </c>
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
+      <c r="G3" s="19"/>
+      <c r="H3" s="19"/>
+      <c r="I3" s="19"/>
+      <c r="J3" s="19"/>
+      <c r="K3" s="19"/>
+      <c r="L3" s="19"/>
+      <c r="M3" s="19"/>
+      <c r="N3" s="19"/>
+      <c r="O3" s="19"/>
+      <c r="P3" s="19"/>
+      <c r="Q3" s="19"/>
+      <c r="R3" s="19"/>
+      <c r="S3" s="19"/>
+      <c r="T3" s="19"/>
+      <c r="U3" s="19"/>
+      <c r="V3" s="19"/>
+      <c r="W3" s="19"/>
+      <c r="X3" s="19"/>
+      <c r="Y3" s="19"/>
+      <c r="Z3" s="19"/>
+      <c r="AF3" s="19"/>
+      <c r="AG3" s="19"/>
+      <c r="AH3" s="19"/>
+      <c r="AI3" s="19"/>
+      <c r="AJ3" s="19"/>
+    </row>
+    <row r="4" spans="1:36" x14ac:dyDescent="0.45">
+      <c r="A4" s="17" t="s">
+        <v>1061</v>
+      </c>
+      <c r="B4" s="18">
+        <v>-1609</v>
+      </c>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
+      <c r="G4" s="19"/>
+      <c r="H4" s="19"/>
+      <c r="I4" s="19"/>
+      <c r="J4" s="19"/>
+      <c r="K4" s="19"/>
+      <c r="L4" s="19"/>
+      <c r="M4" s="19"/>
+      <c r="N4" s="19"/>
+      <c r="O4" s="19"/>
+      <c r="P4" s="19"/>
+      <c r="Q4" s="19"/>
+      <c r="R4" s="19"/>
+      <c r="S4" s="19"/>
+      <c r="T4" s="19"/>
+      <c r="U4" s="19"/>
+      <c r="V4" s="19"/>
+      <c r="W4" s="19"/>
+      <c r="X4" s="19"/>
+      <c r="Y4" s="19"/>
+      <c r="Z4" s="19"/>
+      <c r="AA4" s="19"/>
+      <c r="AB4" s="19"/>
+      <c r="AC4" s="19"/>
+      <c r="AD4" s="19"/>
+      <c r="AE4" s="19"/>
+      <c r="AF4" s="19"/>
+      <c r="AG4" s="19"/>
+      <c r="AH4" s="19"/>
+      <c r="AI4" s="19"/>
+      <c r="AJ4" s="19"/>
+    </row>
+    <row r="5" spans="1:36" x14ac:dyDescent="0.45">
+      <c r="A5" s="17" t="s">
+        <v>1062</v>
+      </c>
+      <c r="B5" s="18">
+        <v>-16008</v>
+      </c>
+      <c r="C5" s="19"/>
+      <c r="D5" s="19"/>
+      <c r="E5" s="19"/>
+      <c r="F5" s="19"/>
+      <c r="G5" s="19"/>
+      <c r="H5" s="19"/>
+      <c r="I5" s="19"/>
+      <c r="J5" s="19"/>
+      <c r="K5" s="19"/>
+      <c r="L5" s="19"/>
+      <c r="M5" s="19"/>
+      <c r="N5" s="19"/>
+      <c r="O5" s="19"/>
+      <c r="P5" s="19"/>
+      <c r="Q5" s="19"/>
+      <c r="R5" s="19"/>
+      <c r="S5" s="19"/>
+      <c r="T5" s="19"/>
+      <c r="U5" s="19"/>
+      <c r="V5" s="19"/>
+      <c r="W5" s="19"/>
+      <c r="X5" s="19"/>
+      <c r="Y5" s="19"/>
+      <c r="Z5" s="19"/>
+      <c r="AF5" s="19"/>
+      <c r="AG5" s="19"/>
+      <c r="AH5" s="19"/>
+      <c r="AI5" s="19"/>
+      <c r="AJ5" s="19"/>
+    </row>
+    <row r="6" spans="1:36" x14ac:dyDescent="0.45">
+      <c r="A6" s="17" t="s">
+        <v>920</v>
+      </c>
+      <c r="B6" s="18">
+        <v>-159395</v>
+      </c>
+      <c r="C6" s="19"/>
+      <c r="D6" s="19"/>
+      <c r="E6" s="19"/>
+      <c r="F6" s="19"/>
+      <c r="G6" s="19"/>
+      <c r="H6" s="19"/>
+      <c r="I6" s="19"/>
+      <c r="J6" s="19"/>
+      <c r="K6" s="19"/>
+      <c r="L6" s="19"/>
+      <c r="M6" s="19"/>
+      <c r="N6" s="19"/>
+      <c r="O6" s="19"/>
+      <c r="P6" s="19"/>
+      <c r="Q6" s="19"/>
+      <c r="R6" s="19"/>
+      <c r="S6" s="19"/>
+      <c r="T6" s="19"/>
+      <c r="U6" s="19"/>
+      <c r="V6" s="19"/>
+      <c r="W6" s="19"/>
+      <c r="X6" s="19"/>
+      <c r="Y6" s="19"/>
+      <c r="Z6" s="19"/>
+      <c r="AA6" s="19"/>
+      <c r="AB6" s="19"/>
+      <c r="AC6" s="19"/>
+      <c r="AD6" s="19"/>
+      <c r="AE6" s="19"/>
+      <c r="AF6" s="19"/>
+      <c r="AG6" s="19"/>
+      <c r="AH6" s="19"/>
+      <c r="AI6" s="19"/>
+      <c r="AJ6" s="19"/>
+    </row>
+    <row r="7" spans="1:36" x14ac:dyDescent="0.45">
+      <c r="A7" s="17" t="s">
+        <v>1063</v>
+      </c>
+      <c r="B7" s="18">
+        <v>-27</v>
+      </c>
+      <c r="C7" s="19"/>
+      <c r="D7" s="19"/>
+      <c r="E7" s="19"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="19"/>
+      <c r="H7" s="19"/>
+      <c r="I7" s="19"/>
+      <c r="J7" s="19"/>
+      <c r="K7" s="19"/>
+      <c r="L7" s="19"/>
+      <c r="M7" s="19"/>
+      <c r="N7" s="19"/>
+      <c r="O7" s="19"/>
+      <c r="P7" s="19"/>
+      <c r="Q7" s="19"/>
+      <c r="R7" s="19"/>
+      <c r="S7" s="19"/>
+      <c r="T7" s="19"/>
+      <c r="U7" s="19"/>
+      <c r="V7" s="19"/>
+      <c r="W7" s="19"/>
+      <c r="X7" s="19"/>
+      <c r="Y7" s="19"/>
+      <c r="Z7" s="19"/>
+      <c r="AA7" s="19"/>
+      <c r="AB7" s="19"/>
+      <c r="AC7" s="19"/>
+      <c r="AD7" s="19"/>
+      <c r="AE7" s="19"/>
+      <c r="AF7" s="19"/>
+      <c r="AG7" s="19"/>
+      <c r="AH7" s="19"/>
+      <c r="AI7" s="19"/>
+      <c r="AJ7" s="19"/>
+    </row>
+    <row r="8" spans="1:36" x14ac:dyDescent="0.45">
+      <c r="A8" s="17" t="s">
+        <v>1064</v>
+      </c>
+      <c r="B8" s="18">
+        <v>-200</v>
+      </c>
+      <c r="C8" s="19"/>
+      <c r="D8" s="19"/>
+      <c r="E8" s="19"/>
+      <c r="F8" s="19"/>
+      <c r="G8" s="19"/>
+      <c r="H8" s="19"/>
+      <c r="I8" s="19"/>
+      <c r="J8" s="19"/>
+      <c r="K8" s="19"/>
+      <c r="L8" s="19"/>
+      <c r="M8" s="19"/>
+      <c r="N8" s="19"/>
+      <c r="O8" s="19"/>
+      <c r="P8" s="19"/>
+      <c r="Q8" s="19"/>
+      <c r="R8" s="19"/>
+      <c r="S8" s="19"/>
+      <c r="T8" s="19"/>
+      <c r="U8" s="19"/>
+      <c r="V8" s="19"/>
+      <c r="W8" s="19"/>
+      <c r="X8" s="19"/>
+      <c r="Y8" s="19"/>
+      <c r="Z8" s="19"/>
+      <c r="AF8" s="19"/>
+      <c r="AG8" s="19"/>
+      <c r="AH8" s="19"/>
+      <c r="AI8" s="19"/>
+      <c r="AJ8" s="19"/>
+    </row>
+    <row r="9" spans="1:36" x14ac:dyDescent="0.45">
+      <c r="A9" s="17" t="s">
+        <v>1065</v>
+      </c>
+      <c r="B9" s="18">
+        <v>-1668</v>
+      </c>
+      <c r="C9" s="19"/>
+      <c r="D9" s="19"/>
+      <c r="E9" s="19"/>
+      <c r="F9" s="19"/>
+      <c r="G9" s="19"/>
+      <c r="H9" s="19"/>
+      <c r="I9" s="19"/>
+      <c r="J9" s="19"/>
+      <c r="K9" s="19"/>
+      <c r="L9" s="19"/>
+      <c r="M9" s="19"/>
+      <c r="N9" s="19"/>
+      <c r="O9" s="19"/>
+      <c r="P9" s="19"/>
+      <c r="Q9" s="19"/>
+      <c r="R9" s="19"/>
+      <c r="S9" s="19"/>
+      <c r="T9" s="19"/>
+      <c r="U9" s="19"/>
+      <c r="V9" s="19"/>
+      <c r="W9" s="19"/>
+      <c r="X9" s="19"/>
+      <c r="Y9" s="19"/>
+      <c r="Z9" s="19"/>
+      <c r="AA9" s="19"/>
+      <c r="AB9" s="19"/>
+      <c r="AC9" s="19"/>
+      <c r="AD9" s="19"/>
+      <c r="AE9" s="19"/>
+      <c r="AF9" s="19"/>
+      <c r="AG9" s="19"/>
+      <c r="AH9" s="19"/>
+      <c r="AI9" s="19"/>
+      <c r="AJ9" s="19"/>
+    </row>
+    <row r="10" spans="1:36" x14ac:dyDescent="0.45">
+      <c r="A10" s="17" t="s">
+        <v>1066</v>
+      </c>
+      <c r="B10" s="18">
+        <v>-16074</v>
+      </c>
+      <c r="C10" s="19"/>
+      <c r="D10" s="19"/>
+      <c r="E10" s="19"/>
+      <c r="F10" s="19"/>
+      <c r="G10" s="19"/>
+      <c r="H10" s="19"/>
+      <c r="I10" s="19"/>
+      <c r="J10" s="19"/>
+      <c r="K10" s="19"/>
+      <c r="L10" s="19"/>
+      <c r="M10" s="19"/>
+      <c r="N10" s="19"/>
+      <c r="O10" s="19"/>
+      <c r="P10" s="19"/>
+      <c r="Q10" s="19"/>
+      <c r="R10" s="19"/>
+      <c r="S10" s="19"/>
+      <c r="T10" s="19"/>
+      <c r="U10" s="19"/>
+      <c r="V10" s="19"/>
+      <c r="W10" s="19"/>
+      <c r="X10" s="19"/>
+      <c r="Y10" s="19"/>
+      <c r="Z10" s="19"/>
+      <c r="AF10" s="19"/>
+      <c r="AG10" s="19"/>
+      <c r="AH10" s="19"/>
+      <c r="AI10" s="19"/>
+      <c r="AJ10" s="19"/>
+    </row>
+    <row r="11" spans="1:36" x14ac:dyDescent="0.45">
+      <c r="A11" s="17" t="s">
+        <v>921</v>
+      </c>
+      <c r="B11" s="18">
+        <v>-159459</v>
+      </c>
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
+      <c r="G11" s="19"/>
+      <c r="H11" s="19"/>
+      <c r="I11" s="19"/>
+      <c r="J11" s="19"/>
+      <c r="K11" s="19"/>
+      <c r="L11" s="19"/>
+      <c r="M11" s="19"/>
+      <c r="N11" s="19"/>
+      <c r="O11" s="19"/>
+      <c r="P11" s="19"/>
+      <c r="Q11" s="19"/>
+      <c r="R11" s="19"/>
+      <c r="S11" s="19"/>
+      <c r="T11" s="19"/>
+      <c r="U11" s="19"/>
+      <c r="V11" s="19"/>
+      <c r="W11" s="19"/>
+      <c r="X11" s="19"/>
+      <c r="Y11" s="19"/>
+      <c r="Z11" s="19"/>
+      <c r="AA11" s="19"/>
+      <c r="AB11" s="19"/>
+      <c r="AC11" s="19"/>
+      <c r="AD11" s="19"/>
+      <c r="AE11" s="19"/>
+      <c r="AF11" s="19"/>
+      <c r="AG11" s="19"/>
+      <c r="AH11" s="19"/>
+      <c r="AI11" s="19"/>
+      <c r="AJ11" s="19"/>
+    </row>
+    <row r="12" spans="1:36" x14ac:dyDescent="0.45">
+      <c r="A12" s="17" t="s">
+        <v>1067</v>
+      </c>
+      <c r="B12" s="18">
+        <v>-39</v>
+      </c>
+    </row>
+    <row r="13" spans="1:36" x14ac:dyDescent="0.45">
+      <c r="A13" s="17" t="s">
+        <v>1068</v>
+      </c>
+      <c r="B13" s="18">
+        <v>-270</v>
+      </c>
+    </row>
+    <row r="14" spans="1:36" x14ac:dyDescent="0.45">
+      <c r="A14" s="17" t="s">
+        <v>1069</v>
+      </c>
+      <c r="B14" s="18">
+        <v>-1991</v>
+      </c>
+    </row>
+    <row r="15" spans="1:36" x14ac:dyDescent="0.45">
+      <c r="A15" s="17" t="s">
+        <v>1070</v>
+      </c>
+      <c r="B15" s="18">
+        <v>-16670</v>
+      </c>
+    </row>
+    <row r="16" spans="1:36" x14ac:dyDescent="0.45">
+      <c r="A16" s="17" t="s">
+        <v>1071</v>
+      </c>
+      <c r="B16" s="18">
+        <v>-160155</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A17" s="17" t="s">
+        <v>1086</v>
+      </c>
+      <c r="B17" s="18">
+        <v>-63</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A18" s="17" t="s">
+        <v>1087</v>
+      </c>
+      <c r="B18" s="18">
+        <v>-383</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A19" s="17" t="s">
+        <v>1088</v>
+      </c>
+      <c r="B19" s="18">
+        <v>-2695</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A20" s="17" t="s">
+        <v>1089</v>
+      </c>
+      <c r="B20" s="18">
+        <v>-19914</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A21" s="17" t="s">
+        <v>1090</v>
+      </c>
+      <c r="B21" s="18">
+        <v>-166442</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A22" s="17" t="s">
+        <v>1035</v>
+      </c>
+      <c r="B22" s="18">
+        <v>-138</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A23" s="17" t="s">
+        <v>1036</v>
+      </c>
+      <c r="B23" s="18">
+        <v>-627</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A24" s="17" t="s">
+        <v>1037</v>
+      </c>
+      <c r="B24" s="18">
+        <v>-3823</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A25" s="17" t="s">
+        <v>1038</v>
+      </c>
+      <c r="B25" s="18">
+        <v>-26902</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A26" s="17" t="s">
+        <v>1039</v>
+      </c>
+      <c r="B26" s="18">
+        <v>-200379</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A27" s="17" t="s">
+        <v>1091</v>
+      </c>
+      <c r="B27" s="18">
+        <v>-452</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A28" s="17" t="s">
+        <v>1092</v>
+      </c>
+      <c r="B28" s="18">
+        <v>-1374</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A29" s="17" t="s">
+        <v>1093</v>
+      </c>
+      <c r="B29" s="18">
+        <v>-6261</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A30" s="17" t="s">
+        <v>1094</v>
+      </c>
+      <c r="B30" s="18">
+        <v>-38186</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A31" s="17" t="s">
+        <v>1095</v>
+      </c>
+      <c r="B31" s="18">
+        <v>-268084</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A32" s="17" t="s">
+        <v>1040</v>
+      </c>
+      <c r="B32" s="18">
+        <v>-1375</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A33" s="17" t="s">
+        <v>1041</v>
+      </c>
+      <c r="B33" s="18">
+        <v>-4406</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A34" s="17" t="s">
+        <v>1042</v>
+      </c>
+      <c r="B34" s="18">
+        <v>-13522</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A35" s="17" t="s">
+        <v>1043</v>
+      </c>
+      <c r="B35" s="18">
+        <v>-62053</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A36" s="17" t="s">
+        <v>1044</v>
+      </c>
+      <c r="B36" s="18">
+        <v>-379630</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:AO23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="21" width="17.06640625" style="12" bestFit="1" customWidth="1"/>
+    <col min="17" max="36" width="17.06640625" style="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:41" x14ac:dyDescent="0.45">
@@ -5294,109 +5930,109 @@
         <v>35</v>
       </c>
       <c r="B1" s="12" t="s">
+        <v>1059</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>1060</v>
+      </c>
+      <c r="D1" s="12" t="s">
+        <v>1061</v>
+      </c>
+      <c r="E1" s="12" t="s">
+        <v>1062</v>
+      </c>
+      <c r="F1" s="12" t="s">
+        <v>920</v>
+      </c>
+      <c r="G1" s="12" t="s">
+        <v>1063</v>
+      </c>
+      <c r="H1" s="12" t="s">
+        <v>1064</v>
+      </c>
+      <c r="I1" s="12" t="s">
+        <v>1065</v>
+      </c>
+      <c r="J1" s="12" t="s">
+        <v>1066</v>
+      </c>
+      <c r="K1" s="12" t="s">
+        <v>921</v>
+      </c>
+      <c r="L1" s="12" t="s">
+        <v>1067</v>
+      </c>
+      <c r="M1" s="12" t="s">
+        <v>1068</v>
+      </c>
+      <c r="N1" s="12" t="s">
+        <v>1069</v>
+      </c>
+      <c r="O1" s="12" t="s">
+        <v>1070</v>
+      </c>
+      <c r="P1" s="12" t="s">
+        <v>1071</v>
+      </c>
+      <c r="Q1" s="12" t="s">
         <v>1086</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="R1" s="12" t="s">
         <v>1087</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="S1" s="12" t="s">
         <v>1088</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="T1" s="12" t="s">
         <v>1089</v>
       </c>
-      <c r="F1" s="12" t="s">
+      <c r="U1" s="12" t="s">
         <v>1090</v>
       </c>
-      <c r="G1" s="12" t="s">
+      <c r="V1" s="12" t="s">
         <v>1035</v>
       </c>
-      <c r="H1" s="12" t="s">
+      <c r="W1" s="12" t="s">
         <v>1036</v>
       </c>
-      <c r="I1" s="12" t="s">
+      <c r="X1" s="12" t="s">
         <v>1037</v>
       </c>
-      <c r="J1" s="12" t="s">
+      <c r="Y1" s="12" t="s">
         <v>1038</v>
       </c>
-      <c r="K1" s="12" t="s">
+      <c r="Z1" s="12" t="s">
         <v>1039</v>
       </c>
-      <c r="L1" s="12" t="s">
+      <c r="AA1" s="12" t="s">
         <v>1091</v>
       </c>
-      <c r="M1" s="12" t="s">
+      <c r="AB1" s="12" t="s">
         <v>1092</v>
       </c>
-      <c r="N1" s="12" t="s">
+      <c r="AC1" s="12" t="s">
         <v>1093</v>
       </c>
-      <c r="O1" s="12" t="s">
+      <c r="AD1" s="12" t="s">
         <v>1094</v>
       </c>
-      <c r="P1" s="12" t="s">
+      <c r="AE1" s="12" t="s">
         <v>1095</v>
       </c>
-      <c r="Q1" s="12" t="s">
+      <c r="AF1" s="12" t="s">
         <v>1040</v>
       </c>
-      <c r="R1" s="12" t="s">
+      <c r="AG1" s="12" t="s">
         <v>1041</v>
       </c>
-      <c r="S1" s="12" t="s">
+      <c r="AH1" s="12" t="s">
         <v>1042</v>
       </c>
-      <c r="T1" s="12" t="s">
+      <c r="AI1" s="12" t="s">
         <v>1043</v>
       </c>
-      <c r="U1" s="12" t="s">
+      <c r="AJ1" s="12" t="s">
         <v>1044</v>
-      </c>
-      <c r="V1" s="12" t="s">
-        <v>1059</v>
-      </c>
-      <c r="W1" s="12" t="s">
-        <v>1060</v>
-      </c>
-      <c r="X1" s="12" t="s">
-        <v>1061</v>
-      </c>
-      <c r="Y1" s="12" t="s">
-        <v>1062</v>
-      </c>
-      <c r="Z1" s="12" t="s">
-        <v>920</v>
-      </c>
-      <c r="AA1" s="12" t="s">
-        <v>1063</v>
-      </c>
-      <c r="AB1" s="12" t="s">
-        <v>1064</v>
-      </c>
-      <c r="AC1" s="12" t="s">
-        <v>1065</v>
-      </c>
-      <c r="AD1" s="12" t="s">
-        <v>1066</v>
-      </c>
-      <c r="AE1" s="12" t="s">
-        <v>921</v>
-      </c>
-      <c r="AF1" s="12" t="s">
-        <v>1067</v>
-      </c>
-      <c r="AG1" s="12" t="s">
-        <v>1068</v>
-      </c>
-      <c r="AH1" s="12" t="s">
-        <v>1069</v>
-      </c>
-      <c r="AI1" s="12" t="s">
-        <v>1070</v>
-      </c>
-      <c r="AJ1" s="12" t="s">
-        <v>1071</v>
       </c>
     </row>
     <row r="2" spans="1:41" x14ac:dyDescent="0.45">
@@ -5519,109 +6155,109 @@
         <v>46</v>
       </c>
       <c r="B3" s="14">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="C3" s="14">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="D3" s="14">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="E3" s="14">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="F3" s="14">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="G3" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="H3" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="I3" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="J3" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="K3" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="L3" s="14">
+        <v>8.6400000000000001E-7</v>
+      </c>
+      <c r="M3" s="14">
+        <v>8.6400000000000001E-7</v>
+      </c>
+      <c r="N3" s="14">
+        <v>8.6400000000000001E-7</v>
+      </c>
+      <c r="O3" s="14">
+        <v>8.6400000000000001E-7</v>
+      </c>
+      <c r="P3" s="14">
+        <v>8.6400000000000001E-7</v>
+      </c>
+      <c r="Q3" s="14">
         <v>8.6400000000000003E-6</v>
       </c>
-      <c r="C3" s="14">
+      <c r="R3" s="14">
         <v>8.6400000000000003E-6</v>
       </c>
-      <c r="D3" s="14">
+      <c r="S3" s="14">
         <v>8.6400000000000003E-6</v>
       </c>
-      <c r="E3" s="14">
+      <c r="T3" s="14">
         <v>8.6400000000000003E-6</v>
       </c>
-      <c r="F3" s="14">
+      <c r="U3" s="14">
         <v>8.6400000000000003E-6</v>
       </c>
-      <c r="G3" s="14">
+      <c r="V3" s="14">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="H3" s="14">
+      <c r="W3" s="14">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="I3" s="14">
+      <c r="X3" s="14">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="J3" s="14">
+      <c r="Y3" s="14">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="K3" s="14">
+      <c r="Z3" s="14">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="L3" s="14">
+      <c r="AA3" s="14">
         <v>8.6399999999999997E-4</v>
       </c>
-      <c r="M3" s="14">
+      <c r="AB3" s="14">
         <v>8.6399999999999997E-4</v>
       </c>
-      <c r="N3" s="14">
+      <c r="AC3" s="14">
         <v>8.6399999999999997E-4</v>
       </c>
-      <c r="O3" s="14">
+      <c r="AD3" s="14">
         <v>8.6399999999999997E-4</v>
       </c>
-      <c r="P3" s="14">
+      <c r="AE3" s="14">
         <v>8.6399999999999997E-4</v>
       </c>
-      <c r="Q3" s="14">
+      <c r="AF3" s="14">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="R3" s="14">
+      <c r="AG3" s="14">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="S3" s="14">
+      <c r="AH3" s="14">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="T3" s="14">
+      <c r="AI3" s="14">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="U3" s="14">
+      <c r="AJ3" s="14">
         <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="V3" s="14">
-        <v>8.6399999999999999E-9</v>
-      </c>
-      <c r="W3" s="14">
-        <v>8.6399999999999999E-9</v>
-      </c>
-      <c r="X3" s="14">
-        <v>8.6399999999999999E-9</v>
-      </c>
-      <c r="Y3" s="14">
-        <v>8.6399999999999999E-9</v>
-      </c>
-      <c r="Z3" s="14">
-        <v>8.6399999999999999E-9</v>
-      </c>
-      <c r="AA3" s="11">
-        <v>8.6400000000000006E-8</v>
-      </c>
-      <c r="AB3" s="11">
-        <v>8.6400000000000006E-8</v>
-      </c>
-      <c r="AC3" s="11">
-        <v>8.6400000000000006E-8</v>
-      </c>
-      <c r="AD3" s="11">
-        <v>8.6400000000000006E-8</v>
-      </c>
-      <c r="AE3" s="11">
-        <v>8.6400000000000006E-8</v>
-      </c>
-      <c r="AF3" s="14">
-        <v>8.6400000000000001E-7</v>
-      </c>
-      <c r="AG3" s="14">
-        <v>8.6400000000000001E-7</v>
-      </c>
-      <c r="AH3" s="14">
-        <v>8.6400000000000001E-7</v>
-      </c>
-      <c r="AI3" s="14">
-        <v>8.6400000000000001E-7</v>
-      </c>
-      <c r="AJ3" s="14">
-        <v>8.6400000000000001E-7</v>
       </c>
       <c r="AK3" s="13"/>
       <c r="AL3" s="13"/>
@@ -5749,109 +6385,109 @@
         <v>50</v>
       </c>
       <c r="B5" s="14">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="C5" s="14">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="D5" s="14">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="E5" s="14">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="F5" s="14">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="G5" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="H5" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="I5" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="J5" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="K5" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="L5" s="14">
+        <v>8.6400000000000001E-7</v>
+      </c>
+      <c r="M5" s="14">
+        <v>8.6400000000000001E-7</v>
+      </c>
+      <c r="N5" s="14">
+        <v>8.6400000000000001E-7</v>
+      </c>
+      <c r="O5" s="14">
+        <v>8.6400000000000001E-7</v>
+      </c>
+      <c r="P5" s="14">
+        <v>8.6400000000000001E-7</v>
+      </c>
+      <c r="Q5" s="14">
         <v>8.6400000000000003E-6</v>
       </c>
-      <c r="C5" s="14">
+      <c r="R5" s="14">
         <v>8.6400000000000003E-6</v>
       </c>
-      <c r="D5" s="14">
+      <c r="S5" s="14">
         <v>8.6400000000000003E-6</v>
       </c>
-      <c r="E5" s="14">
+      <c r="T5" s="14">
         <v>8.6400000000000003E-6</v>
       </c>
-      <c r="F5" s="14">
+      <c r="U5" s="14">
         <v>8.6400000000000003E-6</v>
       </c>
-      <c r="G5" s="14">
+      <c r="V5" s="14">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="H5" s="14">
+      <c r="W5" s="14">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="I5" s="14">
+      <c r="X5" s="14">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="J5" s="14">
+      <c r="Y5" s="14">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="K5" s="14">
+      <c r="Z5" s="14">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="L5" s="14">
+      <c r="AA5" s="14">
         <v>8.6399999999999997E-4</v>
       </c>
-      <c r="M5" s="14">
+      <c r="AB5" s="14">
         <v>8.6399999999999997E-4</v>
       </c>
-      <c r="N5" s="14">
+      <c r="AC5" s="14">
         <v>8.6399999999999997E-4</v>
       </c>
-      <c r="O5" s="14">
+      <c r="AD5" s="14">
         <v>8.6399999999999997E-4</v>
       </c>
-      <c r="P5" s="14">
+      <c r="AE5" s="14">
         <v>8.6399999999999997E-4</v>
       </c>
-      <c r="Q5" s="14">
+      <c r="AF5" s="14">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="R5" s="14">
+      <c r="AG5" s="14">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="S5" s="14">
+      <c r="AH5" s="14">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="T5" s="14">
+      <c r="AI5" s="14">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="U5" s="14">
+      <c r="AJ5" s="14">
         <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="V5" s="14">
-        <v>8.6399999999999999E-9</v>
-      </c>
-      <c r="W5" s="14">
-        <v>8.6399999999999999E-9</v>
-      </c>
-      <c r="X5" s="14">
-        <v>8.6399999999999999E-9</v>
-      </c>
-      <c r="Y5" s="14">
-        <v>8.6399999999999999E-9</v>
-      </c>
-      <c r="Z5" s="14">
-        <v>8.6399999999999999E-9</v>
-      </c>
-      <c r="AA5" s="11">
-        <v>8.6400000000000006E-8</v>
-      </c>
-      <c r="AB5" s="11">
-        <v>8.6400000000000006E-8</v>
-      </c>
-      <c r="AC5" s="11">
-        <v>8.6400000000000006E-8</v>
-      </c>
-      <c r="AD5" s="11">
-        <v>8.6400000000000006E-8</v>
-      </c>
-      <c r="AE5" s="11">
-        <v>8.6400000000000006E-8</v>
-      </c>
-      <c r="AF5" s="14">
-        <v>8.6400000000000001E-7</v>
-      </c>
-      <c r="AG5" s="14">
-        <v>8.6400000000000001E-7</v>
-      </c>
-      <c r="AH5" s="14">
-        <v>8.6400000000000001E-7</v>
-      </c>
-      <c r="AI5" s="14">
-        <v>8.6400000000000001E-7</v>
-      </c>
-      <c r="AJ5" s="14">
-        <v>8.6400000000000001E-7</v>
       </c>
       <c r="AK5" s="13"/>
       <c r="AL5" s="13"/>
@@ -6094,109 +6730,109 @@
         <v>55</v>
       </c>
       <c r="B8" s="14">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="C8" s="14">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="D8" s="14">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="E8" s="14">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="F8" s="14">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="G8" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="H8" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="I8" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="J8" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="K8" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="L8" s="14">
+        <v>8.6400000000000001E-7</v>
+      </c>
+      <c r="M8" s="14">
+        <v>8.6400000000000001E-7</v>
+      </c>
+      <c r="N8" s="14">
+        <v>8.6400000000000001E-7</v>
+      </c>
+      <c r="O8" s="14">
+        <v>8.6400000000000001E-7</v>
+      </c>
+      <c r="P8" s="14">
+        <v>8.6400000000000001E-7</v>
+      </c>
+      <c r="Q8" s="14">
         <v>8.6400000000000003E-6</v>
       </c>
-      <c r="C8" s="14">
+      <c r="R8" s="14">
         <v>8.6400000000000003E-6</v>
       </c>
-      <c r="D8" s="14">
+      <c r="S8" s="14">
         <v>8.6400000000000003E-6</v>
       </c>
-      <c r="E8" s="14">
+      <c r="T8" s="14">
         <v>8.6400000000000003E-6</v>
       </c>
-      <c r="F8" s="14">
+      <c r="U8" s="14">
         <v>8.6400000000000003E-6</v>
       </c>
-      <c r="G8" s="14">
+      <c r="V8" s="14">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="H8" s="14">
+      <c r="W8" s="14">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="I8" s="14">
+      <c r="X8" s="14">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="J8" s="14">
+      <c r="Y8" s="14">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="K8" s="14">
+      <c r="Z8" s="14">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="L8" s="14">
+      <c r="AA8" s="14">
         <v>8.6399999999999997E-4</v>
       </c>
-      <c r="M8" s="14">
+      <c r="AB8" s="14">
         <v>8.6399999999999997E-4</v>
       </c>
-      <c r="N8" s="14">
+      <c r="AC8" s="14">
         <v>8.6399999999999997E-4</v>
       </c>
-      <c r="O8" s="14">
+      <c r="AD8" s="14">
         <v>8.6399999999999997E-4</v>
       </c>
-      <c r="P8" s="14">
+      <c r="AE8" s="14">
         <v>8.6399999999999997E-4</v>
       </c>
-      <c r="Q8" s="14">
+      <c r="AF8" s="14">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="R8" s="14">
+      <c r="AG8" s="14">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="S8" s="14">
+      <c r="AH8" s="14">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="T8" s="14">
+      <c r="AI8" s="14">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="U8" s="14">
+      <c r="AJ8" s="14">
         <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="V8" s="14">
-        <v>8.6399999999999999E-9</v>
-      </c>
-      <c r="W8" s="14">
-        <v>8.6399999999999999E-9</v>
-      </c>
-      <c r="X8" s="14">
-        <v>8.6399999999999999E-9</v>
-      </c>
-      <c r="Y8" s="14">
-        <v>8.6399999999999999E-9</v>
-      </c>
-      <c r="Z8" s="14">
-        <v>8.6399999999999999E-9</v>
-      </c>
-      <c r="AA8" s="11">
-        <v>8.6400000000000006E-8</v>
-      </c>
-      <c r="AB8" s="11">
-        <v>8.6400000000000006E-8</v>
-      </c>
-      <c r="AC8" s="11">
-        <v>8.6400000000000006E-8</v>
-      </c>
-      <c r="AD8" s="11">
-        <v>8.6400000000000006E-8</v>
-      </c>
-      <c r="AE8" s="11">
-        <v>8.6400000000000006E-8</v>
-      </c>
-      <c r="AF8" s="14">
-        <v>8.6400000000000001E-7</v>
-      </c>
-      <c r="AG8" s="14">
-        <v>8.6400000000000001E-7</v>
-      </c>
-      <c r="AH8" s="14">
-        <v>8.6400000000000001E-7</v>
-      </c>
-      <c r="AI8" s="14">
-        <v>8.6400000000000001E-7</v>
-      </c>
-      <c r="AJ8" s="14">
-        <v>8.6400000000000001E-7</v>
       </c>
       <c r="AK8" s="13"/>
       <c r="AL8" s="13"/>
@@ -6324,109 +6960,109 @@
         <v>57</v>
       </c>
       <c r="B10" s="14">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="C10" s="14">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="D10" s="14">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="E10" s="14">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="F10" s="14">
+        <v>8.6399999999999999E-9</v>
+      </c>
+      <c r="G10" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="H10" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="I10" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="J10" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="K10" s="11">
+        <v>8.6400000000000006E-8</v>
+      </c>
+      <c r="L10" s="14">
+        <v>8.6400000000000001E-7</v>
+      </c>
+      <c r="M10" s="14">
+        <v>8.6400000000000001E-7</v>
+      </c>
+      <c r="N10" s="14">
+        <v>8.6400000000000001E-7</v>
+      </c>
+      <c r="O10" s="14">
+        <v>8.6400000000000001E-7</v>
+      </c>
+      <c r="P10" s="14">
+        <v>8.6400000000000001E-7</v>
+      </c>
+      <c r="Q10" s="14">
         <v>8.6400000000000003E-6</v>
       </c>
-      <c r="C10" s="14">
+      <c r="R10" s="14">
         <v>8.6400000000000003E-6</v>
       </c>
-      <c r="D10" s="14">
+      <c r="S10" s="14">
         <v>8.6400000000000003E-6</v>
       </c>
-      <c r="E10" s="14">
+      <c r="T10" s="14">
         <v>8.6400000000000003E-6</v>
       </c>
-      <c r="F10" s="14">
+      <c r="U10" s="14">
         <v>8.6400000000000003E-6</v>
       </c>
-      <c r="G10" s="14">
+      <c r="V10" s="14">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="H10" s="14">
+      <c r="W10" s="14">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="I10" s="14">
+      <c r="X10" s="14">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="J10" s="14">
+      <c r="Y10" s="14">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="K10" s="14">
+      <c r="Z10" s="14">
         <v>8.6399999999999999E-5</v>
       </c>
-      <c r="L10" s="14">
+      <c r="AA10" s="14">
         <v>8.6399999999999997E-4</v>
       </c>
-      <c r="M10" s="14">
+      <c r="AB10" s="14">
         <v>8.6399999999999997E-4</v>
       </c>
-      <c r="N10" s="14">
+      <c r="AC10" s="14">
         <v>8.6399999999999997E-4</v>
       </c>
-      <c r="O10" s="14">
+      <c r="AD10" s="14">
         <v>8.6399999999999997E-4</v>
       </c>
-      <c r="P10" s="14">
+      <c r="AE10" s="14">
         <v>8.6399999999999997E-4</v>
       </c>
-      <c r="Q10" s="14">
+      <c r="AF10" s="14">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="R10" s="14">
+      <c r="AG10" s="14">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="S10" s="14">
+      <c r="AH10" s="14">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="T10" s="14">
+      <c r="AI10" s="14">
         <v>8.6400000000000001E-3</v>
       </c>
-      <c r="U10" s="14">
+      <c r="AJ10" s="14">
         <v>8.6400000000000001E-3</v>
-      </c>
-      <c r="V10" s="14">
-        <v>8.6399999999999999E-9</v>
-      </c>
-      <c r="W10" s="14">
-        <v>8.6399999999999999E-9</v>
-      </c>
-      <c r="X10" s="14">
-        <v>8.6399999999999999E-9</v>
-      </c>
-      <c r="Y10" s="14">
-        <v>8.6399999999999999E-9</v>
-      </c>
-      <c r="Z10" s="14">
-        <v>8.6399999999999999E-9</v>
-      </c>
-      <c r="AA10" s="11">
-        <v>8.6400000000000006E-8</v>
-      </c>
-      <c r="AB10" s="11">
-        <v>8.6400000000000006E-8</v>
-      </c>
-      <c r="AC10" s="11">
-        <v>8.6400000000000006E-8</v>
-      </c>
-      <c r="AD10" s="11">
-        <v>8.6400000000000006E-8</v>
-      </c>
-      <c r="AE10" s="11">
-        <v>8.6400000000000006E-8</v>
-      </c>
-      <c r="AF10" s="14">
-        <v>8.6400000000000001E-7</v>
-      </c>
-      <c r="AG10" s="14">
-        <v>8.6400000000000001E-7</v>
-      </c>
-      <c r="AH10" s="14">
-        <v>8.6400000000000001E-7</v>
-      </c>
-      <c r="AI10" s="14">
-        <v>8.6400000000000001E-7</v>
-      </c>
-      <c r="AJ10" s="14">
-        <v>8.6400000000000001E-7</v>
       </c>
       <c r="AK10" s="13"/>
       <c r="AL10" s="13"/>
@@ -6550,174 +7186,194 @@
       <c r="AO11" s="13"/>
     </row>
     <row r="14" spans="1:41" x14ac:dyDescent="0.45">
-      <c r="B14" s="13"/>
-      <c r="C14" s="13"/>
-      <c r="D14" s="13"/>
-      <c r="E14" s="13"/>
-      <c r="F14" s="13"/>
-      <c r="G14" s="13"/>
-      <c r="H14" s="13"/>
-      <c r="I14" s="13"/>
-      <c r="J14" s="13"/>
-      <c r="K14" s="13"/>
-      <c r="L14" s="13"/>
-      <c r="M14" s="13"/>
-      <c r="N14" s="13"/>
-      <c r="O14" s="13"/>
-      <c r="P14" s="13"/>
+      <c r="Q14" s="13"/>
+      <c r="R14" s="13"/>
+      <c r="S14" s="13"/>
+      <c r="T14" s="13"/>
+      <c r="U14" s="13"/>
+      <c r="V14" s="13"/>
+      <c r="W14" s="13"/>
+      <c r="X14" s="13"/>
+      <c r="Y14" s="13"/>
+      <c r="Z14" s="13"/>
+      <c r="AA14" s="13"/>
+      <c r="AB14" s="13"/>
+      <c r="AC14" s="13"/>
+      <c r="AD14" s="13"/>
+      <c r="AE14" s="13"/>
     </row>
     <row r="15" spans="1:41" x14ac:dyDescent="0.45">
-      <c r="B15" s="14"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="14"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="11"/>
-      <c r="H15" s="11"/>
-      <c r="I15" s="11"/>
-      <c r="J15" s="11"/>
-      <c r="K15" s="11"/>
-      <c r="L15" s="14"/>
-      <c r="M15" s="14"/>
-      <c r="N15" s="14"/>
-      <c r="O15" s="14"/>
-      <c r="P15" s="14"/>
+      <c r="B15" s="13"/>
+      <c r="Q15" s="14"/>
+      <c r="R15" s="14"/>
+      <c r="S15" s="14"/>
+      <c r="T15" s="14"/>
+      <c r="U15" s="14"/>
+      <c r="V15" s="11"/>
+      <c r="W15" s="11"/>
+      <c r="X15" s="11"/>
+      <c r="Y15" s="11"/>
+      <c r="Z15" s="11"/>
+      <c r="AA15" s="14"/>
+      <c r="AB15" s="14"/>
+      <c r="AC15" s="14"/>
+      <c r="AD15" s="14"/>
+      <c r="AE15" s="14"/>
     </row>
     <row r="16" spans="1:41" x14ac:dyDescent="0.45">
-      <c r="B16" s="13"/>
-      <c r="C16" s="13"/>
-      <c r="D16" s="13"/>
-      <c r="E16" s="13"/>
-      <c r="F16" s="13"/>
-      <c r="G16" s="13"/>
-      <c r="H16" s="13"/>
-      <c r="I16" s="13"/>
-      <c r="J16" s="13"/>
-      <c r="K16" s="13"/>
-      <c r="L16" s="13"/>
-      <c r="M16" s="13"/>
-      <c r="N16" s="13"/>
-      <c r="O16" s="13"/>
-      <c r="P16" s="13"/>
-    </row>
-    <row r="17" spans="2:16" x14ac:dyDescent="0.45">
-      <c r="B17" s="14"/>
-      <c r="C17" s="14"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="14"/>
-      <c r="F17" s="14"/>
-      <c r="G17" s="11"/>
-      <c r="H17" s="11"/>
-      <c r="I17" s="11"/>
-      <c r="J17" s="11"/>
-      <c r="K17" s="11"/>
-      <c r="L17" s="14"/>
-      <c r="M17" s="14"/>
-      <c r="N17" s="14"/>
-      <c r="O17" s="14"/>
-      <c r="P17" s="14"/>
-    </row>
-    <row r="18" spans="2:16" x14ac:dyDescent="0.45">
-      <c r="B18" s="13"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="13"/>
-      <c r="F18" s="13"/>
-      <c r="G18" s="13"/>
-      <c r="H18" s="13"/>
-      <c r="I18" s="13"/>
-      <c r="J18" s="13"/>
-      <c r="K18" s="13"/>
-      <c r="L18" s="13"/>
-      <c r="M18" s="13"/>
-      <c r="N18" s="13"/>
-      <c r="O18" s="13"/>
-      <c r="P18" s="13"/>
-    </row>
-    <row r="19" spans="2:16" x14ac:dyDescent="0.45">
-      <c r="B19" s="13"/>
-      <c r="C19" s="13"/>
-      <c r="D19" s="13"/>
-      <c r="E19" s="13"/>
-      <c r="F19" s="13"/>
-      <c r="G19" s="13"/>
-      <c r="H19" s="13"/>
-      <c r="I19" s="13"/>
-      <c r="J19" s="13"/>
-      <c r="K19" s="13"/>
-      <c r="L19" s="13"/>
-      <c r="M19" s="13"/>
-      <c r="N19" s="13"/>
-      <c r="O19" s="13"/>
-      <c r="P19" s="13"/>
-    </row>
-    <row r="20" spans="2:16" x14ac:dyDescent="0.45">
-      <c r="B20" s="14"/>
-      <c r="C20" s="14"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="14"/>
-      <c r="F20" s="14"/>
-      <c r="G20" s="11"/>
-      <c r="H20" s="11"/>
-      <c r="I20" s="11"/>
-      <c r="J20" s="11"/>
-      <c r="K20" s="11"/>
-      <c r="L20" s="14"/>
-      <c r="M20" s="14"/>
-      <c r="N20" s="14"/>
-      <c r="O20" s="14"/>
-      <c r="P20" s="14"/>
-    </row>
-    <row r="21" spans="2:16" x14ac:dyDescent="0.45">
-      <c r="B21" s="13"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="13"/>
-      <c r="E21" s="13"/>
-      <c r="F21" s="13"/>
-      <c r="G21" s="13"/>
-      <c r="H21" s="13"/>
-      <c r="I21" s="13"/>
-      <c r="J21" s="13"/>
-      <c r="K21" s="13"/>
-      <c r="L21" s="13"/>
-      <c r="M21" s="13"/>
-      <c r="N21" s="13"/>
-      <c r="O21" s="13"/>
-      <c r="P21" s="13"/>
-    </row>
-    <row r="22" spans="2:16" x14ac:dyDescent="0.45">
-      <c r="B22" s="14"/>
-      <c r="C22" s="14"/>
-      <c r="D22" s="14"/>
-      <c r="E22" s="14"/>
-      <c r="F22" s="14"/>
-      <c r="G22" s="11"/>
-      <c r="H22" s="11"/>
-      <c r="I22" s="11"/>
-      <c r="J22" s="11"/>
-      <c r="K22" s="11"/>
-      <c r="L22" s="14"/>
-      <c r="M22" s="14"/>
-      <c r="N22" s="14"/>
-      <c r="O22" s="14"/>
-      <c r="P22" s="14"/>
-    </row>
-    <row r="23" spans="2:16" x14ac:dyDescent="0.45">
-      <c r="B23" s="13"/>
-      <c r="C23" s="13"/>
-      <c r="D23" s="13"/>
-      <c r="E23" s="13"/>
-      <c r="F23" s="13"/>
-      <c r="G23" s="13"/>
-      <c r="H23" s="13"/>
-      <c r="I23" s="13"/>
-      <c r="J23" s="13"/>
-      <c r="K23" s="13"/>
-      <c r="L23" s="13"/>
-      <c r="M23" s="13"/>
-      <c r="N23" s="13"/>
-      <c r="O23" s="13"/>
-      <c r="P23" s="13"/>
+      <c r="Q16" s="13"/>
+      <c r="R16" s="13"/>
+      <c r="S16" s="13"/>
+      <c r="T16" s="13"/>
+      <c r="U16" s="13"/>
+      <c r="V16" s="13"/>
+      <c r="W16" s="13"/>
+      <c r="X16" s="13"/>
+      <c r="Y16" s="13"/>
+      <c r="Z16" s="13"/>
+      <c r="AA16" s="13"/>
+      <c r="AB16" s="13"/>
+      <c r="AC16" s="13"/>
+      <c r="AD16" s="13"/>
+      <c r="AE16" s="13"/>
+    </row>
+    <row r="17" spans="2:36" x14ac:dyDescent="0.45">
+      <c r="B17" s="17"/>
+      <c r="C17" s="17"/>
+      <c r="D17" s="17"/>
+      <c r="E17" s="17"/>
+      <c r="F17" s="17"/>
+      <c r="G17" s="17"/>
+      <c r="H17" s="17"/>
+      <c r="I17" s="17"/>
+      <c r="J17" s="17"/>
+      <c r="K17" s="17"/>
+      <c r="L17" s="17"/>
+      <c r="M17" s="17"/>
+      <c r="N17" s="17"/>
+      <c r="O17" s="17"/>
+      <c r="P17" s="17"/>
+      <c r="Q17" s="17"/>
+      <c r="R17" s="17"/>
+      <c r="S17" s="17"/>
+      <c r="T17" s="17"/>
+      <c r="U17" s="17"/>
+      <c r="V17" s="17"/>
+      <c r="W17" s="17"/>
+      <c r="X17" s="17"/>
+      <c r="Y17" s="17"/>
+      <c r="Z17" s="17"/>
+      <c r="AA17" s="17"/>
+      <c r="AB17" s="17"/>
+      <c r="AC17" s="17"/>
+      <c r="AD17" s="17"/>
+      <c r="AE17" s="17"/>
+      <c r="AF17" s="17"/>
+      <c r="AG17" s="17"/>
+      <c r="AH17" s="17"/>
+      <c r="AI17" s="17"/>
+      <c r="AJ17" s="17"/>
+    </row>
+    <row r="18" spans="2:36" x14ac:dyDescent="0.45">
+      <c r="Q18" s="13"/>
+      <c r="R18" s="13"/>
+      <c r="S18" s="13"/>
+      <c r="T18" s="13"/>
+      <c r="U18" s="13"/>
+      <c r="V18" s="13"/>
+      <c r="W18" s="13"/>
+      <c r="X18" s="13"/>
+      <c r="Y18" s="13"/>
+      <c r="Z18" s="13"/>
+      <c r="AA18" s="13"/>
+      <c r="AB18" s="13"/>
+      <c r="AC18" s="13"/>
+      <c r="AD18" s="13"/>
+      <c r="AE18" s="13"/>
+    </row>
+    <row r="19" spans="2:36" x14ac:dyDescent="0.45">
+      <c r="Q19" s="13"/>
+      <c r="R19" s="13"/>
+      <c r="S19" s="13"/>
+      <c r="T19" s="13"/>
+      <c r="U19" s="13"/>
+      <c r="V19" s="13"/>
+      <c r="W19" s="13"/>
+      <c r="X19" s="13"/>
+      <c r="Y19" s="13"/>
+      <c r="Z19" s="13"/>
+      <c r="AA19" s="13"/>
+      <c r="AB19" s="13"/>
+      <c r="AC19" s="13"/>
+      <c r="AD19" s="13"/>
+      <c r="AE19" s="13"/>
+    </row>
+    <row r="20" spans="2:36" x14ac:dyDescent="0.45">
+      <c r="C20" s="12"/>
+      <c r="D20" s="12"/>
+      <c r="E20" s="12"/>
+      <c r="F20" s="12"/>
+      <c r="G20" s="12"/>
+      <c r="H20" s="12"/>
+      <c r="I20" s="12"/>
+      <c r="J20" s="12"/>
+      <c r="K20" s="12"/>
+      <c r="L20" s="12"/>
+      <c r="M20" s="12"/>
+      <c r="N20" s="12"/>
+      <c r="O20" s="12"/>
+      <c r="P20" s="12"/>
+    </row>
+    <row r="21" spans="2:36" x14ac:dyDescent="0.45">
+      <c r="Q21" s="13"/>
+      <c r="R21" s="13"/>
+      <c r="S21" s="13"/>
+      <c r="T21" s="13"/>
+      <c r="U21" s="13"/>
+      <c r="V21" s="13"/>
+      <c r="W21" s="13"/>
+      <c r="X21" s="13"/>
+      <c r="Y21" s="13"/>
+      <c r="Z21" s="13"/>
+      <c r="AA21" s="13"/>
+      <c r="AB21" s="13"/>
+      <c r="AC21" s="13"/>
+      <c r="AD21" s="13"/>
+      <c r="AE21" s="13"/>
+    </row>
+    <row r="22" spans="2:36" x14ac:dyDescent="0.45">
+      <c r="Q22" s="14"/>
+      <c r="R22" s="14"/>
+      <c r="S22" s="14"/>
+      <c r="T22" s="14"/>
+      <c r="U22" s="14"/>
+      <c r="V22" s="11"/>
+      <c r="W22" s="11"/>
+      <c r="X22" s="11"/>
+      <c r="Y22" s="11"/>
+      <c r="Z22" s="11"/>
+      <c r="AA22" s="14"/>
+      <c r="AB22" s="14"/>
+      <c r="AC22" s="14"/>
+      <c r="AD22" s="14"/>
+      <c r="AE22" s="14"/>
+    </row>
+    <row r="23" spans="2:36" x14ac:dyDescent="0.45">
+      <c r="Q23" s="13"/>
+      <c r="R23" s="13"/>
+      <c r="S23" s="13"/>
+      <c r="T23" s="13"/>
+      <c r="U23" s="13"/>
+      <c r="V23" s="13"/>
+      <c r="W23" s="13"/>
+      <c r="X23" s="13"/>
+      <c r="Y23" s="13"/>
+      <c r="Z23" s="13"/>
+      <c r="AA23" s="13"/>
+      <c r="AB23" s="13"/>
+      <c r="AC23" s="13"/>
+      <c r="AD23" s="13"/>
+      <c r="AE23" s="13"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6725,7 +7381,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:BZ364"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -26963,7 +27619,7 @@
         <v>70</v>
       </c>
       <c r="J2">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K2">
         <v>1</v>
@@ -26997,8 +27653,8 @@
       <c r="I3">
         <v>70</v>
       </c>
-      <c r="J3">
-        <v>3</v>
+      <c r="J3" s="12">
+        <v>0</v>
       </c>
       <c r="K3">
         <v>2</v>
@@ -27032,8 +27688,8 @@
       <c r="I4">
         <v>70</v>
       </c>
-      <c r="J4">
-        <v>3</v>
+      <c r="J4" s="12">
+        <v>0</v>
       </c>
       <c r="K4">
         <v>3</v>
@@ -27067,8 +27723,8 @@
       <c r="I5">
         <v>70</v>
       </c>
-      <c r="J5">
-        <v>3</v>
+      <c r="J5" s="12">
+        <v>0</v>
       </c>
       <c r="K5">
         <v>4</v>
@@ -27102,8 +27758,8 @@
       <c r="I6">
         <v>70</v>
       </c>
-      <c r="J6">
-        <v>3</v>
+      <c r="J6" s="12">
+        <v>0</v>
       </c>
       <c r="K6">
         <v>5</v>
@@ -45937,7 +46593,7 @@
         <v>892</v>
       </c>
       <c r="B2">
-        <v>1E-3</v>
+        <v>0.01</v>
       </c>
       <c r="C2" t="s">
         <v>893</v>

</xml_diff>

<commit_message>
Set a wide range of pumping rates for sustainable yield maximization
</commit_message>
<xml_diff>
--- a/assets/3D/sust yield server/setup.xlsx
+++ b/assets/3D/sust yield server/setup.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmarinriver\Projects\ConfinedLab\assets\3D\sust yield server\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmarinriver\Projects\ConfinedLab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7403F4B1-8A79-44A4-829C-6CC146A0529B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5FCA7BF-8163-4B47-9558-247109C6C449}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" firstSheet="3" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15796" firstSheet="3" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="grid" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2541" uniqueCount="1193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2542" uniqueCount="1194">
   <si>
     <t>nlay</t>
   </si>
@@ -3626,13 +3626,16 @@
   </si>
   <si>
     <t>q_init</t>
+  </si>
+  <si>
+    <t>qv_11</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3679,6 +3682,12 @@
     </font>
     <font>
       <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -4402,7 +4411,7 @@
     <col min="10" max="10" width="10.9296875" style="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A1" s="12" t="s">
         <v>884</v>
       </c>
@@ -4442,8 +4451,11 @@
       <c r="M1" s="12" t="s">
         <v>918</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N1" s="12" t="s">
+        <v>1193</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A2" s="12" t="s">
         <v>886</v>
       </c>
@@ -4483,8 +4495,11 @@
       <c r="M2" s="12">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N2" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A3" s="12" t="s">
         <v>886</v>
       </c>
@@ -4495,37 +4510,40 @@
         <v>0</v>
       </c>
       <c r="D3" s="12">
+        <v>-100</v>
+      </c>
+      <c r="E3" s="12">
         <v>-200</v>
       </c>
-      <c r="E3" s="12">
+      <c r="F3" s="12">
         <v>-1000</v>
       </c>
-      <c r="F3" s="12">
+      <c r="G3" s="12">
         <v>-2000</v>
       </c>
-      <c r="G3" s="12">
+      <c r="H3" s="12">
         <v>-20000</v>
       </c>
-      <c r="H3" s="12">
+      <c r="I3" s="12">
         <v>-100000</v>
       </c>
-      <c r="I3" s="12">
+      <c r="J3" s="12">
         <v>-200000</v>
       </c>
-      <c r="J3" s="12">
+      <c r="K3" s="12">
         <v>-600000</v>
       </c>
-      <c r="K3" s="12">
+      <c r="L3" s="12">
         <v>-1200000</v>
       </c>
-      <c r="L3" s="12">
+      <c r="M3" s="12">
         <v>-2400000</v>
       </c>
-      <c r="M3" s="12">
+      <c r="N3" s="12">
         <v>-4800000</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A4" s="12" t="s">
         <v>886</v>
       </c>
@@ -4536,37 +4554,40 @@
         <v>0</v>
       </c>
       <c r="D4" s="12">
+        <v>-100</v>
+      </c>
+      <c r="E4" s="12">
         <v>-200</v>
       </c>
-      <c r="E4" s="12">
+      <c r="F4" s="12">
         <v>-1000</v>
       </c>
-      <c r="F4" s="12">
+      <c r="G4" s="12">
         <v>-2000</v>
       </c>
-      <c r="G4" s="12">
+      <c r="H4" s="12">
         <v>-20000</v>
       </c>
-      <c r="H4" s="12">
+      <c r="I4" s="12">
         <v>-100000</v>
       </c>
-      <c r="I4" s="12">
+      <c r="J4" s="12">
         <v>-200000</v>
       </c>
-      <c r="J4" s="12">
+      <c r="K4" s="12">
         <v>-600000</v>
       </c>
-      <c r="K4" s="12">
+      <c r="L4" s="12">
         <v>-1200000</v>
       </c>
-      <c r="L4" s="12">
+      <c r="M4" s="12">
         <v>-2400000</v>
       </c>
-      <c r="M4" s="12">
+      <c r="N4" s="12">
         <v>-4800000</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A5" s="12" t="s">
         <v>887</v>
       </c>
@@ -4606,8 +4627,11 @@
       <c r="M5" s="12">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N5" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A6" s="12" t="s">
         <v>887</v>
       </c>
@@ -4618,37 +4642,40 @@
         <v>0</v>
       </c>
       <c r="D6" s="12">
+        <v>-100</v>
+      </c>
+      <c r="E6" s="12">
         <v>-200</v>
       </c>
-      <c r="E6" s="12">
+      <c r="F6" s="12">
         <v>-1000</v>
       </c>
-      <c r="F6" s="12">
+      <c r="G6" s="12">
         <v>-2000</v>
       </c>
-      <c r="G6" s="12">
+      <c r="H6" s="12">
         <v>-20000</v>
       </c>
-      <c r="H6" s="12">
+      <c r="I6" s="12">
         <v>-100000</v>
       </c>
-      <c r="I6" s="12">
+      <c r="J6" s="12">
         <v>-200000</v>
       </c>
-      <c r="J6" s="12">
+      <c r="K6" s="12">
         <v>-600000</v>
       </c>
-      <c r="K6" s="12">
+      <c r="L6" s="12">
         <v>-1200000</v>
       </c>
-      <c r="L6" s="12">
+      <c r="M6" s="12">
         <v>-2400000</v>
       </c>
-      <c r="M6" s="12">
+      <c r="N6" s="12">
         <v>-4800000</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A7" s="12" t="s">
         <v>887</v>
       </c>
@@ -4659,37 +4686,40 @@
         <v>0</v>
       </c>
       <c r="D7" s="12">
+        <v>-100</v>
+      </c>
+      <c r="E7" s="12">
         <v>-200</v>
       </c>
-      <c r="E7" s="12">
+      <c r="F7" s="12">
         <v>-1000</v>
       </c>
-      <c r="F7" s="12">
+      <c r="G7" s="12">
         <v>-2000</v>
       </c>
-      <c r="G7" s="12">
+      <c r="H7" s="12">
         <v>-20000</v>
       </c>
-      <c r="H7" s="12">
+      <c r="I7" s="12">
         <v>-100000</v>
       </c>
-      <c r="I7" s="12">
+      <c r="J7" s="12">
         <v>-200000</v>
       </c>
-      <c r="J7" s="12">
+      <c r="K7" s="12">
         <v>-600000</v>
       </c>
-      <c r="K7" s="12">
+      <c r="L7" s="12">
         <v>-1200000</v>
       </c>
-      <c r="L7" s="12">
+      <c r="M7" s="12">
         <v>-2400000</v>
       </c>
-      <c r="M7" s="12">
+      <c r="N7" s="12">
         <v>-4800000</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A8" s="12" t="s">
         <v>888</v>
       </c>
@@ -4729,8 +4759,11 @@
       <c r="M8" s="12">
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N8" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A9" s="12" t="s">
         <v>888</v>
       </c>
@@ -4741,37 +4774,40 @@
         <v>0</v>
       </c>
       <c r="D9" s="12">
+        <v>-100</v>
+      </c>
+      <c r="E9" s="12">
         <v>-200</v>
       </c>
-      <c r="E9" s="12">
+      <c r="F9" s="12">
         <v>-1000</v>
       </c>
-      <c r="F9" s="12">
+      <c r="G9" s="12">
         <v>-2000</v>
       </c>
-      <c r="G9" s="12">
+      <c r="H9" s="12">
         <v>-20000</v>
       </c>
-      <c r="H9" s="12">
+      <c r="I9" s="12">
         <v>-100000</v>
       </c>
-      <c r="I9" s="12">
+      <c r="J9" s="12">
         <v>-200000</v>
       </c>
-      <c r="J9" s="12">
+      <c r="K9" s="12">
         <v>-600000</v>
       </c>
-      <c r="K9" s="12">
+      <c r="L9" s="12">
         <v>-1200000</v>
       </c>
-      <c r="L9" s="12">
+      <c r="M9" s="12">
         <v>-2400000</v>
       </c>
-      <c r="M9" s="12">
+      <c r="N9" s="12">
         <v>-4800000</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A10" s="12" t="s">
         <v>888</v>
       </c>
@@ -4782,37 +4818,40 @@
         <v>0</v>
       </c>
       <c r="D10" s="12">
+        <v>-100</v>
+      </c>
+      <c r="E10" s="12">
         <v>-200</v>
       </c>
-      <c r="E10" s="12">
+      <c r="F10" s="12">
         <v>-1000</v>
       </c>
-      <c r="F10" s="12">
+      <c r="G10" s="12">
         <v>-2000</v>
       </c>
-      <c r="G10" s="12">
+      <c r="H10" s="12">
         <v>-20000</v>
       </c>
-      <c r="H10" s="12">
+      <c r="I10" s="12">
         <v>-100000</v>
       </c>
-      <c r="I10" s="12">
+      <c r="J10" s="12">
         <v>-200000</v>
       </c>
-      <c r="J10" s="12">
+      <c r="K10" s="12">
         <v>-600000</v>
       </c>
-      <c r="K10" s="12">
+      <c r="L10" s="12">
         <v>-1200000</v>
       </c>
-      <c r="L10" s="12">
+      <c r="M10" s="12">
         <v>-2400000</v>
       </c>
-      <c r="M10" s="12">
+      <c r="N10" s="12">
         <v>-4800000</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A11" s="12" t="s">
         <v>889</v>
       </c>
@@ -4852,8 +4891,11 @@
       <c r="M11" s="12">
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N11" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A12" s="12" t="s">
         <v>889</v>
       </c>
@@ -4864,37 +4906,40 @@
         <v>0</v>
       </c>
       <c r="D12" s="12">
+        <v>-100</v>
+      </c>
+      <c r="E12" s="12">
         <v>-200</v>
       </c>
-      <c r="E12" s="12">
+      <c r="F12" s="12">
         <v>-1000</v>
       </c>
-      <c r="F12" s="12">
+      <c r="G12" s="12">
         <v>-2000</v>
       </c>
-      <c r="G12" s="12">
+      <c r="H12" s="12">
         <v>-20000</v>
       </c>
-      <c r="H12" s="12">
+      <c r="I12" s="12">
         <v>-100000</v>
       </c>
-      <c r="I12" s="12">
+      <c r="J12" s="12">
         <v>-200000</v>
       </c>
-      <c r="J12" s="12">
+      <c r="K12" s="12">
         <v>-600000</v>
       </c>
-      <c r="K12" s="12">
+      <c r="L12" s="12">
         <v>-1200000</v>
       </c>
-      <c r="L12" s="12">
+      <c r="M12" s="12">
         <v>-2400000</v>
       </c>
-      <c r="M12" s="12">
+      <c r="N12" s="12">
         <v>-4800000</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A13" s="12" t="s">
         <v>889</v>
       </c>
@@ -4905,37 +4950,40 @@
         <v>0</v>
       </c>
       <c r="D13" s="12">
+        <v>-100</v>
+      </c>
+      <c r="E13" s="12">
         <v>-200</v>
       </c>
-      <c r="E13" s="12">
+      <c r="F13" s="12">
         <v>-1000</v>
       </c>
-      <c r="F13" s="12">
+      <c r="G13" s="12">
         <v>-2000</v>
       </c>
-      <c r="G13" s="12">
+      <c r="H13" s="12">
         <v>-20000</v>
       </c>
-      <c r="H13" s="12">
+      <c r="I13" s="12">
         <v>-100000</v>
       </c>
-      <c r="I13" s="12">
+      <c r="J13" s="12">
         <v>-200000</v>
       </c>
-      <c r="J13" s="12">
+      <c r="K13" s="12">
         <v>-600000</v>
       </c>
-      <c r="K13" s="12">
+      <c r="L13" s="12">
         <v>-1200000</v>
       </c>
-      <c r="L13" s="12">
+      <c r="M13" s="12">
         <v>-2400000</v>
       </c>
-      <c r="M13" s="12">
+      <c r="N13" s="12">
         <v>-4800000</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A14" s="12" t="s">
         <v>890</v>
       </c>
@@ -4975,8 +5023,11 @@
       <c r="M14" s="12">
         <v>0</v>
       </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="N14" s="12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A15" s="12" t="s">
         <v>890</v>
       </c>
@@ -4987,37 +5038,40 @@
         <v>0</v>
       </c>
       <c r="D15" s="12">
+        <v>-100</v>
+      </c>
+      <c r="E15" s="12">
         <v>-200</v>
       </c>
-      <c r="E15" s="12">
+      <c r="F15" s="12">
         <v>-1000</v>
       </c>
-      <c r="F15" s="12">
+      <c r="G15" s="12">
         <v>-2000</v>
       </c>
-      <c r="G15" s="12">
+      <c r="H15" s="12">
         <v>-20000</v>
       </c>
-      <c r="H15" s="12">
+      <c r="I15" s="12">
         <v>-100000</v>
       </c>
-      <c r="I15" s="12">
+      <c r="J15" s="12">
         <v>-200000</v>
       </c>
-      <c r="J15" s="12">
+      <c r="K15" s="12">
         <v>-600000</v>
       </c>
-      <c r="K15" s="12">
+      <c r="L15" s="12">
         <v>-1200000</v>
       </c>
-      <c r="L15" s="12">
+      <c r="M15" s="12">
         <v>-2400000</v>
       </c>
-      <c r="M15" s="12">
+      <c r="N15" s="12">
         <v>-4800000</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A16" s="12" t="s">
         <v>890</v>
       </c>
@@ -5028,33 +5082,36 @@
         <v>0</v>
       </c>
       <c r="D16" s="12">
+        <v>-100</v>
+      </c>
+      <c r="E16" s="12">
         <v>-200</v>
       </c>
-      <c r="E16" s="12">
+      <c r="F16" s="12">
         <v>-1000</v>
       </c>
-      <c r="F16" s="12">
+      <c r="G16" s="12">
         <v>-2000</v>
       </c>
-      <c r="G16" s="12">
+      <c r="H16" s="12">
         <v>-20000</v>
       </c>
-      <c r="H16" s="12">
+      <c r="I16" s="12">
         <v>-100000</v>
       </c>
-      <c r="I16" s="12">
+      <c r="J16" s="12">
         <v>-200000</v>
       </c>
-      <c r="J16" s="12">
+      <c r="K16" s="12">
         <v>-600000</v>
       </c>
-      <c r="K16" s="12">
+      <c r="L16" s="12">
         <v>-1200000</v>
       </c>
-      <c r="L16" s="12">
+      <c r="M16" s="12">
         <v>-2400000</v>
       </c>
-      <c r="M16" s="12">
+      <c r="N16" s="12">
         <v>-4800000</v>
       </c>
     </row>
@@ -5290,6 +5347,7 @@
       <c r="F44" s="2"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="8" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>